<commit_message>
mejoramos la prueba en cuento a la pregunta 62
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE79A2F4-6E1A-4733-98F6-91A780C52368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3318277F-797B-48CC-8D0A-B59D2454A15B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
@@ -580,9 +580,6 @@
     <t>3205392830</t>
   </si>
   <si>
-    <t>MARÍA ISABEL QUIÑONES HERNÁNDEZ@GAILMEL.COM</t>
-  </si>
-  <si>
     <t xml:space="preserve">LUISA FERNANDA VILORIA VASQUEZ </t>
   </si>
   <si>
@@ -773,6 +770,9 @@
   </si>
   <si>
     <t>SOFIASAGA36@GMaIL.COM</t>
+  </si>
+  <si>
+    <t>MARÍA ISABEL QUIÑONES HERNÁNDEZ@gmail.COM</t>
   </si>
 </sst>
 </file>
@@ -1420,6 +1420,96 @@
       <alignment horizontal="justify" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="12" borderId="1" xfId="3" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1432,94 +1522,88 @@
     <xf numFmtId="0" fontId="19" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1549,15 +1633,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1610,81 +1685,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2193,28 +2193,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="93" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="65"/>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="95"/>
     </row>
     <row r="2" spans="1:8" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -2247,25 +2247,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C4" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D4" s="59" t="s">
+        <v>231</v>
+      </c>
+      <c r="E4" s="57" t="s">
         <v>232</v>
       </c>
-      <c r="E4" s="57" t="s">
-        <v>233</v>
-      </c>
       <c r="F4" s="59" t="s">
+        <v>228</v>
+      </c>
+      <c r="G4" s="57" t="s">
         <v>229</v>
       </c>
-      <c r="G4" s="57" t="s">
-        <v>230</v>
-      </c>
       <c r="H4" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2274,25 +2274,25 @@
         <v>2</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C5" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="59" t="s">
+        <v>226</v>
+      </c>
+      <c r="E5" s="57" t="s">
         <v>227</v>
       </c>
-      <c r="E5" s="57" t="s">
+      <c r="F5" s="59" t="s">
         <v>228</v>
       </c>
-      <c r="F5" s="59" t="s">
+      <c r="G5" s="57" t="s">
         <v>229</v>
       </c>
-      <c r="G5" s="57" t="s">
-        <v>230</v>
-      </c>
       <c r="H5" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2319,7 +2319,7 @@
         <v>62</v>
       </c>
       <c r="H6" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2346,7 +2346,7 @@
         <v>86</v>
       </c>
       <c r="H7" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2373,7 +2373,7 @@
         <v>127</v>
       </c>
       <c r="H8" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2400,7 +2400,7 @@
         <v>53</v>
       </c>
       <c r="H9" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2427,7 +2427,7 @@
         <v>149</v>
       </c>
       <c r="H10" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2454,7 +2454,7 @@
         <v>154</v>
       </c>
       <c r="H11" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2463,25 +2463,25 @@
         <v>9</v>
       </c>
       <c r="B12" s="57" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C12" s="57" t="s">
         <v>30</v>
       </c>
       <c r="D12" s="59" t="s">
+        <v>193</v>
+      </c>
+      <c r="E12" s="57" t="s">
         <v>194</v>
       </c>
-      <c r="E12" s="57" t="s">
+      <c r="F12" s="59" t="s">
         <v>195</v>
       </c>
-      <c r="F12" s="59" t="s">
+      <c r="G12" s="57" t="s">
         <v>196</v>
       </c>
-      <c r="G12" s="57" t="s">
-        <v>197</v>
-      </c>
       <c r="H12" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2490,25 +2490,25 @@
         <v>10</v>
       </c>
       <c r="B13" s="57" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C13" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D13" s="59" t="s">
+        <v>221</v>
+      </c>
+      <c r="E13" s="57" t="s">
         <v>222</v>
       </c>
-      <c r="E13" s="57" t="s">
+      <c r="F13" s="59" t="s">
         <v>223</v>
       </c>
-      <c r="F13" s="59" t="s">
+      <c r="G13" s="57" t="s">
         <v>224</v>
       </c>
-      <c r="G13" s="57" t="s">
-        <v>225</v>
-      </c>
       <c r="H13" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2517,25 +2517,25 @@
         <v>11</v>
       </c>
       <c r="B14" s="57" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C14" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="59" t="s">
+        <v>211</v>
+      </c>
+      <c r="E14" s="57" t="s">
         <v>212</v>
       </c>
-      <c r="E14" s="57" t="s">
+      <c r="F14" s="59" t="s">
         <v>213</v>
       </c>
-      <c r="F14" s="59" t="s">
+      <c r="G14" s="57" t="s">
         <v>214</v>
       </c>
-      <c r="G14" s="57" t="s">
-        <v>215</v>
-      </c>
       <c r="H14" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2562,7 +2562,7 @@
         <v>40</v>
       </c>
       <c r="H15" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2589,7 +2589,7 @@
         <v>171</v>
       </c>
       <c r="H16" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2616,7 +2616,7 @@
         <v>120</v>
       </c>
       <c r="H17" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2643,7 +2643,7 @@
         <v>124</v>
       </c>
       <c r="H18" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2670,7 +2670,7 @@
         <v>45</v>
       </c>
       <c r="H19" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2697,7 +2697,7 @@
         <v>98</v>
       </c>
       <c r="H20" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2724,7 +2724,7 @@
         <v>167</v>
       </c>
       <c r="H21" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2733,25 +2733,25 @@
         <v>19</v>
       </c>
       <c r="B22" s="57" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C22" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D22" s="59" t="s">
+        <v>206</v>
+      </c>
+      <c r="E22" s="57" t="s">
         <v>207</v>
       </c>
-      <c r="E22" s="57" t="s">
+      <c r="F22" s="59" t="s">
         <v>208</v>
       </c>
-      <c r="F22" s="59" t="s">
+      <c r="G22" s="57" t="s">
         <v>209</v>
       </c>
-      <c r="G22" s="57" t="s">
-        <v>210</v>
-      </c>
       <c r="H22" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2760,25 +2760,25 @@
         <v>20</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C23" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D23" s="59" t="s">
+        <v>216</v>
+      </c>
+      <c r="E23" s="57" t="s">
         <v>217</v>
       </c>
-      <c r="E23" s="57" t="s">
+      <c r="F23" s="59" t="s">
         <v>218</v>
       </c>
-      <c r="F23" s="59" t="s">
+      <c r="G23" s="57" t="s">
         <v>219</v>
       </c>
-      <c r="G23" s="57" t="s">
-        <v>220</v>
-      </c>
       <c r="H23" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2805,7 +2805,7 @@
         <v>81</v>
       </c>
       <c r="H24" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2832,7 +2832,7 @@
         <v>117</v>
       </c>
       <c r="H25" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2859,7 +2859,7 @@
         <v>77</v>
       </c>
       <c r="H26" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2868,25 +2868,25 @@
         <v>24</v>
       </c>
       <c r="B27" s="57" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C27" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D27" s="59" t="s">
+        <v>238</v>
+      </c>
+      <c r="E27" s="57" t="s">
         <v>239</v>
       </c>
-      <c r="E27" s="57" t="s">
+      <c r="F27" s="59" t="s">
         <v>240</v>
       </c>
-      <c r="F27" s="59" t="s">
+      <c r="G27" s="57" t="s">
         <v>241</v>
       </c>
-      <c r="G27" s="57" t="s">
+      <c r="H27" s="57" t="s">
         <v>242</v>
-      </c>
-      <c r="H27" s="57" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2913,7 +2913,7 @@
         <v>72</v>
       </c>
       <c r="H28" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2940,7 +2940,7 @@
         <v>135</v>
       </c>
       <c r="H29" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2967,7 +2967,7 @@
         <v>103</v>
       </c>
       <c r="H30" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2994,7 +2994,7 @@
         <v>144</v>
       </c>
       <c r="H31" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3003,25 +3003,25 @@
         <v>29</v>
       </c>
       <c r="B32" s="57" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C32" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D32" s="59" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E32" s="57" t="s">
         <v>70</v>
       </c>
       <c r="F32" s="59" t="s">
+        <v>203</v>
+      </c>
+      <c r="G32" s="57" t="s">
         <v>204</v>
       </c>
-      <c r="G32" s="57" t="s">
-        <v>205</v>
-      </c>
       <c r="H32" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3030,25 +3030,25 @@
         <v>30</v>
       </c>
       <c r="B33" s="57" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C33" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D33" s="59" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E33" s="57" t="s">
         <v>34</v>
       </c>
       <c r="F33" s="59" t="s">
+        <v>190</v>
+      </c>
+      <c r="G33" s="57" t="s">
         <v>191</v>
       </c>
-      <c r="G33" s="57" t="s">
-        <v>192</v>
-      </c>
       <c r="H33" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3075,7 +3075,7 @@
         <v>175</v>
       </c>
       <c r="H34" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3102,7 +3102,7 @@
         <v>131</v>
       </c>
       <c r="H35" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3111,25 +3111,25 @@
         <v>33</v>
       </c>
       <c r="B36" s="57" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C36" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D36" s="59" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E36" s="57" t="s">
         <v>178</v>
       </c>
       <c r="F36" s="59" t="s">
+        <v>182</v>
+      </c>
+      <c r="G36" s="57" t="s">
         <v>183</v>
       </c>
-      <c r="G36" s="57" t="s">
-        <v>184</v>
-      </c>
       <c r="H36" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3153,10 +3153,10 @@
         <v>179</v>
       </c>
       <c r="G37" s="57" t="s">
-        <v>180</v>
+        <v>244</v>
       </c>
       <c r="H37" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3183,7 +3183,7 @@
         <v>108</v>
       </c>
       <c r="H38" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3192,25 +3192,25 @@
         <v>36</v>
       </c>
       <c r="B39" s="57" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C39" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D39" s="59" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E39" s="57" t="s">
         <v>101</v>
       </c>
       <c r="F39" s="59" t="s">
+        <v>235</v>
+      </c>
+      <c r="G39" s="57" t="s">
         <v>236</v>
       </c>
-      <c r="G39" s="57" t="s">
-        <v>237</v>
-      </c>
       <c r="H39" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3219,25 +3219,25 @@
         <v>37</v>
       </c>
       <c r="B40" s="57" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C40" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D40" s="59" t="s">
+        <v>198</v>
+      </c>
+      <c r="E40" s="57" t="s">
+        <v>194</v>
+      </c>
+      <c r="F40" s="59" t="s">
         <v>199</v>
       </c>
-      <c r="E40" s="57" t="s">
-        <v>195</v>
-      </c>
-      <c r="F40" s="59" t="s">
+      <c r="G40" s="57" t="s">
         <v>200</v>
       </c>
-      <c r="G40" s="57" t="s">
-        <v>201</v>
-      </c>
       <c r="H40" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3264,7 +3264,7 @@
         <v>112</v>
       </c>
       <c r="H41" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3291,7 +3291,7 @@
         <v>163</v>
       </c>
       <c r="H42" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3318,7 +3318,7 @@
         <v>89</v>
       </c>
       <c r="H43" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3327,25 +3327,25 @@
         <v>41</v>
       </c>
       <c r="B44" s="57" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C44" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D44" s="59" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E44" s="57" t="s">
         <v>178</v>
       </c>
       <c r="F44" s="59" t="s">
+        <v>186</v>
+      </c>
+      <c r="G44" s="57" t="s">
         <v>187</v>
       </c>
-      <c r="G44" s="57" t="s">
-        <v>188</v>
-      </c>
       <c r="H44" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3372,7 +3372,7 @@
         <v>159</v>
       </c>
       <c r="H45" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3396,10 +3396,10 @@
         <v>57</v>
       </c>
       <c r="G46" s="61" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H46" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3426,7 +3426,7 @@
         <v>94</v>
       </c>
       <c r="H47" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3453,7 +3453,7 @@
         <v>49</v>
       </c>
       <c r="H48" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3480,7 +3480,7 @@
         <v>36</v>
       </c>
       <c r="H49" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3507,7 +3507,7 @@
         <v>139</v>
       </c>
       <c r="H50" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3534,7 +3534,7 @@
         <v>67</v>
       </c>
       <c r="H51" s="57" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3723,37 +3723,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="73" t="s">
+      <c r="B1" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="73"/>
-      <c r="R1" s="73"/>
-      <c r="S1" s="73"/>
-      <c r="T1" s="73"/>
-      <c r="U1" s="73"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="73"/>
-      <c r="X1" s="73"/>
-      <c r="Y1" s="73"/>
-      <c r="Z1" s="73"/>
-      <c r="AA1" s="73"/>
-      <c r="AB1" s="73"/>
-      <c r="AC1" s="73"/>
-      <c r="AD1" s="73"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
     </row>
     <row r="2" spans="1:30" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="55" t="s">
@@ -3765,120 +3765,120 @@
       <c r="C2" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="89" t="s">
+      <c r="D2" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="91"/>
-      <c r="H2" s="74" t="s">
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="75"/>
-      <c r="J2" s="75"/>
-      <c r="K2" s="75"/>
-      <c r="L2" s="75"/>
-      <c r="M2" s="75"/>
-      <c r="N2" s="75"/>
-      <c r="O2" s="75"/>
-      <c r="P2" s="76"/>
-      <c r="Q2" s="83" t="s">
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+      <c r="P2" s="72"/>
+      <c r="Q2" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="84"/>
-      <c r="S2" s="84"/>
-      <c r="T2" s="84"/>
-      <c r="U2" s="84"/>
-      <c r="V2" s="84"/>
-      <c r="W2" s="84"/>
-      <c r="X2" s="84"/>
-      <c r="Y2" s="85"/>
-      <c r="Z2" s="66" t="s">
+      <c r="R2" s="80"/>
+      <c r="S2" s="80"/>
+      <c r="T2" s="80"/>
+      <c r="U2" s="80"/>
+      <c r="V2" s="80"/>
+      <c r="W2" s="80"/>
+      <c r="X2" s="80"/>
+      <c r="Y2" s="81"/>
+      <c r="Z2" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="AA2" s="67"/>
-      <c r="AB2" s="67"/>
-      <c r="AC2" s="67"/>
-      <c r="AD2" s="68"/>
+      <c r="AA2" s="63"/>
+      <c r="AB2" s="63"/>
+      <c r="AC2" s="63"/>
+      <c r="AD2" s="64"/>
     </row>
     <row r="3" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="56"/>
       <c r="B3" s="54"/>
       <c r="C3" s="56"/>
-      <c r="D3" s="92" t="s">
+      <c r="D3" s="88" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="77" t="s">
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="78"/>
-      <c r="J3" s="78"/>
-      <c r="K3" s="78"/>
-      <c r="L3" s="78"/>
-      <c r="M3" s="78"/>
-      <c r="N3" s="78"/>
-      <c r="O3" s="78"/>
-      <c r="P3" s="79"/>
-      <c r="Q3" s="86" t="s">
+      <c r="I3" s="74"/>
+      <c r="J3" s="74"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="74"/>
+      <c r="M3" s="74"/>
+      <c r="N3" s="74"/>
+      <c r="O3" s="74"/>
+      <c r="P3" s="75"/>
+      <c r="Q3" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="R3" s="87"/>
-      <c r="S3" s="87"/>
-      <c r="T3" s="87"/>
-      <c r="U3" s="87"/>
-      <c r="V3" s="87"/>
-      <c r="W3" s="87"/>
-      <c r="X3" s="87"/>
-      <c r="Y3" s="88"/>
-      <c r="Z3" s="69" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="70"/>
-      <c r="AB3" s="70"/>
-      <c r="AC3" s="70"/>
-      <c r="AD3" s="71"/>
+      <c r="R3" s="83"/>
+      <c r="S3" s="83"/>
+      <c r="T3" s="83"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="83"/>
+      <c r="W3" s="83"/>
+      <c r="X3" s="83"/>
+      <c r="Y3" s="84"/>
+      <c r="Z3" s="65" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="66"/>
+      <c r="AB3" s="66"/>
+      <c r="AC3" s="66"/>
+      <c r="AD3" s="67"/>
     </row>
     <row r="4" spans="1:30" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="56"/>
       <c r="B4" s="54"/>
       <c r="C4" s="56"/>
-      <c r="D4" s="95" t="s">
+      <c r="D4" s="91" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="81"/>
-      <c r="F4" s="81"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="80" t="s">
+      <c r="H4" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="81"/>
-      <c r="J4" s="81"/>
-      <c r="K4" s="81"/>
-      <c r="L4" s="81"/>
-      <c r="M4" s="81"/>
-      <c r="N4" s="81"/>
-      <c r="O4" s="82"/>
+      <c r="I4" s="77"/>
+      <c r="J4" s="77"/>
+      <c r="K4" s="77"/>
+      <c r="L4" s="77"/>
+      <c r="M4" s="77"/>
+      <c r="N4" s="77"/>
+      <c r="O4" s="78"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="80" t="s">
+      <c r="Q4" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="R4" s="81"/>
-      <c r="S4" s="81"/>
-      <c r="T4" s="81"/>
-      <c r="U4" s="81"/>
-      <c r="V4" s="81"/>
-      <c r="W4" s="81"/>
-      <c r="X4" s="82"/>
+      <c r="R4" s="77"/>
+      <c r="S4" s="77"/>
+      <c r="T4" s="77"/>
+      <c r="U4" s="77"/>
+      <c r="V4" s="77"/>
+      <c r="W4" s="77"/>
+      <c r="X4" s="78"/>
       <c r="Y4" s="13"/>
-      <c r="Z4" s="72" t="s">
+      <c r="Z4" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="AA4" s="72"/>
-      <c r="AB4" s="72"/>
-      <c r="AC4" s="72"/>
+      <c r="AA4" s="68"/>
+      <c r="AB4" s="68"/>
+      <c r="AC4" s="68"/>
       <c r="AD4" s="3"/>
     </row>
     <row r="5" spans="1:30" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -3954,7 +3954,7 @@
       <c r="N6" s="39"/>
       <c r="O6" s="40"/>
       <c r="P6" s="38">
-        <f>+SUM(H6:O6)/8</f>
+        <f t="shared" ref="P6:P53" si="0">+SUM(H6:O6)/8</f>
         <v>0</v>
       </c>
       <c r="Q6" s="39"/>
@@ -3966,7 +3966,7 @@
       <c r="W6" s="40"/>
       <c r="X6" s="39"/>
       <c r="Y6" s="38">
-        <f t="shared" ref="Y6:Y54" si="0">+SUM(Q6:X6)/8</f>
+        <f t="shared" ref="Y6:Y54" si="1">+SUM(Q6:X6)/8</f>
         <v>0</v>
       </c>
       <c r="Z6" s="41"/>
@@ -3974,7 +3974,7 @@
       <c r="AB6" s="40"/>
       <c r="AC6" s="40"/>
       <c r="AD6" s="38">
-        <f t="shared" ref="AD6:AD54" si="1">+SUM(Z6:AC6)/4</f>
+        <f t="shared" ref="AD6:AD54" si="2">+SUM(Z6:AC6)/4</f>
         <v>0</v>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
       <c r="G7" s="38">
-        <f t="shared" ref="G7:G63" si="2">+SUM(D7:F7)/3</f>
+        <f t="shared" ref="G7:G63" si="3">+SUM(D7:F7)/3</f>
         <v>0</v>
       </c>
       <c r="H7" s="14">
@@ -4007,7 +4007,7 @@
       <c r="N7" s="39"/>
       <c r="O7" s="40"/>
       <c r="P7" s="38">
-        <f>+SUM(H7:O7)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q7" s="39"/>
@@ -4019,7 +4019,7 @@
       <c r="W7" s="40"/>
       <c r="X7" s="39"/>
       <c r="Y7" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z7" s="41"/>
@@ -4027,7 +4027,7 @@
       <c r="AB7" s="40"/>
       <c r="AC7" s="40"/>
       <c r="AD7" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4046,7 +4046,7 @@
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H8" s="14">
@@ -4060,7 +4060,7 @@
       <c r="N8" s="39"/>
       <c r="O8" s="40"/>
       <c r="P8" s="38">
-        <f>+SUM(H8:O8)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q8" s="39"/>
@@ -4072,7 +4072,7 @@
       <c r="W8" s="40"/>
       <c r="X8" s="39"/>
       <c r="Y8" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z8" s="41"/>
@@ -4080,7 +4080,7 @@
       <c r="AB8" s="40"/>
       <c r="AC8" s="40"/>
       <c r="AD8" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4099,7 +4099,7 @@
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
       <c r="G9" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H9" s="14">
@@ -4113,7 +4113,7 @@
       <c r="N9" s="39"/>
       <c r="O9" s="39"/>
       <c r="P9" s="38">
-        <f>+SUM(H9:O9)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q9" s="39"/>
@@ -4125,7 +4125,7 @@
       <c r="W9" s="40"/>
       <c r="X9" s="39"/>
       <c r="Y9" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z9" s="41"/>
@@ -4133,7 +4133,7 @@
       <c r="AB9" s="40"/>
       <c r="AC9" s="40"/>
       <c r="AD9" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4152,7 +4152,7 @@
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
       <c r="G10" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H10" s="14">
@@ -4166,7 +4166,7 @@
       <c r="N10" s="39"/>
       <c r="O10" s="39"/>
       <c r="P10" s="38">
-        <f>+SUM(H10:O10)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q10" s="39"/>
@@ -4178,7 +4178,7 @@
       <c r="W10" s="40"/>
       <c r="X10" s="39"/>
       <c r="Y10" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z10" s="41"/>
@@ -4186,7 +4186,7 @@
       <c r="AB10" s="40"/>
       <c r="AC10" s="40"/>
       <c r="AD10" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
       <c r="G11" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H11" s="14">
@@ -4219,7 +4219,7 @@
       <c r="N11" s="39"/>
       <c r="O11" s="40"/>
       <c r="P11" s="38">
-        <f>+SUM(H11:O11)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q11" s="39"/>
@@ -4231,7 +4231,7 @@
       <c r="W11" s="40"/>
       <c r="X11" s="39"/>
       <c r="Y11" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z11" s="41"/>
@@ -4239,7 +4239,7 @@
       <c r="AB11" s="40"/>
       <c r="AC11" s="40"/>
       <c r="AD11" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4258,7 +4258,7 @@
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
       <c r="G12" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H12" s="14">
@@ -4272,7 +4272,7 @@
       <c r="N12" s="39"/>
       <c r="O12" s="40"/>
       <c r="P12" s="38">
-        <f>+SUM(H12:O12)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q12" s="39"/>
@@ -4284,7 +4284,7 @@
       <c r="W12" s="40"/>
       <c r="X12" s="39"/>
       <c r="Y12" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z12" s="41"/>
@@ -4292,7 +4292,7 @@
       <c r="AB12" s="40"/>
       <c r="AC12" s="40"/>
       <c r="AD12" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4311,7 +4311,7 @@
       <c r="E13" s="14"/>
       <c r="F13" s="14"/>
       <c r="G13" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H13" s="14">
@@ -4325,7 +4325,7 @@
       <c r="N13" s="39"/>
       <c r="O13" s="39"/>
       <c r="P13" s="38">
-        <f>+SUM(H13:O13)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q13" s="39"/>
@@ -4337,7 +4337,7 @@
       <c r="W13" s="40"/>
       <c r="X13" s="39"/>
       <c r="Y13" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z13" s="41"/>
@@ -4345,7 +4345,7 @@
       <c r="AB13" s="40"/>
       <c r="AC13" s="40"/>
       <c r="AD13" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4364,7 +4364,7 @@
       <c r="E14" s="14"/>
       <c r="F14" s="14"/>
       <c r="G14" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H14" s="14">
@@ -4378,7 +4378,7 @@
       <c r="N14" s="39"/>
       <c r="O14" s="40"/>
       <c r="P14" s="38">
-        <f>+SUM(H14:O14)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q14" s="39"/>
@@ -4390,7 +4390,7 @@
       <c r="W14" s="40"/>
       <c r="X14" s="39"/>
       <c r="Y14" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z14" s="41"/>
@@ -4398,7 +4398,7 @@
       <c r="AB14" s="40"/>
       <c r="AC14" s="40"/>
       <c r="AD14" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4417,7 +4417,7 @@
       <c r="E15" s="14"/>
       <c r="F15" s="14"/>
       <c r="G15" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H15" s="14">
@@ -4431,7 +4431,7 @@
       <c r="N15" s="39"/>
       <c r="O15" s="40"/>
       <c r="P15" s="38">
-        <f>+SUM(H15:O15)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q15" s="39"/>
@@ -4443,7 +4443,7 @@
       <c r="W15" s="40"/>
       <c r="X15" s="39"/>
       <c r="Y15" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z15" s="41"/>
@@ -4451,7 +4451,7 @@
       <c r="AB15" s="40"/>
       <c r="AC15" s="40"/>
       <c r="AD15" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4470,7 +4470,7 @@
       <c r="E16" s="14"/>
       <c r="F16" s="14"/>
       <c r="G16" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H16" s="14">
@@ -4484,7 +4484,7 @@
       <c r="N16" s="39"/>
       <c r="O16" s="40"/>
       <c r="P16" s="38">
-        <f>+SUM(H16:O16)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q16" s="39"/>
@@ -4496,7 +4496,7 @@
       <c r="W16" s="40"/>
       <c r="X16" s="39"/>
       <c r="Y16" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z16" s="41"/>
@@ -4504,7 +4504,7 @@
       <c r="AB16" s="40"/>
       <c r="AC16" s="40"/>
       <c r="AD16" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4523,7 +4523,7 @@
       <c r="E17" s="14"/>
       <c r="F17" s="14"/>
       <c r="G17" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H17" s="14">
@@ -4537,7 +4537,7 @@
       <c r="N17" s="39"/>
       <c r="O17" s="40"/>
       <c r="P17" s="38">
-        <f>+SUM(H17:O17)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q17" s="39"/>
@@ -4549,7 +4549,7 @@
       <c r="W17" s="40"/>
       <c r="X17" s="39"/>
       <c r="Y17" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z17" s="41"/>
@@ -4557,7 +4557,7 @@
       <c r="AB17" s="40"/>
       <c r="AC17" s="40"/>
       <c r="AD17" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       <c r="E18" s="14"/>
       <c r="F18" s="14"/>
       <c r="G18" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H18" s="14">
@@ -4590,7 +4590,7 @@
       <c r="N18" s="39"/>
       <c r="O18" s="40"/>
       <c r="P18" s="38">
-        <f>+SUM(H18:O18)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q18" s="39"/>
@@ -4602,7 +4602,7 @@
       <c r="W18" s="40"/>
       <c r="X18" s="39"/>
       <c r="Y18" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z18" s="41"/>
@@ -4610,7 +4610,7 @@
       <c r="AB18" s="40"/>
       <c r="AC18" s="40"/>
       <c r="AD18" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
       <c r="G19" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H19" s="14">
@@ -4643,7 +4643,7 @@
       <c r="N19" s="39"/>
       <c r="O19" s="40"/>
       <c r="P19" s="38">
-        <f>+SUM(H19:O19)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q19" s="39"/>
@@ -4655,7 +4655,7 @@
       <c r="W19" s="40"/>
       <c r="X19" s="39"/>
       <c r="Y19" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z19" s="41"/>
@@ -4663,7 +4663,7 @@
       <c r="AB19" s="40"/>
       <c r="AC19" s="40"/>
       <c r="AD19" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       <c r="E20" s="14"/>
       <c r="F20" s="14"/>
       <c r="G20" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H20" s="14">
@@ -4696,7 +4696,7 @@
       <c r="N20" s="39"/>
       <c r="O20" s="40"/>
       <c r="P20" s="38">
-        <f>+SUM(H20:O20)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q20" s="39"/>
@@ -4708,7 +4708,7 @@
       <c r="W20" s="40"/>
       <c r="X20" s="39"/>
       <c r="Y20" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z20" s="41"/>
@@ -4716,7 +4716,7 @@
       <c r="AB20" s="40"/>
       <c r="AC20" s="40"/>
       <c r="AD20" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4735,7 +4735,7 @@
       <c r="E21" s="14"/>
       <c r="F21" s="14"/>
       <c r="G21" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H21" s="14">
@@ -4749,7 +4749,7 @@
       <c r="N21" s="39"/>
       <c r="O21" s="39"/>
       <c r="P21" s="38">
-        <f>+SUM(H21:O21)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q21" s="39"/>
@@ -4761,7 +4761,7 @@
       <c r="W21" s="40"/>
       <c r="X21" s="39"/>
       <c r="Y21" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z21" s="41"/>
@@ -4769,7 +4769,7 @@
       <c r="AB21" s="40"/>
       <c r="AC21" s="40"/>
       <c r="AD21" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4788,7 +4788,7 @@
       <c r="E22" s="14"/>
       <c r="F22" s="14"/>
       <c r="G22" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H22" s="14">
@@ -4802,7 +4802,7 @@
       <c r="N22" s="39"/>
       <c r="O22" s="40"/>
       <c r="P22" s="38">
-        <f>+SUM(H22:O22)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q22" s="39"/>
@@ -4814,7 +4814,7 @@
       <c r="W22" s="40"/>
       <c r="X22" s="39"/>
       <c r="Y22" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z22" s="41"/>
@@ -4822,7 +4822,7 @@
       <c r="AB22" s="40"/>
       <c r="AC22" s="40"/>
       <c r="AD22" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4841,7 +4841,7 @@
       <c r="E23" s="14"/>
       <c r="F23" s="14"/>
       <c r="G23" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H23" s="14">
@@ -4855,7 +4855,7 @@
       <c r="N23" s="39"/>
       <c r="O23" s="40"/>
       <c r="P23" s="38">
-        <f>+SUM(H23:O23)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q23" s="39"/>
@@ -4867,7 +4867,7 @@
       <c r="W23" s="40"/>
       <c r="X23" s="39"/>
       <c r="Y23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z23" s="41"/>
@@ -4875,7 +4875,7 @@
       <c r="AB23" s="40"/>
       <c r="AC23" s="40"/>
       <c r="AD23" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
       <c r="E24" s="14"/>
       <c r="F24" s="14"/>
       <c r="G24" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H24" s="14">
@@ -4908,7 +4908,7 @@
       <c r="N24" s="39"/>
       <c r="O24" s="40"/>
       <c r="P24" s="38">
-        <f>+SUM(H24:O24)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q24" s="39"/>
@@ -4920,7 +4920,7 @@
       <c r="W24" s="40"/>
       <c r="X24" s="39"/>
       <c r="Y24" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z24" s="41"/>
@@ -4928,7 +4928,7 @@
       <c r="AB24" s="40"/>
       <c r="AC24" s="40"/>
       <c r="AD24" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       <c r="E25" s="14"/>
       <c r="F25" s="14"/>
       <c r="G25" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H25" s="14">
@@ -4961,7 +4961,7 @@
       <c r="N25" s="39"/>
       <c r="O25" s="39"/>
       <c r="P25" s="38">
-        <f>+SUM(H25:O25)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q25" s="39"/>
@@ -4973,7 +4973,7 @@
       <c r="W25" s="40"/>
       <c r="X25" s="39"/>
       <c r="Y25" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z25" s="41"/>
@@ -4981,7 +4981,7 @@
       <c r="AB25" s="40"/>
       <c r="AC25" s="40"/>
       <c r="AD25" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5000,7 +5000,7 @@
       <c r="E26" s="14"/>
       <c r="F26" s="14"/>
       <c r="G26" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H26" s="14">
@@ -5014,7 +5014,7 @@
       <c r="N26" s="39"/>
       <c r="O26" s="40"/>
       <c r="P26" s="38">
-        <f>+SUM(H26:O26)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q26" s="39"/>
@@ -5026,7 +5026,7 @@
       <c r="W26" s="40"/>
       <c r="X26" s="39"/>
       <c r="Y26" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z26" s="42"/>
@@ -5034,7 +5034,7 @@
       <c r="AB26" s="43"/>
       <c r="AC26" s="43"/>
       <c r="AD26" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5053,7 +5053,7 @@
       <c r="E27" s="14"/>
       <c r="F27" s="14"/>
       <c r="G27" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H27" s="14">
@@ -5067,7 +5067,7 @@
       <c r="N27" s="39"/>
       <c r="O27" s="40"/>
       <c r="P27" s="38">
-        <f>+SUM(H27:O27)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q27" s="39"/>
@@ -5079,7 +5079,7 @@
       <c r="W27" s="40"/>
       <c r="X27" s="39"/>
       <c r="Y27" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z27" s="41"/>
@@ -5087,7 +5087,7 @@
       <c r="AB27" s="40"/>
       <c r="AC27" s="40"/>
       <c r="AD27" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       <c r="E28" s="14"/>
       <c r="F28" s="14"/>
       <c r="G28" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H28" s="14">
@@ -5120,7 +5120,7 @@
       <c r="N28" s="39"/>
       <c r="O28" s="40"/>
       <c r="P28" s="38">
-        <f>+SUM(H28:O28)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q28" s="39"/>
@@ -5132,7 +5132,7 @@
       <c r="W28" s="40"/>
       <c r="X28" s="39"/>
       <c r="Y28" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z28" s="41"/>
@@ -5140,7 +5140,7 @@
       <c r="AB28" s="40"/>
       <c r="AC28" s="40"/>
       <c r="AD28" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       <c r="E29" s="14"/>
       <c r="F29" s="14"/>
       <c r="G29" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H29" s="14">
@@ -5173,7 +5173,7 @@
       <c r="N29" s="39"/>
       <c r="O29" s="40"/>
       <c r="P29" s="38">
-        <f>+SUM(H29:O29)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q29" s="39"/>
@@ -5185,7 +5185,7 @@
       <c r="W29" s="40"/>
       <c r="X29" s="39"/>
       <c r="Y29" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z29" s="41"/>
@@ -5193,7 +5193,7 @@
       <c r="AB29" s="40"/>
       <c r="AC29" s="40"/>
       <c r="AD29" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5212,7 +5212,7 @@
       <c r="E30" s="14"/>
       <c r="F30" s="14"/>
       <c r="G30" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H30" s="14">
@@ -5226,7 +5226,7 @@
       <c r="N30" s="39"/>
       <c r="O30" s="39"/>
       <c r="P30" s="38">
-        <f>+SUM(H30:O30)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q30" s="39"/>
@@ -5238,7 +5238,7 @@
       <c r="W30" s="40"/>
       <c r="X30" s="39"/>
       <c r="Y30" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z30" s="41"/>
@@ -5246,7 +5246,7 @@
       <c r="AB30" s="40"/>
       <c r="AC30" s="40"/>
       <c r="AD30" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5265,7 +5265,7 @@
       <c r="E31" s="14"/>
       <c r="F31" s="14"/>
       <c r="G31" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H31" s="14">
@@ -5279,7 +5279,7 @@
       <c r="N31" s="39"/>
       <c r="O31" s="40"/>
       <c r="P31" s="38">
-        <f>+SUM(H31:O31)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q31" s="39"/>
@@ -5291,7 +5291,7 @@
       <c r="W31" s="40"/>
       <c r="X31" s="39"/>
       <c r="Y31" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z31" s="41"/>
@@ -5299,7 +5299,7 @@
       <c r="AB31" s="40"/>
       <c r="AC31" s="40"/>
       <c r="AD31" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5318,7 +5318,7 @@
       <c r="E32" s="14"/>
       <c r="F32" s="14"/>
       <c r="G32" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H32" s="14">
@@ -5332,7 +5332,7 @@
       <c r="N32" s="39"/>
       <c r="O32" s="40"/>
       <c r="P32" s="38">
-        <f>+SUM(H32:O32)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q32" s="39"/>
@@ -5344,7 +5344,7 @@
       <c r="W32" s="40"/>
       <c r="X32" s="39"/>
       <c r="Y32" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z32" s="41"/>
@@ -5352,7 +5352,7 @@
       <c r="AB32" s="40"/>
       <c r="AC32" s="40"/>
       <c r="AD32" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5371,7 +5371,7 @@
       <c r="E33" s="14"/>
       <c r="F33" s="14"/>
       <c r="G33" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H33" s="14">
@@ -5385,7 +5385,7 @@
       <c r="N33" s="39"/>
       <c r="O33" s="40"/>
       <c r="P33" s="38">
-        <f>+SUM(H33:O33)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q33" s="39"/>
@@ -5397,7 +5397,7 @@
       <c r="W33" s="40"/>
       <c r="X33" s="39"/>
       <c r="Y33" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z33" s="41"/>
@@ -5405,7 +5405,7 @@
       <c r="AB33" s="40"/>
       <c r="AC33" s="40"/>
       <c r="AD33" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5424,7 +5424,7 @@
       <c r="E34" s="14"/>
       <c r="F34" s="14"/>
       <c r="G34" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H34" s="14">
@@ -5438,7 +5438,7 @@
       <c r="N34" s="39"/>
       <c r="O34" s="40"/>
       <c r="P34" s="38">
-        <f>+SUM(H34:O34)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q34" s="39"/>
@@ -5450,7 +5450,7 @@
       <c r="W34" s="40"/>
       <c r="X34" s="39"/>
       <c r="Y34" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z34" s="41"/>
@@ -5458,7 +5458,7 @@
       <c r="AB34" s="40"/>
       <c r="AC34" s="40"/>
       <c r="AD34" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5477,7 +5477,7 @@
       <c r="E35" s="14"/>
       <c r="F35" s="14"/>
       <c r="G35" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H35" s="14">
@@ -5491,7 +5491,7 @@
       <c r="N35" s="39"/>
       <c r="O35" s="40"/>
       <c r="P35" s="38">
-        <f>+SUM(H35:O35)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q35" s="39"/>
@@ -5503,7 +5503,7 @@
       <c r="W35" s="40"/>
       <c r="X35" s="39"/>
       <c r="Y35" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z35" s="41"/>
@@ -5511,7 +5511,7 @@
       <c r="AB35" s="40"/>
       <c r="AC35" s="40"/>
       <c r="AD35" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5530,7 +5530,7 @@
       <c r="E36" s="14"/>
       <c r="F36" s="14"/>
       <c r="G36" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H36" s="14">
@@ -5544,7 +5544,7 @@
       <c r="N36" s="39"/>
       <c r="O36" s="39"/>
       <c r="P36" s="38">
-        <f>+SUM(H36:O36)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q36" s="39"/>
@@ -5556,7 +5556,7 @@
       <c r="W36" s="40"/>
       <c r="X36" s="39"/>
       <c r="Y36" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z36" s="42"/>
@@ -5564,7 +5564,7 @@
       <c r="AB36" s="43"/>
       <c r="AC36" s="43"/>
       <c r="AD36" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5583,7 +5583,7 @@
       <c r="E37" s="14"/>
       <c r="F37" s="14"/>
       <c r="G37" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H37" s="14">
@@ -5597,7 +5597,7 @@
       <c r="N37" s="39"/>
       <c r="O37" s="40"/>
       <c r="P37" s="38">
-        <f>+SUM(H37:O37)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q37" s="39"/>
@@ -5609,7 +5609,7 @@
       <c r="W37" s="40"/>
       <c r="X37" s="39"/>
       <c r="Y37" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z37" s="41"/>
@@ -5617,7 +5617,7 @@
       <c r="AB37" s="40"/>
       <c r="AC37" s="40"/>
       <c r="AD37" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5636,7 +5636,7 @@
       <c r="E38" s="14"/>
       <c r="F38" s="14"/>
       <c r="G38" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H38" s="14">
@@ -5650,7 +5650,7 @@
       <c r="N38" s="39"/>
       <c r="O38" s="40"/>
       <c r="P38" s="38">
-        <f>+SUM(H38:O38)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q38" s="39"/>
@@ -5662,7 +5662,7 @@
       <c r="W38" s="40"/>
       <c r="X38" s="39"/>
       <c r="Y38" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z38" s="41"/>
@@ -5670,7 +5670,7 @@
       <c r="AB38" s="40"/>
       <c r="AC38" s="40"/>
       <c r="AD38" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5689,7 +5689,7 @@
       <c r="E39" s="14"/>
       <c r="F39" s="14"/>
       <c r="G39" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H39" s="14">
@@ -5703,7 +5703,7 @@
       <c r="N39" s="39"/>
       <c r="O39" s="40"/>
       <c r="P39" s="38">
-        <f>+SUM(H39:O39)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q39" s="39"/>
@@ -5715,7 +5715,7 @@
       <c r="W39" s="40"/>
       <c r="X39" s="39"/>
       <c r="Y39" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z39" s="41"/>
@@ -5723,7 +5723,7 @@
       <c r="AB39" s="40"/>
       <c r="AC39" s="40"/>
       <c r="AD39" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5742,7 +5742,7 @@
       <c r="E40" s="14"/>
       <c r="F40" s="14"/>
       <c r="G40" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H40" s="14">
@@ -5756,7 +5756,7 @@
       <c r="N40" s="39"/>
       <c r="O40" s="39"/>
       <c r="P40" s="38">
-        <f>+SUM(H40:O40)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q40" s="39"/>
@@ -5768,7 +5768,7 @@
       <c r="W40" s="40"/>
       <c r="X40" s="39"/>
       <c r="Y40" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z40" s="41"/>
@@ -5776,7 +5776,7 @@
       <c r="AB40" s="40"/>
       <c r="AC40" s="40"/>
       <c r="AD40" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5795,7 +5795,7 @@
       <c r="E41" s="14"/>
       <c r="F41" s="14"/>
       <c r="G41" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H41" s="14">
@@ -5809,7 +5809,7 @@
       <c r="N41" s="39"/>
       <c r="O41" s="39"/>
       <c r="P41" s="38">
-        <f>+SUM(H41:O41)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q41" s="39"/>
@@ -5821,7 +5821,7 @@
       <c r="W41" s="40"/>
       <c r="X41" s="40"/>
       <c r="Y41" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z41" s="41"/>
@@ -5829,7 +5829,7 @@
       <c r="AB41" s="40"/>
       <c r="AC41" s="40"/>
       <c r="AD41" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5848,7 +5848,7 @@
       <c r="E42" s="14"/>
       <c r="F42" s="14"/>
       <c r="G42" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H42" s="14">
@@ -5862,7 +5862,7 @@
       <c r="N42" s="39"/>
       <c r="O42" s="40"/>
       <c r="P42" s="38">
-        <f>+SUM(H42:O42)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q42" s="39"/>
@@ -5874,7 +5874,7 @@
       <c r="W42" s="40"/>
       <c r="X42" s="40"/>
       <c r="Y42" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z42" s="42"/>
@@ -5882,7 +5882,7 @@
       <c r="AB42" s="43"/>
       <c r="AC42" s="43"/>
       <c r="AD42" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5901,7 +5901,7 @@
       <c r="E43" s="14"/>
       <c r="F43" s="14"/>
       <c r="G43" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H43" s="14">
@@ -5915,7 +5915,7 @@
       <c r="N43" s="39"/>
       <c r="O43" s="40"/>
       <c r="P43" s="38">
-        <f>+SUM(H43:O43)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q43" s="39"/>
@@ -5927,7 +5927,7 @@
       <c r="W43" s="39"/>
       <c r="X43" s="39"/>
       <c r="Y43" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z43" s="41"/>
@@ -5935,7 +5935,7 @@
       <c r="AB43" s="40"/>
       <c r="AC43" s="40"/>
       <c r="AD43" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
       <c r="E44" s="14"/>
       <c r="F44" s="14"/>
       <c r="G44" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H44" s="14">
@@ -5968,7 +5968,7 @@
       <c r="N44" s="39"/>
       <c r="O44" s="40"/>
       <c r="P44" s="38">
-        <f>+SUM(H44:O44)/8</f>
+        <f t="shared" si="0"/>
         <v>0.125</v>
       </c>
       <c r="Q44" s="39"/>
@@ -5980,7 +5980,7 @@
       <c r="W44" s="39"/>
       <c r="X44" s="39"/>
       <c r="Y44" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z44" s="41"/>
@@ -5988,7 +5988,7 @@
       <c r="AB44" s="40"/>
       <c r="AC44" s="40"/>
       <c r="AD44" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6007,7 +6007,7 @@
       <c r="E45" s="14"/>
       <c r="F45" s="14"/>
       <c r="G45" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H45" s="14">
@@ -6021,7 +6021,7 @@
       <c r="N45" s="39"/>
       <c r="O45" s="40"/>
       <c r="P45" s="38">
-        <f>+SUM(H45:O45)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q45" s="39"/>
@@ -6033,7 +6033,7 @@
       <c r="W45" s="39"/>
       <c r="X45" s="39"/>
       <c r="Y45" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z45" s="41"/>
@@ -6041,7 +6041,7 @@
       <c r="AB45" s="40"/>
       <c r="AC45" s="40"/>
       <c r="AD45" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6060,7 +6060,7 @@
       <c r="E46" s="14"/>
       <c r="F46" s="14"/>
       <c r="G46" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H46" s="14">
@@ -6074,7 +6074,7 @@
       <c r="N46" s="39"/>
       <c r="O46" s="39"/>
       <c r="P46" s="38">
-        <f>+SUM(H46:O46)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q46" s="39"/>
@@ -6086,7 +6086,7 @@
       <c r="W46" s="39"/>
       <c r="X46" s="39"/>
       <c r="Y46" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z46" s="41"/>
@@ -6094,7 +6094,7 @@
       <c r="AB46" s="40"/>
       <c r="AC46" s="40"/>
       <c r="AD46" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6113,7 +6113,7 @@
       <c r="E47" s="14"/>
       <c r="F47" s="14"/>
       <c r="G47" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H47" s="14">
@@ -6127,7 +6127,7 @@
       <c r="N47" s="39"/>
       <c r="O47" s="40"/>
       <c r="P47" s="38">
-        <f>+SUM(H47:O47)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q47" s="39"/>
@@ -6139,7 +6139,7 @@
       <c r="W47" s="39"/>
       <c r="X47" s="39"/>
       <c r="Y47" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z47" s="41"/>
@@ -6147,7 +6147,7 @@
       <c r="AB47" s="40"/>
       <c r="AC47" s="40"/>
       <c r="AD47" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6166,7 +6166,7 @@
       <c r="E48" s="14"/>
       <c r="F48" s="14"/>
       <c r="G48" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H48" s="14">
@@ -6180,7 +6180,7 @@
       <c r="N48" s="39"/>
       <c r="O48" s="40"/>
       <c r="P48" s="38">
-        <f>+SUM(H48:O48)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q48" s="39"/>
@@ -6192,7 +6192,7 @@
       <c r="W48" s="39"/>
       <c r="X48" s="39"/>
       <c r="Y48" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z48" s="41"/>
@@ -6200,7 +6200,7 @@
       <c r="AB48" s="40"/>
       <c r="AC48" s="40"/>
       <c r="AD48" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6219,7 +6219,7 @@
       <c r="E49" s="14"/>
       <c r="F49" s="14"/>
       <c r="G49" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H49" s="14">
@@ -6233,7 +6233,7 @@
       <c r="N49" s="39"/>
       <c r="O49" s="40"/>
       <c r="P49" s="38">
-        <f>+SUM(H49:O49)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q49" s="39"/>
@@ -6245,7 +6245,7 @@
       <c r="W49" s="39"/>
       <c r="X49" s="39"/>
       <c r="Y49" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z49" s="41"/>
@@ -6253,7 +6253,7 @@
       <c r="AB49" s="40"/>
       <c r="AC49" s="40"/>
       <c r="AD49" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6272,7 +6272,7 @@
       <c r="E50" s="14"/>
       <c r="F50" s="14"/>
       <c r="G50" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H50" s="14">
@@ -6286,7 +6286,7 @@
       <c r="N50" s="39"/>
       <c r="O50" s="39"/>
       <c r="P50" s="38">
-        <f>+SUM(H50:O50)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q50" s="39"/>
@@ -6298,7 +6298,7 @@
       <c r="W50" s="39"/>
       <c r="X50" s="39"/>
       <c r="Y50" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z50" s="41"/>
@@ -6306,7 +6306,7 @@
       <c r="AB50" s="40"/>
       <c r="AC50" s="40"/>
       <c r="AD50" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6325,7 +6325,7 @@
       <c r="E51" s="14"/>
       <c r="F51" s="14"/>
       <c r="G51" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H51" s="14">
@@ -6339,7 +6339,7 @@
       <c r="N51" s="39"/>
       <c r="O51" s="40"/>
       <c r="P51" s="38">
-        <f>+SUM(H51:O51)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q51" s="39"/>
@@ -6351,7 +6351,7 @@
       <c r="W51" s="39"/>
       <c r="X51" s="39"/>
       <c r="Y51" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z51" s="41"/>
@@ -6359,7 +6359,7 @@
       <c r="AB51" s="40"/>
       <c r="AC51" s="40"/>
       <c r="AD51" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6378,7 +6378,7 @@
       <c r="E52" s="14"/>
       <c r="F52" s="14"/>
       <c r="G52" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H52" s="14">
@@ -6392,7 +6392,7 @@
       <c r="N52" s="39"/>
       <c r="O52" s="40"/>
       <c r="P52" s="38">
-        <f>+SUM(H52:O52)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q52" s="39"/>
@@ -6404,7 +6404,7 @@
       <c r="W52" s="39"/>
       <c r="X52" s="39"/>
       <c r="Y52" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z52" s="41"/>
@@ -6412,7 +6412,7 @@
       <c r="AB52" s="40"/>
       <c r="AC52" s="40"/>
       <c r="AD52" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6431,7 +6431,7 @@
       <c r="E53" s="14"/>
       <c r="F53" s="14"/>
       <c r="G53" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H53" s="14">
@@ -6445,7 +6445,7 @@
       <c r="N53" s="39"/>
       <c r="O53" s="40"/>
       <c r="P53" s="38">
-        <f>+SUM(H53:O53)/8</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q53" s="39"/>
@@ -6457,7 +6457,7 @@
       <c r="W53" s="39"/>
       <c r="X53" s="39"/>
       <c r="Y53" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z53" s="40"/>
@@ -6465,7 +6465,7 @@
       <c r="AB53" s="40"/>
       <c r="AC53" s="40"/>
       <c r="AD53" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6485,7 +6485,7 @@
       <c r="E54" s="14"/>
       <c r="F54" s="14"/>
       <c r="G54" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H54" s="39"/>
@@ -6497,7 +6497,7 @@
       <c r="N54" s="39"/>
       <c r="O54" s="40"/>
       <c r="P54" s="38">
-        <f t="shared" ref="P6:P54" si="3">+SUM(H54:O54)/8</f>
+        <f t="shared" ref="P54" si="4">+SUM(H54:O54)/8</f>
         <v>0</v>
       </c>
       <c r="Q54" s="39"/>
@@ -6509,7 +6509,7 @@
       <c r="W54" s="39"/>
       <c r="X54" s="39"/>
       <c r="Y54" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="Z54" s="40"/>
@@ -6517,7 +6517,7 @@
       <c r="AB54" s="40"/>
       <c r="AC54" s="40"/>
       <c r="AD54" s="38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -6537,7 +6537,7 @@
       <c r="E55" s="14"/>
       <c r="F55" s="14"/>
       <c r="G55" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H55" s="39"/>
@@ -6549,7 +6549,7 @@
       <c r="N55" s="39"/>
       <c r="O55" s="39"/>
       <c r="P55" s="38">
-        <f t="shared" ref="P55:P64" si="4">+SUM(H55:O55)/8</f>
+        <f t="shared" ref="P55:P64" si="5">+SUM(H55:O55)/8</f>
         <v>0</v>
       </c>
       <c r="Q55" s="39"/>
@@ -6561,7 +6561,7 @@
       <c r="W55" s="39"/>
       <c r="X55" s="39"/>
       <c r="Y55" s="38">
-        <f t="shared" ref="Y55:Y64" si="5">+SUM(Q55:X55)/8</f>
+        <f t="shared" ref="Y55:Y64" si="6">+SUM(Q55:X55)/8</f>
         <v>0</v>
       </c>
       <c r="Z55" s="41"/>
@@ -6569,7 +6569,7 @@
       <c r="AB55" s="40"/>
       <c r="AC55" s="40"/>
       <c r="AD55" s="38">
-        <f t="shared" ref="AD55:AD64" si="6">+SUM(Z55:AC55)/4</f>
+        <f t="shared" ref="AD55:AD64" si="7">+SUM(Z55:AC55)/4</f>
         <v>0</v>
       </c>
     </row>
@@ -6589,7 +6589,7 @@
       <c r="E56" s="14"/>
       <c r="F56" s="14"/>
       <c r="G56" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H56" s="39"/>
@@ -6601,7 +6601,7 @@
       <c r="N56" s="39"/>
       <c r="O56" s="40"/>
       <c r="P56" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q56" s="39"/>
@@ -6613,7 +6613,7 @@
       <c r="W56" s="39"/>
       <c r="X56" s="39"/>
       <c r="Y56" s="38">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z56" s="41"/>
@@ -6621,7 +6621,7 @@
       <c r="AB56" s="40"/>
       <c r="AC56" s="40"/>
       <c r="AD56" s="38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -6641,7 +6641,7 @@
       <c r="E57" s="14"/>
       <c r="F57" s="14"/>
       <c r="G57" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H57" s="39"/>
@@ -6653,7 +6653,7 @@
       <c r="N57" s="39"/>
       <c r="O57" s="40"/>
       <c r="P57" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q57" s="39"/>
@@ -6665,7 +6665,7 @@
       <c r="W57" s="39"/>
       <c r="X57" s="39"/>
       <c r="Y57" s="38">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z57" s="41"/>
@@ -6673,7 +6673,7 @@
       <c r="AB57" s="40"/>
       <c r="AC57" s="40"/>
       <c r="AD57" s="38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -6693,7 +6693,7 @@
       <c r="E58" s="14"/>
       <c r="F58" s="14"/>
       <c r="G58" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H58" s="39"/>
@@ -6705,7 +6705,7 @@
       <c r="N58" s="39"/>
       <c r="O58" s="40"/>
       <c r="P58" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q58" s="39"/>
@@ -6717,7 +6717,7 @@
       <c r="W58" s="39"/>
       <c r="X58" s="39"/>
       <c r="Y58" s="38">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z58" s="40"/>
@@ -6725,7 +6725,7 @@
       <c r="AB58" s="40"/>
       <c r="AC58" s="40"/>
       <c r="AD58" s="38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -6745,7 +6745,7 @@
       <c r="E59" s="14"/>
       <c r="F59" s="14"/>
       <c r="G59" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H59" s="39"/>
@@ -6757,7 +6757,7 @@
       <c r="N59" s="39"/>
       <c r="O59" s="40"/>
       <c r="P59" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q59" s="39"/>
@@ -6769,7 +6769,7 @@
       <c r="W59" s="39"/>
       <c r="X59" s="39"/>
       <c r="Y59" s="38">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z59" s="40"/>
@@ -6777,7 +6777,7 @@
       <c r="AB59" s="40"/>
       <c r="AC59" s="40"/>
       <c r="AD59" s="38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -6797,7 +6797,7 @@
       <c r="E60" s="14"/>
       <c r="F60" s="14"/>
       <c r="G60" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H60" s="39"/>
@@ -6809,7 +6809,7 @@
       <c r="N60" s="39"/>
       <c r="O60" s="39"/>
       <c r="P60" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q60" s="39"/>
@@ -6821,7 +6821,7 @@
       <c r="W60" s="39"/>
       <c r="X60" s="39"/>
       <c r="Y60" s="38">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z60" s="41"/>
@@ -6829,7 +6829,7 @@
       <c r="AB60" s="40"/>
       <c r="AC60" s="40"/>
       <c r="AD60" s="38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -6849,7 +6849,7 @@
       <c r="E61" s="14"/>
       <c r="F61" s="14"/>
       <c r="G61" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H61" s="39"/>
@@ -6861,7 +6861,7 @@
       <c r="N61" s="39"/>
       <c r="O61" s="40"/>
       <c r="P61" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q61" s="39"/>
@@ -6873,7 +6873,7 @@
       <c r="W61" s="39"/>
       <c r="X61" s="39"/>
       <c r="Y61" s="38">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z61" s="41"/>
@@ -6881,7 +6881,7 @@
       <c r="AB61" s="40"/>
       <c r="AC61" s="40"/>
       <c r="AD61" s="38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       <c r="E62" s="14"/>
       <c r="F62" s="14"/>
       <c r="G62" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H62" s="39"/>
@@ -6913,7 +6913,7 @@
       <c r="N62" s="39"/>
       <c r="O62" s="40"/>
       <c r="P62" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q62" s="39"/>
@@ -6925,7 +6925,7 @@
       <c r="W62" s="39"/>
       <c r="X62" s="39"/>
       <c r="Y62" s="38">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z62" s="41"/>
@@ -6933,7 +6933,7 @@
       <c r="AB62" s="40"/>
       <c r="AC62" s="40"/>
       <c r="AD62" s="38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -6953,7 +6953,7 @@
       <c r="E63" s="14"/>
       <c r="F63" s="14"/>
       <c r="G63" s="38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H63" s="39"/>
@@ -6965,7 +6965,7 @@
       <c r="N63" s="39"/>
       <c r="O63" s="40"/>
       <c r="P63" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q63" s="39"/>
@@ -6977,7 +6977,7 @@
       <c r="W63" s="39"/>
       <c r="X63" s="39"/>
       <c r="Y63" s="38">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z63" s="40"/>
@@ -6985,7 +6985,7 @@
       <c r="AB63" s="40"/>
       <c r="AC63" s="40"/>
       <c r="AD63" s="38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -7017,7 +7017,7 @@
       <c r="N64" s="39"/>
       <c r="O64" s="40"/>
       <c r="P64" s="38">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="Q64" s="39"/>
@@ -7029,7 +7029,7 @@
       <c r="W64" s="39"/>
       <c r="X64" s="39"/>
       <c r="Y64" s="38">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="Z64" s="40"/>
@@ -7037,7 +7037,7 @@
       <c r="AB64" s="40"/>
       <c r="AC64" s="40"/>
       <c r="AD64" s="38">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -7087,123 +7087,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="96" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="126"/>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
-      <c r="F1" s="126"/>
-      <c r="G1" s="126"/>
-      <c r="H1" s="126"/>
-      <c r="I1" s="126"/>
-      <c r="J1" s="126"/>
-      <c r="K1" s="126"/>
-      <c r="L1" s="126"/>
-      <c r="M1" s="126"/>
-      <c r="N1" s="126"/>
-      <c r="O1" s="126"/>
-      <c r="P1" s="126"/>
-      <c r="Q1" s="126"/>
-      <c r="R1" s="126"/>
-      <c r="S1" s="126"/>
-      <c r="T1" s="126"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="96"/>
+      <c r="J1" s="96"/>
+      <c r="K1" s="96"/>
+      <c r="L1" s="96"/>
+      <c r="M1" s="96"/>
+      <c r="N1" s="96"/>
+      <c r="O1" s="96"/>
+      <c r="P1" s="96"/>
+      <c r="Q1" s="96"/>
+      <c r="R1" s="96"/>
+      <c r="S1" s="96"/>
+      <c r="T1" s="96"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="133" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="122" t="s">
+      <c r="B2" s="147" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="124" t="s">
+      <c r="C2" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="96" t="str">
+      <c r="D2" s="124" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="97"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="96" t="str">
+      <c r="E2" s="125"/>
+      <c r="F2" s="126"/>
+      <c r="G2" s="124" t="str">
         <f>Asistencia!H2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="97"/>
-      <c r="I2" s="97"/>
-      <c r="J2" s="97"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="96" t="s">
+      <c r="H2" s="125"/>
+      <c r="I2" s="125"/>
+      <c r="J2" s="125"/>
+      <c r="K2" s="126"/>
+      <c r="L2" s="124" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="97"/>
-      <c r="N2" s="97"/>
-      <c r="O2" s="97"/>
-      <c r="P2" s="98"/>
-      <c r="Q2" s="96" t="str">
+      <c r="M2" s="125"/>
+      <c r="N2" s="125"/>
+      <c r="O2" s="125"/>
+      <c r="P2" s="126"/>
+      <c r="Q2" s="124" t="str">
         <f>Asistencia!Z2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="97"/>
-      <c r="S2" s="97"/>
-      <c r="T2" s="98"/>
+      <c r="R2" s="125"/>
+      <c r="S2" s="125"/>
+      <c r="T2" s="126"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="109"/>
-      <c r="B3" s="123"/>
-      <c r="C3" s="125"/>
-      <c r="D3" s="116" t="s">
+      <c r="A3" s="134"/>
+      <c r="B3" s="148"/>
+      <c r="C3" s="150"/>
+      <c r="D3" s="141" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="117"/>
-      <c r="F3" s="118"/>
-      <c r="G3" s="110" t="s">
+      <c r="E3" s="142"/>
+      <c r="F3" s="143"/>
+      <c r="G3" s="135" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="112"/>
-      <c r="L3" s="145" t="s">
+      <c r="H3" s="136"/>
+      <c r="I3" s="136"/>
+      <c r="J3" s="136"/>
+      <c r="K3" s="137"/>
+      <c r="L3" s="118" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="146"/>
-      <c r="N3" s="146"/>
-      <c r="O3" s="146"/>
-      <c r="P3" s="147"/>
-      <c r="Q3" s="99" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="100"/>
-      <c r="S3" s="100"/>
-      <c r="T3" s="101"/>
+      <c r="M3" s="119"/>
+      <c r="N3" s="119"/>
+      <c r="O3" s="119"/>
+      <c r="P3" s="120"/>
+      <c r="Q3" s="127" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="128"/>
+      <c r="S3" s="128"/>
+      <c r="T3" s="129"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="109"/>
-      <c r="B4" s="123"/>
-      <c r="C4" s="125"/>
-      <c r="D4" s="119"/>
-      <c r="E4" s="120"/>
-      <c r="F4" s="121"/>
-      <c r="G4" s="113"/>
-      <c r="H4" s="114"/>
-      <c r="I4" s="114"/>
-      <c r="J4" s="114"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="148"/>
-      <c r="M4" s="149"/>
-      <c r="N4" s="149"/>
-      <c r="O4" s="149"/>
-      <c r="P4" s="150"/>
-      <c r="Q4" s="102"/>
-      <c r="R4" s="103"/>
-      <c r="S4" s="103"/>
-      <c r="T4" s="104"/>
+      <c r="A4" s="134"/>
+      <c r="B4" s="148"/>
+      <c r="C4" s="150"/>
+      <c r="D4" s="144"/>
+      <c r="E4" s="145"/>
+      <c r="F4" s="146"/>
+      <c r="G4" s="138"/>
+      <c r="H4" s="139"/>
+      <c r="I4" s="139"/>
+      <c r="J4" s="139"/>
+      <c r="K4" s="140"/>
+      <c r="L4" s="121"/>
+      <c r="M4" s="122"/>
+      <c r="N4" s="122"/>
+      <c r="O4" s="122"/>
+      <c r="P4" s="123"/>
+      <c r="Q4" s="130"/>
+      <c r="R4" s="131"/>
+      <c r="S4" s="131"/>
+      <c r="T4" s="132"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="109"/>
-      <c r="B5" s="123"/>
-      <c r="C5" s="125"/>
+      <c r="A5" s="134"/>
+      <c r="B5" s="148"/>
+      <c r="C5" s="150"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -9735,183 +9735,192 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D65" s="130" t="s">
+      <c r="D65" s="100" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="133" t="s">
+      <c r="E65" s="103" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="127" t="s">
+      <c r="G65" s="97" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="139" t="s">
+      <c r="H65" s="112" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="139" t="s">
+      <c r="I65" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="127" t="s">
+      <c r="J65" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="105" t="s">
+      <c r="L65" s="106" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="136" t="s">
+      <c r="M65" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="136" t="s">
+      <c r="N65" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="105" t="s">
+      <c r="O65" s="106" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="142" t="s">
+      <c r="Q65" s="115" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="142" t="s">
+      <c r="R65" s="115" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="142" t="s">
+      <c r="S65" s="115" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D66" s="131"/>
-      <c r="E66" s="134"/>
-      <c r="G66" s="128"/>
-      <c r="H66" s="140"/>
-      <c r="I66" s="140"/>
-      <c r="J66" s="128"/>
-      <c r="L66" s="106"/>
-      <c r="M66" s="137"/>
-      <c r="N66" s="137"/>
-      <c r="O66" s="106"/>
-      <c r="Q66" s="143"/>
-      <c r="R66" s="143"/>
-      <c r="S66" s="143"/>
+      <c r="D66" s="101"/>
+      <c r="E66" s="104"/>
+      <c r="G66" s="98"/>
+      <c r="H66" s="113"/>
+      <c r="I66" s="113"/>
+      <c r="J66" s="98"/>
+      <c r="L66" s="107"/>
+      <c r="M66" s="110"/>
+      <c r="N66" s="110"/>
+      <c r="O66" s="107"/>
+      <c r="Q66" s="116"/>
+      <c r="R66" s="116"/>
+      <c r="S66" s="116"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D67" s="131"/>
-      <c r="E67" s="134"/>
-      <c r="G67" s="128"/>
-      <c r="H67" s="140"/>
-      <c r="I67" s="140"/>
-      <c r="J67" s="128"/>
-      <c r="L67" s="106"/>
-      <c r="M67" s="137"/>
-      <c r="N67" s="137"/>
-      <c r="O67" s="106"/>
-      <c r="Q67" s="143"/>
-      <c r="R67" s="143"/>
-      <c r="S67" s="143"/>
+      <c r="D67" s="101"/>
+      <c r="E67" s="104"/>
+      <c r="G67" s="98"/>
+      <c r="H67" s="113"/>
+      <c r="I67" s="113"/>
+      <c r="J67" s="98"/>
+      <c r="L67" s="107"/>
+      <c r="M67" s="110"/>
+      <c r="N67" s="110"/>
+      <c r="O67" s="107"/>
+      <c r="Q67" s="116"/>
+      <c r="R67" s="116"/>
+      <c r="S67" s="116"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D68" s="131"/>
-      <c r="E68" s="134"/>
-      <c r="G68" s="128"/>
-      <c r="H68" s="140"/>
-      <c r="I68" s="140"/>
-      <c r="J68" s="128"/>
-      <c r="L68" s="106"/>
-      <c r="M68" s="137"/>
-      <c r="N68" s="137"/>
-      <c r="O68" s="106"/>
-      <c r="Q68" s="143"/>
-      <c r="R68" s="143"/>
-      <c r="S68" s="143"/>
+      <c r="D68" s="101"/>
+      <c r="E68" s="104"/>
+      <c r="G68" s="98"/>
+      <c r="H68" s="113"/>
+      <c r="I68" s="113"/>
+      <c r="J68" s="98"/>
+      <c r="L68" s="107"/>
+      <c r="M68" s="110"/>
+      <c r="N68" s="110"/>
+      <c r="O68" s="107"/>
+      <c r="Q68" s="116"/>
+      <c r="R68" s="116"/>
+      <c r="S68" s="116"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D69" s="131"/>
-      <c r="E69" s="134"/>
-      <c r="G69" s="128"/>
-      <c r="H69" s="140"/>
-      <c r="I69" s="140"/>
-      <c r="J69" s="128"/>
-      <c r="L69" s="106"/>
-      <c r="M69" s="137"/>
-      <c r="N69" s="137"/>
-      <c r="O69" s="106"/>
-      <c r="Q69" s="143"/>
-      <c r="R69" s="143"/>
-      <c r="S69" s="143"/>
+      <c r="D69" s="101"/>
+      <c r="E69" s="104"/>
+      <c r="G69" s="98"/>
+      <c r="H69" s="113"/>
+      <c r="I69" s="113"/>
+      <c r="J69" s="98"/>
+      <c r="L69" s="107"/>
+      <c r="M69" s="110"/>
+      <c r="N69" s="110"/>
+      <c r="O69" s="107"/>
+      <c r="Q69" s="116"/>
+      <c r="R69" s="116"/>
+      <c r="S69" s="116"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D70" s="131"/>
-      <c r="E70" s="134"/>
-      <c r="G70" s="128"/>
-      <c r="H70" s="140"/>
-      <c r="I70" s="140"/>
-      <c r="J70" s="128"/>
-      <c r="L70" s="106"/>
-      <c r="M70" s="137"/>
-      <c r="N70" s="137"/>
-      <c r="O70" s="106"/>
-      <c r="Q70" s="143"/>
-      <c r="R70" s="143"/>
-      <c r="S70" s="143"/>
+      <c r="D70" s="101"/>
+      <c r="E70" s="104"/>
+      <c r="G70" s="98"/>
+      <c r="H70" s="113"/>
+      <c r="I70" s="113"/>
+      <c r="J70" s="98"/>
+      <c r="L70" s="107"/>
+      <c r="M70" s="110"/>
+      <c r="N70" s="110"/>
+      <c r="O70" s="107"/>
+      <c r="Q70" s="116"/>
+      <c r="R70" s="116"/>
+      <c r="S70" s="116"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D71" s="131"/>
-      <c r="E71" s="134"/>
-      <c r="G71" s="128"/>
-      <c r="H71" s="140"/>
-      <c r="I71" s="140"/>
-      <c r="J71" s="128"/>
-      <c r="L71" s="106"/>
-      <c r="M71" s="137"/>
-      <c r="N71" s="137"/>
-      <c r="O71" s="106"/>
-      <c r="Q71" s="143"/>
-      <c r="R71" s="143"/>
-      <c r="S71" s="143"/>
+      <c r="D71" s="101"/>
+      <c r="E71" s="104"/>
+      <c r="G71" s="98"/>
+      <c r="H71" s="113"/>
+      <c r="I71" s="113"/>
+      <c r="J71" s="98"/>
+      <c r="L71" s="107"/>
+      <c r="M71" s="110"/>
+      <c r="N71" s="110"/>
+      <c r="O71" s="107"/>
+      <c r="Q71" s="116"/>
+      <c r="R71" s="116"/>
+      <c r="S71" s="116"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D72" s="131"/>
-      <c r="E72" s="134"/>
-      <c r="G72" s="128"/>
-      <c r="H72" s="140"/>
-      <c r="I72" s="140"/>
-      <c r="J72" s="128"/>
-      <c r="L72" s="106"/>
-      <c r="M72" s="137"/>
-      <c r="N72" s="137"/>
-      <c r="O72" s="106"/>
-      <c r="Q72" s="143"/>
-      <c r="R72" s="143"/>
-      <c r="S72" s="143"/>
+      <c r="D72" s="101"/>
+      <c r="E72" s="104"/>
+      <c r="G72" s="98"/>
+      <c r="H72" s="113"/>
+      <c r="I72" s="113"/>
+      <c r="J72" s="98"/>
+      <c r="L72" s="107"/>
+      <c r="M72" s="110"/>
+      <c r="N72" s="110"/>
+      <c r="O72" s="107"/>
+      <c r="Q72" s="116"/>
+      <c r="R72" s="116"/>
+      <c r="S72" s="116"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D73" s="131"/>
-      <c r="E73" s="134"/>
-      <c r="G73" s="128"/>
-      <c r="H73" s="140"/>
-      <c r="I73" s="140"/>
-      <c r="J73" s="128"/>
-      <c r="L73" s="106"/>
-      <c r="M73" s="137"/>
-      <c r="N73" s="137"/>
-      <c r="O73" s="106"/>
-      <c r="Q73" s="143"/>
-      <c r="R73" s="143"/>
-      <c r="S73" s="143"/>
+      <c r="D73" s="101"/>
+      <c r="E73" s="104"/>
+      <c r="G73" s="98"/>
+      <c r="H73" s="113"/>
+      <c r="I73" s="113"/>
+      <c r="J73" s="98"/>
+      <c r="L73" s="107"/>
+      <c r="M73" s="110"/>
+      <c r="N73" s="110"/>
+      <c r="O73" s="107"/>
+      <c r="Q73" s="116"/>
+      <c r="R73" s="116"/>
+      <c r="S73" s="116"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D74" s="132"/>
-      <c r="E74" s="135"/>
-      <c r="G74" s="129"/>
-      <c r="H74" s="141"/>
-      <c r="I74" s="141"/>
-      <c r="J74" s="129"/>
-      <c r="L74" s="107"/>
-      <c r="M74" s="138"/>
-      <c r="N74" s="138"/>
-      <c r="O74" s="107"/>
-      <c r="Q74" s="144"/>
-      <c r="R74" s="144"/>
-      <c r="S74" s="144"/>
+      <c r="D74" s="102"/>
+      <c r="E74" s="105"/>
+      <c r="G74" s="99"/>
+      <c r="H74" s="114"/>
+      <c r="I74" s="114"/>
+      <c r="J74" s="99"/>
+      <c r="L74" s="108"/>
+      <c r="M74" s="111"/>
+      <c r="N74" s="111"/>
+      <c r="O74" s="108"/>
+      <c r="Q74" s="117"/>
+      <c r="R74" s="117"/>
+      <c r="S74" s="117"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -9928,15 +9937,6 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
diagnostico en geometría y operaciones no convenciaonales
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3318277F-797B-48CC-8D0A-B59D2454A15B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93206883-83FD-46DF-AF41-400E3F755C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="249">
   <si>
     <t>METODOLOGÍA DE ESTUDIO</t>
   </si>
@@ -773,6 +773,18 @@
   </si>
   <si>
     <t>MARÍA ISABEL QUIÑONES HERNÁNDEZ@gmail.COM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dairo jose Montiel Muñoz </t>
+  </si>
+  <si>
+    <t>cc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El porvenir </t>
+  </si>
+  <si>
+    <t xml:space="preserve">momtieldairo@gmail.com </t>
   </si>
 </sst>
 </file>
@@ -1241,7 +1253,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="151">
+  <cellXfs count="152">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1420,6 +1432,18 @@
       <alignment horizontal="justify" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="12" borderId="1" xfId="3" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1510,16 +1534,94 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1552,15 +1654,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1606,86 +1699,8 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2193,28 +2208,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="95"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="65"/>
     </row>
     <row r="2" spans="1:8" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="92"/>
-      <c r="C2" s="92"/>
-      <c r="D2" s="92"/>
-      <c r="E2" s="92"/>
-      <c r="F2" s="92"/>
-      <c r="G2" s="92"/>
-      <c r="H2" s="92"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -3542,13 +3557,27 @@
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="B52" s="50"/>
-      <c r="C52" s="51"/>
-      <c r="D52" s="47"/>
-      <c r="E52" s="45"/>
-      <c r="F52" s="15"/>
-      <c r="G52" s="18"/>
-      <c r="H52" s="52"/>
+      <c r="B52" s="50" t="s">
+        <v>245</v>
+      </c>
+      <c r="C52" s="51" t="s">
+        <v>246</v>
+      </c>
+      <c r="D52" s="47">
+        <v>1063358976</v>
+      </c>
+      <c r="E52" s="45" t="s">
+        <v>247</v>
+      </c>
+      <c r="F52" s="15">
+        <v>3001754755</v>
+      </c>
+      <c r="G52" s="151" t="s">
+        <v>248</v>
+      </c>
+      <c r="H52" s="52" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="53" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="44">
@@ -3696,10 +3725,11 @@
     <hyperlink ref="G43" r:id="rId1" xr:uid="{8BB50FD2-7F54-4B64-A918-7390D521BAFB}"/>
     <hyperlink ref="G17" r:id="rId2" xr:uid="{092C4A61-E23C-4BF6-9661-B7CE860226C9}"/>
     <hyperlink ref="G46" r:id="rId3" xr:uid="{042E7418-FA4C-4F84-A42C-9C4C96034294}"/>
+    <hyperlink ref="G52" r:id="rId4" xr:uid="{62763121-B2C7-4BA6-9D17-0FBBCE3C3654}"/>
   </hyperlinks>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="80" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId4"/>
-  <drawing r:id="rId5"/>
+  <pageSetup scale="80" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId5"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
 
@@ -3723,37 +3753,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="69" t="s">
+      <c r="B1" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
-      <c r="S1" s="69"/>
-      <c r="T1" s="69"/>
-      <c r="U1" s="69"/>
-      <c r="V1" s="69"/>
-      <c r="W1" s="69"/>
-      <c r="X1" s="69"/>
-      <c r="Y1" s="69"/>
-      <c r="Z1" s="69"/>
-      <c r="AA1" s="69"/>
-      <c r="AB1" s="69"/>
-      <c r="AC1" s="69"/>
-      <c r="AD1" s="69"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="73"/>
+      <c r="Q1" s="73"/>
+      <c r="R1" s="73"/>
+      <c r="S1" s="73"/>
+      <c r="T1" s="73"/>
+      <c r="U1" s="73"/>
+      <c r="V1" s="73"/>
+      <c r="W1" s="73"/>
+      <c r="X1" s="73"/>
+      <c r="Y1" s="73"/>
+      <c r="Z1" s="73"/>
+      <c r="AA1" s="73"/>
+      <c r="AB1" s="73"/>
+      <c r="AC1" s="73"/>
+      <c r="AD1" s="73"/>
     </row>
     <row r="2" spans="1:30" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="55" t="s">
@@ -3765,120 +3795,120 @@
       <c r="C2" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="85" t="s">
+      <c r="D2" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="87"/>
-      <c r="H2" s="70" t="s">
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71"/>
-      <c r="O2" s="71"/>
-      <c r="P2" s="72"/>
-      <c r="Q2" s="79" t="s">
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="75"/>
+      <c r="M2" s="75"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="75"/>
+      <c r="P2" s="76"/>
+      <c r="Q2" s="83" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="80"/>
-      <c r="S2" s="80"/>
-      <c r="T2" s="80"/>
-      <c r="U2" s="80"/>
-      <c r="V2" s="80"/>
-      <c r="W2" s="80"/>
-      <c r="X2" s="80"/>
-      <c r="Y2" s="81"/>
-      <c r="Z2" s="62" t="s">
+      <c r="R2" s="84"/>
+      <c r="S2" s="84"/>
+      <c r="T2" s="84"/>
+      <c r="U2" s="84"/>
+      <c r="V2" s="84"/>
+      <c r="W2" s="84"/>
+      <c r="X2" s="84"/>
+      <c r="Y2" s="85"/>
+      <c r="Z2" s="66" t="s">
         <v>21</v>
       </c>
-      <c r="AA2" s="63"/>
-      <c r="AB2" s="63"/>
-      <c r="AC2" s="63"/>
-      <c r="AD2" s="64"/>
+      <c r="AA2" s="67"/>
+      <c r="AB2" s="67"/>
+      <c r="AC2" s="67"/>
+      <c r="AD2" s="68"/>
     </row>
     <row r="3" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="56"/>
       <c r="B3" s="54"/>
       <c r="C3" s="56"/>
-      <c r="D3" s="88" t="s">
+      <c r="D3" s="92" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="73" t="s">
+      <c r="E3" s="93"/>
+      <c r="F3" s="93"/>
+      <c r="G3" s="94"/>
+      <c r="H3" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="74"/>
-      <c r="J3" s="74"/>
-      <c r="K3" s="74"/>
-      <c r="L3" s="74"/>
-      <c r="M3" s="74"/>
-      <c r="N3" s="74"/>
-      <c r="O3" s="74"/>
-      <c r="P3" s="75"/>
-      <c r="Q3" s="82" t="s">
+      <c r="I3" s="78"/>
+      <c r="J3" s="78"/>
+      <c r="K3" s="78"/>
+      <c r="L3" s="78"/>
+      <c r="M3" s="78"/>
+      <c r="N3" s="78"/>
+      <c r="O3" s="78"/>
+      <c r="P3" s="79"/>
+      <c r="Q3" s="86" t="s">
         <v>1</v>
       </c>
-      <c r="R3" s="83"/>
-      <c r="S3" s="83"/>
-      <c r="T3" s="83"/>
-      <c r="U3" s="83"/>
-      <c r="V3" s="83"/>
-      <c r="W3" s="83"/>
-      <c r="X3" s="83"/>
-      <c r="Y3" s="84"/>
-      <c r="Z3" s="65" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="66"/>
-      <c r="AB3" s="66"/>
-      <c r="AC3" s="66"/>
-      <c r="AD3" s="67"/>
+      <c r="R3" s="87"/>
+      <c r="S3" s="87"/>
+      <c r="T3" s="87"/>
+      <c r="U3" s="87"/>
+      <c r="V3" s="87"/>
+      <c r="W3" s="87"/>
+      <c r="X3" s="87"/>
+      <c r="Y3" s="88"/>
+      <c r="Z3" s="69" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="70"/>
+      <c r="AB3" s="70"/>
+      <c r="AC3" s="70"/>
+      <c r="AD3" s="71"/>
     </row>
     <row r="4" spans="1:30" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="56"/>
       <c r="B4" s="54"/>
       <c r="C4" s="56"/>
-      <c r="D4" s="91" t="s">
+      <c r="D4" s="95" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="77"/>
-      <c r="F4" s="77"/>
+      <c r="E4" s="81"/>
+      <c r="F4" s="81"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="76" t="s">
+      <c r="H4" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="77"/>
-      <c r="J4" s="77"/>
-      <c r="K4" s="77"/>
-      <c r="L4" s="77"/>
-      <c r="M4" s="77"/>
-      <c r="N4" s="77"/>
-      <c r="O4" s="78"/>
+      <c r="I4" s="81"/>
+      <c r="J4" s="81"/>
+      <c r="K4" s="81"/>
+      <c r="L4" s="81"/>
+      <c r="M4" s="81"/>
+      <c r="N4" s="81"/>
+      <c r="O4" s="82"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="76" t="s">
+      <c r="Q4" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="R4" s="77"/>
-      <c r="S4" s="77"/>
-      <c r="T4" s="77"/>
-      <c r="U4" s="77"/>
-      <c r="V4" s="77"/>
-      <c r="W4" s="77"/>
-      <c r="X4" s="78"/>
+      <c r="R4" s="81"/>
+      <c r="S4" s="81"/>
+      <c r="T4" s="81"/>
+      <c r="U4" s="81"/>
+      <c r="V4" s="81"/>
+      <c r="W4" s="81"/>
+      <c r="X4" s="82"/>
       <c r="Y4" s="13"/>
-      <c r="Z4" s="68" t="s">
+      <c r="Z4" s="72" t="s">
         <v>24</v>
       </c>
-      <c r="AA4" s="68"/>
-      <c r="AB4" s="68"/>
-      <c r="AC4" s="68"/>
+      <c r="AA4" s="72"/>
+      <c r="AB4" s="72"/>
+      <c r="AC4" s="72"/>
       <c r="AD4" s="3"/>
     </row>
     <row r="5" spans="1:30" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -6473,13 +6503,13 @@
       <c r="A54" s="21">
         <v>49</v>
       </c>
-      <c r="B54" s="19">
+      <c r="B54" s="19" t="str">
         <f>+Inscritos!B52</f>
-        <v>0</v>
+        <v xml:space="preserve">Dairo jose Montiel Muñoz </v>
       </c>
       <c r="C54" s="22">
         <f>+Inscritos!D52</f>
-        <v>0</v>
+        <v>1063358976</v>
       </c>
       <c r="D54" s="14"/>
       <c r="E54" s="14"/>
@@ -7087,123 +7117,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="96" t="s">
+      <c r="B1" s="126" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="96"/>
-      <c r="K1" s="96"/>
-      <c r="L1" s="96"/>
-      <c r="M1" s="96"/>
-      <c r="N1" s="96"/>
-      <c r="O1" s="96"/>
-      <c r="P1" s="96"/>
-      <c r="Q1" s="96"/>
-      <c r="R1" s="96"/>
-      <c r="S1" s="96"/>
-      <c r="T1" s="96"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+      <c r="I1" s="126"/>
+      <c r="J1" s="126"/>
+      <c r="K1" s="126"/>
+      <c r="L1" s="126"/>
+      <c r="M1" s="126"/>
+      <c r="N1" s="126"/>
+      <c r="O1" s="126"/>
+      <c r="P1" s="126"/>
+      <c r="Q1" s="126"/>
+      <c r="R1" s="126"/>
+      <c r="S1" s="126"/>
+      <c r="T1" s="126"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="133" t="s">
+      <c r="A2" s="108" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="147" t="s">
+      <c r="B2" s="122" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="149" t="s">
+      <c r="C2" s="124" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="124" t="str">
+      <c r="D2" s="96" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="125"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="124" t="str">
+      <c r="E2" s="97"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="96" t="str">
         <f>Asistencia!H2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="125"/>
-      <c r="I2" s="125"/>
-      <c r="J2" s="125"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="124" t="s">
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="96" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="125"/>
-      <c r="N2" s="125"/>
-      <c r="O2" s="125"/>
-      <c r="P2" s="126"/>
-      <c r="Q2" s="124" t="str">
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
+      <c r="P2" s="98"/>
+      <c r="Q2" s="96" t="str">
         <f>Asistencia!Z2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="125"/>
-      <c r="S2" s="125"/>
-      <c r="T2" s="126"/>
+      <c r="R2" s="97"/>
+      <c r="S2" s="97"/>
+      <c r="T2" s="98"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="134"/>
-      <c r="B3" s="148"/>
-      <c r="C3" s="150"/>
-      <c r="D3" s="141" t="s">
+      <c r="A3" s="109"/>
+      <c r="B3" s="123"/>
+      <c r="C3" s="125"/>
+      <c r="D3" s="116" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="142"/>
-      <c r="F3" s="143"/>
-      <c r="G3" s="135" t="s">
+      <c r="E3" s="117"/>
+      <c r="F3" s="118"/>
+      <c r="G3" s="110" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="136"/>
-      <c r="I3" s="136"/>
-      <c r="J3" s="136"/>
-      <c r="K3" s="137"/>
-      <c r="L3" s="118" t="s">
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="112"/>
+      <c r="L3" s="145" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="119"/>
-      <c r="N3" s="119"/>
-      <c r="O3" s="119"/>
-      <c r="P3" s="120"/>
-      <c r="Q3" s="127" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="128"/>
-      <c r="S3" s="128"/>
-      <c r="T3" s="129"/>
+      <c r="M3" s="146"/>
+      <c r="N3" s="146"/>
+      <c r="O3" s="146"/>
+      <c r="P3" s="147"/>
+      <c r="Q3" s="99" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="100"/>
+      <c r="S3" s="100"/>
+      <c r="T3" s="101"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="134"/>
-      <c r="B4" s="148"/>
-      <c r="C4" s="150"/>
-      <c r="D4" s="144"/>
-      <c r="E4" s="145"/>
-      <c r="F4" s="146"/>
-      <c r="G4" s="138"/>
-      <c r="H4" s="139"/>
-      <c r="I4" s="139"/>
-      <c r="J4" s="139"/>
-      <c r="K4" s="140"/>
-      <c r="L4" s="121"/>
-      <c r="M4" s="122"/>
-      <c r="N4" s="122"/>
-      <c r="O4" s="122"/>
-      <c r="P4" s="123"/>
-      <c r="Q4" s="130"/>
-      <c r="R4" s="131"/>
-      <c r="S4" s="131"/>
-      <c r="T4" s="132"/>
+      <c r="A4" s="109"/>
+      <c r="B4" s="123"/>
+      <c r="C4" s="125"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="120"/>
+      <c r="F4" s="121"/>
+      <c r="G4" s="113"/>
+      <c r="H4" s="114"/>
+      <c r="I4" s="114"/>
+      <c r="J4" s="114"/>
+      <c r="K4" s="115"/>
+      <c r="L4" s="148"/>
+      <c r="M4" s="149"/>
+      <c r="N4" s="149"/>
+      <c r="O4" s="149"/>
+      <c r="P4" s="150"/>
+      <c r="Q4" s="102"/>
+      <c r="R4" s="103"/>
+      <c r="S4" s="103"/>
+      <c r="T4" s="104"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="134"/>
-      <c r="B5" s="148"/>
-      <c r="C5" s="150"/>
+      <c r="A5" s="109"/>
+      <c r="B5" s="123"/>
+      <c r="C5" s="125"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -9276,13 +9306,13 @@
       <c r="A54" s="10">
         <v>49</v>
       </c>
-      <c r="B54" s="19">
+      <c r="B54" s="19" t="str">
         <f>Inscritos!B52</f>
-        <v>0</v>
+        <v xml:space="preserve">Dairo jose Montiel Muñoz </v>
       </c>
       <c r="C54" s="19">
         <f>+Inscritos!D52</f>
-        <v>0</v>
+        <v>1063358976</v>
       </c>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
@@ -9735,192 +9765,183 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D65" s="100" t="s">
+      <c r="D65" s="130" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="103" t="s">
+      <c r="E65" s="133" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="97" t="s">
+      <c r="G65" s="127" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="112" t="s">
+      <c r="H65" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="112" t="s">
+      <c r="I65" s="139" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="97" t="s">
+      <c r="J65" s="127" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="106" t="s">
+      <c r="L65" s="105" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="109" t="s">
+      <c r="M65" s="136" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="109" t="s">
+      <c r="N65" s="136" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="106" t="s">
+      <c r="O65" s="105" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="115" t="s">
+      <c r="Q65" s="142" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="115" t="s">
+      <c r="R65" s="142" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="115" t="s">
+      <c r="S65" s="142" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D66" s="101"/>
-      <c r="E66" s="104"/>
-      <c r="G66" s="98"/>
-      <c r="H66" s="113"/>
-      <c r="I66" s="113"/>
-      <c r="J66" s="98"/>
-      <c r="L66" s="107"/>
-      <c r="M66" s="110"/>
-      <c r="N66" s="110"/>
-      <c r="O66" s="107"/>
-      <c r="Q66" s="116"/>
-      <c r="R66" s="116"/>
-      <c r="S66" s="116"/>
+      <c r="D66" s="131"/>
+      <c r="E66" s="134"/>
+      <c r="G66" s="128"/>
+      <c r="H66" s="140"/>
+      <c r="I66" s="140"/>
+      <c r="J66" s="128"/>
+      <c r="L66" s="106"/>
+      <c r="M66" s="137"/>
+      <c r="N66" s="137"/>
+      <c r="O66" s="106"/>
+      <c r="Q66" s="143"/>
+      <c r="R66" s="143"/>
+      <c r="S66" s="143"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D67" s="101"/>
-      <c r="E67" s="104"/>
-      <c r="G67" s="98"/>
-      <c r="H67" s="113"/>
-      <c r="I67" s="113"/>
-      <c r="J67" s="98"/>
-      <c r="L67" s="107"/>
-      <c r="M67" s="110"/>
-      <c r="N67" s="110"/>
-      <c r="O67" s="107"/>
-      <c r="Q67" s="116"/>
-      <c r="R67" s="116"/>
-      <c r="S67" s="116"/>
+      <c r="D67" s="131"/>
+      <c r="E67" s="134"/>
+      <c r="G67" s="128"/>
+      <c r="H67" s="140"/>
+      <c r="I67" s="140"/>
+      <c r="J67" s="128"/>
+      <c r="L67" s="106"/>
+      <c r="M67" s="137"/>
+      <c r="N67" s="137"/>
+      <c r="O67" s="106"/>
+      <c r="Q67" s="143"/>
+      <c r="R67" s="143"/>
+      <c r="S67" s="143"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D68" s="101"/>
-      <c r="E68" s="104"/>
-      <c r="G68" s="98"/>
-      <c r="H68" s="113"/>
-      <c r="I68" s="113"/>
-      <c r="J68" s="98"/>
-      <c r="L68" s="107"/>
-      <c r="M68" s="110"/>
-      <c r="N68" s="110"/>
-      <c r="O68" s="107"/>
-      <c r="Q68" s="116"/>
-      <c r="R68" s="116"/>
-      <c r="S68" s="116"/>
+      <c r="D68" s="131"/>
+      <c r="E68" s="134"/>
+      <c r="G68" s="128"/>
+      <c r="H68" s="140"/>
+      <c r="I68" s="140"/>
+      <c r="J68" s="128"/>
+      <c r="L68" s="106"/>
+      <c r="M68" s="137"/>
+      <c r="N68" s="137"/>
+      <c r="O68" s="106"/>
+      <c r="Q68" s="143"/>
+      <c r="R68" s="143"/>
+      <c r="S68" s="143"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D69" s="101"/>
-      <c r="E69" s="104"/>
-      <c r="G69" s="98"/>
-      <c r="H69" s="113"/>
-      <c r="I69" s="113"/>
-      <c r="J69" s="98"/>
-      <c r="L69" s="107"/>
-      <c r="M69" s="110"/>
-      <c r="N69" s="110"/>
-      <c r="O69" s="107"/>
-      <c r="Q69" s="116"/>
-      <c r="R69" s="116"/>
-      <c r="S69" s="116"/>
+      <c r="D69" s="131"/>
+      <c r="E69" s="134"/>
+      <c r="G69" s="128"/>
+      <c r="H69" s="140"/>
+      <c r="I69" s="140"/>
+      <c r="J69" s="128"/>
+      <c r="L69" s="106"/>
+      <c r="M69" s="137"/>
+      <c r="N69" s="137"/>
+      <c r="O69" s="106"/>
+      <c r="Q69" s="143"/>
+      <c r="R69" s="143"/>
+      <c r="S69" s="143"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D70" s="101"/>
-      <c r="E70" s="104"/>
-      <c r="G70" s="98"/>
-      <c r="H70" s="113"/>
-      <c r="I70" s="113"/>
-      <c r="J70" s="98"/>
-      <c r="L70" s="107"/>
-      <c r="M70" s="110"/>
-      <c r="N70" s="110"/>
-      <c r="O70" s="107"/>
-      <c r="Q70" s="116"/>
-      <c r="R70" s="116"/>
-      <c r="S70" s="116"/>
+      <c r="D70" s="131"/>
+      <c r="E70" s="134"/>
+      <c r="G70" s="128"/>
+      <c r="H70" s="140"/>
+      <c r="I70" s="140"/>
+      <c r="J70" s="128"/>
+      <c r="L70" s="106"/>
+      <c r="M70" s="137"/>
+      <c r="N70" s="137"/>
+      <c r="O70" s="106"/>
+      <c r="Q70" s="143"/>
+      <c r="R70" s="143"/>
+      <c r="S70" s="143"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D71" s="101"/>
-      <c r="E71" s="104"/>
-      <c r="G71" s="98"/>
-      <c r="H71" s="113"/>
-      <c r="I71" s="113"/>
-      <c r="J71" s="98"/>
-      <c r="L71" s="107"/>
-      <c r="M71" s="110"/>
-      <c r="N71" s="110"/>
-      <c r="O71" s="107"/>
-      <c r="Q71" s="116"/>
-      <c r="R71" s="116"/>
-      <c r="S71" s="116"/>
+      <c r="D71" s="131"/>
+      <c r="E71" s="134"/>
+      <c r="G71" s="128"/>
+      <c r="H71" s="140"/>
+      <c r="I71" s="140"/>
+      <c r="J71" s="128"/>
+      <c r="L71" s="106"/>
+      <c r="M71" s="137"/>
+      <c r="N71" s="137"/>
+      <c r="O71" s="106"/>
+      <c r="Q71" s="143"/>
+      <c r="R71" s="143"/>
+      <c r="S71" s="143"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D72" s="101"/>
-      <c r="E72" s="104"/>
-      <c r="G72" s="98"/>
-      <c r="H72" s="113"/>
-      <c r="I72" s="113"/>
-      <c r="J72" s="98"/>
-      <c r="L72" s="107"/>
-      <c r="M72" s="110"/>
-      <c r="N72" s="110"/>
-      <c r="O72" s="107"/>
-      <c r="Q72" s="116"/>
-      <c r="R72" s="116"/>
-      <c r="S72" s="116"/>
+      <c r="D72" s="131"/>
+      <c r="E72" s="134"/>
+      <c r="G72" s="128"/>
+      <c r="H72" s="140"/>
+      <c r="I72" s="140"/>
+      <c r="J72" s="128"/>
+      <c r="L72" s="106"/>
+      <c r="M72" s="137"/>
+      <c r="N72" s="137"/>
+      <c r="O72" s="106"/>
+      <c r="Q72" s="143"/>
+      <c r="R72" s="143"/>
+      <c r="S72" s="143"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D73" s="101"/>
-      <c r="E73" s="104"/>
-      <c r="G73" s="98"/>
-      <c r="H73" s="113"/>
-      <c r="I73" s="113"/>
-      <c r="J73" s="98"/>
-      <c r="L73" s="107"/>
-      <c r="M73" s="110"/>
-      <c r="N73" s="110"/>
-      <c r="O73" s="107"/>
-      <c r="Q73" s="116"/>
-      <c r="R73" s="116"/>
-      <c r="S73" s="116"/>
+      <c r="D73" s="131"/>
+      <c r="E73" s="134"/>
+      <c r="G73" s="128"/>
+      <c r="H73" s="140"/>
+      <c r="I73" s="140"/>
+      <c r="J73" s="128"/>
+      <c r="L73" s="106"/>
+      <c r="M73" s="137"/>
+      <c r="N73" s="137"/>
+      <c r="O73" s="106"/>
+      <c r="Q73" s="143"/>
+      <c r="R73" s="143"/>
+      <c r="S73" s="143"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D74" s="102"/>
-      <c r="E74" s="105"/>
-      <c r="G74" s="99"/>
-      <c r="H74" s="114"/>
-      <c r="I74" s="114"/>
-      <c r="J74" s="99"/>
-      <c r="L74" s="108"/>
-      <c r="M74" s="111"/>
-      <c r="N74" s="111"/>
-      <c r="O74" s="108"/>
-      <c r="Q74" s="117"/>
-      <c r="R74" s="117"/>
-      <c r="S74" s="117"/>
+      <c r="D74" s="132"/>
+      <c r="E74" s="135"/>
+      <c r="G74" s="129"/>
+      <c r="H74" s="141"/>
+      <c r="I74" s="141"/>
+      <c r="J74" s="129"/>
+      <c r="L74" s="107"/>
+      <c r="M74" s="138"/>
+      <c r="N74" s="138"/>
+      <c r="O74" s="107"/>
+      <c r="Q74" s="144"/>
+      <c r="R74" s="144"/>
+      <c r="S74" s="144"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -9937,6 +9958,15 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
voy a preparar clase para mañana 13 de junio
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93206883-83FD-46DF-AF41-400E3F755C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACEE989-BB64-45A9-B5A8-6795D148C788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="251">
   <si>
     <t>METODOLOGÍA DE ESTUDIO</t>
   </si>
@@ -187,9 +187,6 @@
     <t>CAMILO JIMÉNEZ</t>
   </si>
   <si>
-    <t>VERONICAARRIETA297GMAIL.COM</t>
-  </si>
-  <si>
     <t xml:space="preserve">ANDRES EDUARDO CISNEROS MARTINEZ </t>
   </si>
   <si>
@@ -400,9 +397,6 @@
     <t>RAMON RUBIO</t>
   </si>
   <si>
-    <t>ELKINQUINTERO4720@GMAIL.COM</t>
-  </si>
-  <si>
     <t xml:space="preserve">EMILYS PATRICIA OVIEDO ROMERO </t>
   </si>
   <si>
@@ -472,9 +466,6 @@
     <t>3114199768</t>
   </si>
   <si>
-    <t>TUIRANCUIVAK@GMAIL.COM</t>
-  </si>
-  <si>
     <t>ANGEL GABRIEL ARROYO ARRIETA</t>
   </si>
   <si>
@@ -553,9 +544,6 @@
     <t>3022710092</t>
   </si>
   <si>
-    <t>DUBERNEYJARAMILLO04@GMAIL.COM</t>
-  </si>
-  <si>
     <t xml:space="preserve">LENIS ENITH ORTEGA FUENTES </t>
   </si>
   <si>
@@ -772,9 +760,6 @@
     <t>SOFIASAGA36@GMaIL.COM</t>
   </si>
   <si>
-    <t>MARÍA ISABEL QUIÑONES HERNÁNDEZ@gmail.COM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dairo jose Montiel Muñoz </t>
   </si>
   <si>
@@ -785,6 +770,27 @@
   </si>
   <si>
     <t xml:space="preserve">momtieldairo@gmail.com </t>
+  </si>
+  <si>
+    <t>mariaisabelquiñoneshernandez@gmail.com</t>
+  </si>
+  <si>
+    <t>VERONICAARRIETA297@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>DUBERNEYJARAMILLO09@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>tuirancuitivak@gmail.com</t>
+  </si>
+  <si>
+    <t>6 de junio</t>
+  </si>
+  <si>
+    <t>13 de junio</t>
+  </si>
+  <si>
+    <t>elkinq719@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1253,7 +1259,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1428,10 +1434,16 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" xfId="3" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="1" xfId="3" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1698,9 +1710,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2208,28 +2217,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="65"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="67"/>
     </row>
     <row r="2" spans="1:8" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -2262,25 +2271,25 @@
         <v>1</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C4" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D4" s="59" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="E4" s="57" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="F4" s="59" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G4" s="57" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="H4" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2289,25 +2298,25 @@
         <v>2</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C5" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="59" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="E5" s="57" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="F5" s="59" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="G5" s="57" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="H5" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2316,25 +2325,25 @@
         <v>3</v>
       </c>
       <c r="B6" s="57" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C6" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D6" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="E6" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="E6" s="57" t="s">
+      <c r="F6" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="59" t="s">
+      <c r="G6" s="57" t="s">
         <v>61</v>
       </c>
-      <c r="G6" s="57" t="s">
-        <v>62</v>
-      </c>
       <c r="H6" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2343,25 +2352,25 @@
         <v>4</v>
       </c>
       <c r="B7" s="57" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C7" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="59" t="s">
+        <v>82</v>
+      </c>
+      <c r="E7" s="57" t="s">
         <v>83</v>
       </c>
-      <c r="E7" s="57" t="s">
+      <c r="F7" s="59" t="s">
         <v>84</v>
       </c>
-      <c r="F7" s="59" t="s">
+      <c r="G7" s="57" t="s">
         <v>85</v>
       </c>
-      <c r="G7" s="57" t="s">
-        <v>86</v>
-      </c>
       <c r="H7" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2370,7 +2379,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="57" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C8" s="57" t="s">
         <v>29</v>
@@ -2379,16 +2388,16 @@
         <v>1063359856</v>
       </c>
       <c r="E8" s="57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F8" s="59" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G8" s="57" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H8" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2397,25 +2406,25 @@
         <v>6</v>
       </c>
       <c r="B9" s="57" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C9" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="59" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E9" s="57" t="s">
         <v>48</v>
       </c>
       <c r="F9" s="59" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="57" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="57" t="s">
-        <v>53</v>
-      </c>
       <c r="H9" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2424,25 +2433,25 @@
         <v>7</v>
       </c>
       <c r="B10" s="57" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C10" s="57" t="s">
         <v>30</v>
       </c>
       <c r="D10" s="59" t="s">
+        <v>143</v>
+      </c>
+      <c r="E10" s="57" t="s">
+        <v>144</v>
+      </c>
+      <c r="F10" s="59" t="s">
+        <v>145</v>
+      </c>
+      <c r="G10" s="57" t="s">
         <v>146</v>
       </c>
-      <c r="E10" s="57" t="s">
-        <v>147</v>
-      </c>
-      <c r="F10" s="59" t="s">
-        <v>148</v>
-      </c>
-      <c r="G10" s="57" t="s">
-        <v>149</v>
-      </c>
       <c r="H10" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2451,25 +2460,25 @@
         <v>8</v>
       </c>
       <c r="B11" s="57" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C11" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="59" t="s">
+        <v>148</v>
+      </c>
+      <c r="E11" s="57" t="s">
+        <v>149</v>
+      </c>
+      <c r="F11" s="59" t="s">
+        <v>150</v>
+      </c>
+      <c r="G11" s="57" t="s">
         <v>151</v>
       </c>
-      <c r="E11" s="57" t="s">
-        <v>152</v>
-      </c>
-      <c r="F11" s="59" t="s">
-        <v>153</v>
-      </c>
-      <c r="G11" s="57" t="s">
-        <v>154</v>
-      </c>
       <c r="H11" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2478,25 +2487,25 @@
         <v>9</v>
       </c>
       <c r="B12" s="57" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C12" s="57" t="s">
         <v>30</v>
       </c>
       <c r="D12" s="59" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="E12" s="57" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F12" s="59" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G12" s="57" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="H12" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2505,25 +2514,25 @@
         <v>10</v>
       </c>
       <c r="B13" s="57" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C13" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D13" s="59" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="E13" s="57" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="F13" s="59" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="G13" s="57" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="H13" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2532,25 +2541,25 @@
         <v>11</v>
       </c>
       <c r="B14" s="57" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="C14" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="59" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="E14" s="57" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="F14" s="59" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="G14" s="57" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="H14" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2577,7 +2586,7 @@
         <v>40</v>
       </c>
       <c r="H15" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2586,25 +2595,25 @@
         <v>13</v>
       </c>
       <c r="B16" s="57" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C16" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D16" s="59" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E16" s="57" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F16" s="59" t="s">
-        <v>170</v>
-      </c>
-      <c r="G16" s="57" t="s">
-        <v>171</v>
+        <v>167</v>
+      </c>
+      <c r="G16" s="60" t="s">
+        <v>246</v>
       </c>
       <c r="H16" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2613,7 +2622,7 @@
         <v>14</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C17" s="57" t="s">
         <v>29</v>
@@ -2622,16 +2631,16 @@
         <v>163788493</v>
       </c>
       <c r="E17" s="57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F17" s="59">
         <v>3113436761</v>
       </c>
-      <c r="G17" s="57" t="s">
-        <v>120</v>
+      <c r="G17" s="60" t="s">
+        <v>250</v>
       </c>
       <c r="H17" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2640,25 +2649,25 @@
         <v>15</v>
       </c>
       <c r="B18" s="57" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C18" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D18" s="59" t="s">
+        <v>120</v>
+      </c>
+      <c r="E18" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="F18" s="59" t="s">
+        <v>121</v>
+      </c>
+      <c r="G18" s="57" t="s">
         <v>122</v>
       </c>
-      <c r="E18" s="57" t="s">
-        <v>119</v>
-      </c>
-      <c r="F18" s="59" t="s">
-        <v>123</v>
-      </c>
-      <c r="G18" s="57" t="s">
-        <v>124</v>
-      </c>
       <c r="H18" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2685,7 +2694,7 @@
         <v>45</v>
       </c>
       <c r="H19" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2694,25 +2703,25 @@
         <v>17</v>
       </c>
       <c r="B20" s="57" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C20" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D20" s="59" t="s">
+        <v>95</v>
+      </c>
+      <c r="E20" s="57" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="E20" s="57" t="s">
-        <v>92</v>
-      </c>
-      <c r="F20" s="59" t="s">
+      <c r="G20" s="57" t="s">
         <v>97</v>
       </c>
-      <c r="G20" s="57" t="s">
-        <v>98</v>
-      </c>
       <c r="H20" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2721,25 +2730,25 @@
         <v>18</v>
       </c>
       <c r="B21" s="57" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C21" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D21" s="59" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="E21" s="57" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F21" s="59" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G21" s="57" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="H21" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2748,25 +2757,25 @@
         <v>19</v>
       </c>
       <c r="B22" s="57" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C22" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D22" s="59" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E22" s="57" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="F22" s="59" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="G22" s="57" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="H22" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2775,25 +2784,25 @@
         <v>20</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C23" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D23" s="59" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E23" s="57" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="F23" s="59" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="G23" s="57" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="H23" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2802,25 +2811,25 @@
         <v>21</v>
       </c>
       <c r="B24" s="57" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C24" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D24" s="59" t="s">
+        <v>78</v>
+      </c>
+      <c r="E24" s="57" t="s">
+        <v>74</v>
+      </c>
+      <c r="F24" s="59" t="s">
         <v>79</v>
       </c>
-      <c r="E24" s="57" t="s">
-        <v>75</v>
-      </c>
-      <c r="F24" s="59" t="s">
+      <c r="G24" s="57" t="s">
         <v>80</v>
       </c>
-      <c r="G24" s="57" t="s">
-        <v>81</v>
-      </c>
       <c r="H24" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2829,25 +2838,25 @@
         <v>22</v>
       </c>
       <c r="B25" s="57" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C25" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D25" s="59" t="s">
+        <v>113</v>
+      </c>
+      <c r="E25" s="57" t="s">
         <v>114</v>
       </c>
-      <c r="E25" s="57" t="s">
+      <c r="F25" s="59" t="s">
         <v>115</v>
       </c>
-      <c r="F25" s="59" t="s">
+      <c r="G25" s="57" t="s">
         <v>116</v>
       </c>
-      <c r="G25" s="57" t="s">
-        <v>117</v>
-      </c>
       <c r="H25" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2856,25 +2865,25 @@
         <v>23</v>
       </c>
       <c r="B26" s="57" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C26" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D26" s="59" t="s">
+        <v>73</v>
+      </c>
+      <c r="E26" s="57" t="s">
         <v>74</v>
       </c>
-      <c r="E26" s="57" t="s">
+      <c r="F26" s="59" t="s">
         <v>75</v>
       </c>
-      <c r="F26" s="59" t="s">
+      <c r="G26" s="57" t="s">
         <v>76</v>
       </c>
-      <c r="G26" s="57" t="s">
-        <v>77</v>
-      </c>
       <c r="H26" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2883,25 +2892,25 @@
         <v>24</v>
       </c>
       <c r="B27" s="57" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="C27" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D27" s="59" t="s">
+        <v>234</v>
+      </c>
+      <c r="E27" s="57" t="s">
+        <v>235</v>
+      </c>
+      <c r="F27" s="59" t="s">
+        <v>236</v>
+      </c>
+      <c r="G27" s="57" t="s">
+        <v>237</v>
+      </c>
+      <c r="H27" s="57" t="s">
         <v>238</v>
-      </c>
-      <c r="E27" s="57" t="s">
-        <v>239</v>
-      </c>
-      <c r="F27" s="59" t="s">
-        <v>240</v>
-      </c>
-      <c r="G27" s="57" t="s">
-        <v>241</v>
-      </c>
-      <c r="H27" s="57" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2910,25 +2919,25 @@
         <v>25</v>
       </c>
       <c r="B28" s="57" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C28" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D28" s="59" t="s">
+        <v>68</v>
+      </c>
+      <c r="E28" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="E28" s="57" t="s">
+      <c r="F28" s="59" t="s">
         <v>70</v>
       </c>
-      <c r="F28" s="59" t="s">
+      <c r="G28" s="57" t="s">
         <v>71</v>
       </c>
-      <c r="G28" s="57" t="s">
-        <v>72</v>
-      </c>
       <c r="H28" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2937,25 +2946,25 @@
         <v>26</v>
       </c>
       <c r="B29" s="57" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C29" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D29" s="59" t="s">
+        <v>131</v>
+      </c>
+      <c r="E29" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="F29" s="59" t="s">
+        <v>132</v>
+      </c>
+      <c r="G29" s="57" t="s">
         <v>133</v>
       </c>
-      <c r="E29" s="57" t="s">
-        <v>119</v>
-      </c>
-      <c r="F29" s="59" t="s">
-        <v>134</v>
-      </c>
-      <c r="G29" s="57" t="s">
-        <v>135</v>
-      </c>
       <c r="H29" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2964,25 +2973,25 @@
         <v>27</v>
       </c>
       <c r="B30" s="57" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C30" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D30" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="E30" s="57" t="s">
         <v>100</v>
       </c>
-      <c r="E30" s="57" t="s">
+      <c r="F30" s="59" t="s">
         <v>101</v>
       </c>
-      <c r="F30" s="59" t="s">
+      <c r="G30" s="57" t="s">
         <v>102</v>
       </c>
-      <c r="G30" s="57" t="s">
-        <v>103</v>
-      </c>
       <c r="H30" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -2991,25 +3000,25 @@
         <v>28</v>
       </c>
       <c r="B31" s="57" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C31" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D31" s="59" t="s">
+        <v>139</v>
+      </c>
+      <c r="E31" s="57" t="s">
+        <v>140</v>
+      </c>
+      <c r="F31" s="59" t="s">
         <v>141</v>
       </c>
-      <c r="E31" s="57" t="s">
-        <v>142</v>
-      </c>
-      <c r="F31" s="59" t="s">
-        <v>143</v>
-      </c>
-      <c r="G31" s="57" t="s">
-        <v>144</v>
+      <c r="G31" s="60" t="s">
+        <v>247</v>
       </c>
       <c r="H31" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3018,25 +3027,25 @@
         <v>29</v>
       </c>
       <c r="B32" s="57" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C32" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D32" s="59" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E32" s="57" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F32" s="59" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="G32" s="57" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="H32" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3045,25 +3054,25 @@
         <v>30</v>
       </c>
       <c r="B33" s="57" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C33" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D33" s="59" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E33" s="57" t="s">
         <v>34</v>
       </c>
       <c r="F33" s="59" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="G33" s="57" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="H33" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3072,25 +3081,25 @@
         <v>31</v>
       </c>
       <c r="B34" s="57" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C34" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D34" s="59" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E34" s="57" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F34" s="59" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="G34" s="57" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="H34" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3099,25 +3108,25 @@
         <v>32</v>
       </c>
       <c r="B35" s="57" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C35" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D35" s="59" t="s">
+        <v>127</v>
+      </c>
+      <c r="E35" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="F35" s="58" t="s">
+        <v>128</v>
+      </c>
+      <c r="G35" s="57" t="s">
         <v>129</v>
       </c>
-      <c r="E35" s="57" t="s">
-        <v>119</v>
-      </c>
-      <c r="F35" s="58" t="s">
-        <v>130</v>
-      </c>
-      <c r="G35" s="57" t="s">
-        <v>131</v>
-      </c>
       <c r="H35" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3126,25 +3135,25 @@
         <v>33</v>
       </c>
       <c r="B36" s="57" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C36" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D36" s="59" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E36" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="F36" s="59" t="s">
         <v>178</v>
       </c>
-      <c r="F36" s="59" t="s">
-        <v>182</v>
-      </c>
       <c r="G36" s="57" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="H36" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3153,25 +3162,25 @@
         <v>34</v>
       </c>
       <c r="B37" s="57" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C37" s="57" t="s">
         <v>30</v>
       </c>
       <c r="D37" s="59" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E37" s="57" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F37" s="59" t="s">
-        <v>179</v>
-      </c>
-      <c r="G37" s="57" t="s">
+        <v>175</v>
+      </c>
+      <c r="G37" s="60" t="s">
         <v>244</v>
       </c>
       <c r="H37" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3180,25 +3189,25 @@
         <v>35</v>
       </c>
       <c r="B38" s="57" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C38" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D38" s="59" t="s">
+        <v>104</v>
+      </c>
+      <c r="E38" s="57" t="s">
         <v>105</v>
       </c>
-      <c r="E38" s="57" t="s">
+      <c r="F38" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="F38" s="59" t="s">
+      <c r="G38" s="57" t="s">
         <v>107</v>
       </c>
-      <c r="G38" s="57" t="s">
-        <v>108</v>
-      </c>
       <c r="H38" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3207,25 +3216,25 @@
         <v>36</v>
       </c>
       <c r="B39" s="57" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C39" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D39" s="59" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="E39" s="57" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F39" s="59" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="G39" s="57" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="H39" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3234,25 +3243,25 @@
         <v>37</v>
       </c>
       <c r="B40" s="57" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C40" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D40" s="59" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="E40" s="57" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F40" s="59" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="G40" s="57" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="H40" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3261,25 +3270,25 @@
         <v>38</v>
       </c>
       <c r="B41" s="57" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C41" s="57" t="s">
         <v>30</v>
       </c>
       <c r="D41" s="59" t="s">
+        <v>109</v>
+      </c>
+      <c r="E41" s="57" t="s">
+        <v>105</v>
+      </c>
+      <c r="F41" s="59" t="s">
         <v>110</v>
       </c>
-      <c r="E41" s="57" t="s">
-        <v>106</v>
-      </c>
-      <c r="F41" s="59" t="s">
+      <c r="G41" s="57" t="s">
         <v>111</v>
       </c>
-      <c r="G41" s="57" t="s">
-        <v>112</v>
-      </c>
       <c r="H41" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3288,25 +3297,25 @@
         <v>39</v>
       </c>
       <c r="B42" s="57" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C42" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D42" s="59" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E42" s="57" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F42" s="59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="G42" s="57" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="H42" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3315,7 +3324,7 @@
         <v>40</v>
       </c>
       <c r="B43" s="57" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C43" s="57" t="s">
         <v>29</v>
@@ -3324,16 +3333,16 @@
         <v>1063359483</v>
       </c>
       <c r="E43" s="57" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F43" s="59">
         <v>3045804294</v>
       </c>
       <c r="G43" s="57" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H43" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3342,25 +3351,25 @@
         <v>41</v>
       </c>
       <c r="B44" s="57" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C44" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D44" s="59" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E44" s="57" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F44" s="59" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="G44" s="57" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="H44" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3369,25 +3378,25 @@
         <v>42</v>
       </c>
       <c r="B45" s="57" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C45" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D45" s="59" t="s">
+        <v>153</v>
+      </c>
+      <c r="E45" s="57" t="s">
+        <v>154</v>
+      </c>
+      <c r="F45" s="59" t="s">
+        <v>155</v>
+      </c>
+      <c r="G45" s="57" t="s">
         <v>156</v>
       </c>
-      <c r="E45" s="57" t="s">
-        <v>157</v>
-      </c>
-      <c r="F45" s="59" t="s">
-        <v>158</v>
-      </c>
-      <c r="G45" s="57" t="s">
-        <v>159</v>
-      </c>
       <c r="H45" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3396,25 +3405,25 @@
         <v>43</v>
       </c>
       <c r="B46" s="57" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C46" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D46" s="59" t="s">
+        <v>54</v>
+      </c>
+      <c r="E46" s="57" t="s">
         <v>55</v>
       </c>
-      <c r="E46" s="57" t="s">
+      <c r="F46" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="F46" s="59" t="s">
-        <v>57</v>
-      </c>
-      <c r="G46" s="61" t="s">
-        <v>243</v>
+      <c r="G46" s="60" t="s">
+        <v>239</v>
       </c>
       <c r="H46" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3423,25 +3432,25 @@
         <v>44</v>
       </c>
       <c r="B47" s="57" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C47" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D47" s="59" t="s">
+        <v>90</v>
+      </c>
+      <c r="E47" s="57" t="s">
         <v>91</v>
       </c>
-      <c r="E47" s="57" t="s">
+      <c r="F47" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="F47" s="59" t="s">
+      <c r="G47" s="57" t="s">
         <v>93</v>
       </c>
-      <c r="G47" s="57" t="s">
-        <v>94</v>
-      </c>
       <c r="H47" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3464,11 +3473,11 @@
       <c r="F48" s="59" t="s">
         <v>47</v>
       </c>
-      <c r="G48" s="57" t="s">
-        <v>49</v>
+      <c r="G48" s="60" t="s">
+        <v>245</v>
       </c>
       <c r="H48" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3495,7 +3504,7 @@
         <v>36</v>
       </c>
       <c r="H49" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3504,25 +3513,25 @@
         <v>47</v>
       </c>
       <c r="B50" s="57" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C50" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D50" s="59" t="s">
+        <v>135</v>
+      </c>
+      <c r="E50" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="F50" s="59" t="s">
+        <v>136</v>
+      </c>
+      <c r="G50" s="57" t="s">
         <v>137</v>
       </c>
-      <c r="E50" s="57" t="s">
-        <v>119</v>
-      </c>
-      <c r="F50" s="59" t="s">
-        <v>138</v>
-      </c>
-      <c r="G50" s="57" t="s">
-        <v>139</v>
-      </c>
       <c r="H50" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3531,25 +3540,25 @@
         <v>48</v>
       </c>
       <c r="B51" s="57" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C51" s="57" t="s">
         <v>29</v>
       </c>
       <c r="D51" s="59" t="s">
+        <v>63</v>
+      </c>
+      <c r="E51" s="57" t="s">
         <v>64</v>
       </c>
-      <c r="E51" s="57" t="s">
+      <c r="F51" s="59" t="s">
         <v>65</v>
       </c>
-      <c r="F51" s="59" t="s">
+      <c r="G51" s="57" t="s">
         <v>66</v>
       </c>
-      <c r="G51" s="57" t="s">
-        <v>67</v>
-      </c>
       <c r="H51" s="57" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3558,25 +3567,25 @@
         <v>49</v>
       </c>
       <c r="B52" s="50" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C52" s="51" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="D52" s="47">
         <v>1063358976</v>
       </c>
       <c r="E52" s="45" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="F52" s="15">
         <v>3001754755</v>
       </c>
-      <c r="G52" s="151" t="s">
-        <v>248</v>
+      <c r="G52" s="61" t="s">
+        <v>243</v>
       </c>
       <c r="H52" s="52" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
@@ -3726,10 +3735,14 @@
     <hyperlink ref="G17" r:id="rId2" xr:uid="{092C4A61-E23C-4BF6-9661-B7CE860226C9}"/>
     <hyperlink ref="G46" r:id="rId3" xr:uid="{042E7418-FA4C-4F84-A42C-9C4C96034294}"/>
     <hyperlink ref="G52" r:id="rId4" xr:uid="{62763121-B2C7-4BA6-9D17-0FBBCE3C3654}"/>
+    <hyperlink ref="G37" r:id="rId5" xr:uid="{3CA2440D-8BCE-4E18-B317-8E843E2D7A3E}"/>
+    <hyperlink ref="G48" r:id="rId6" xr:uid="{A74B16DD-3DD0-45C8-830B-91FFE26BB69A}"/>
+    <hyperlink ref="G16" r:id="rId7" xr:uid="{36822912-61D4-449D-899A-5E87D7F11EBE}"/>
+    <hyperlink ref="G31" r:id="rId8" xr:uid="{0C63496A-BB3B-48F5-B0EF-D695EBC9F202}"/>
   </hyperlinks>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="80" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId5"/>
-  <drawing r:id="rId6"/>
+  <pageSetup scale="80" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId9"/>
+  <drawing r:id="rId10"/>
 </worksheet>
 </file>
 
@@ -3744,7 +3757,10 @@
     <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.33203125" style="2" customWidth="1"/>
-    <col min="8" max="15" width="7.33203125" customWidth="1"/>
+    <col min="8" max="8" width="7.33203125" customWidth="1"/>
+    <col min="9" max="9" width="11.33203125" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" customWidth="1"/>
+    <col min="11" max="15" width="7.33203125" customWidth="1"/>
     <col min="16" max="16" width="7.33203125" style="2" customWidth="1"/>
     <col min="17" max="24" width="7.33203125" customWidth="1"/>
     <col min="25" max="25" width="7.33203125" style="2" customWidth="1"/>
@@ -3753,37 +3769,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="73" t="s">
+      <c r="B1" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="73"/>
-      <c r="R1" s="73"/>
-      <c r="S1" s="73"/>
-      <c r="T1" s="73"/>
-      <c r="U1" s="73"/>
-      <c r="V1" s="73"/>
-      <c r="W1" s="73"/>
-      <c r="X1" s="73"/>
-      <c r="Y1" s="73"/>
-      <c r="Z1" s="73"/>
-      <c r="AA1" s="73"/>
-      <c r="AB1" s="73"/>
-      <c r="AC1" s="73"/>
-      <c r="AD1" s="73"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
+      <c r="M1" s="75"/>
+      <c r="N1" s="75"/>
+      <c r="O1" s="75"/>
+      <c r="P1" s="75"/>
+      <c r="Q1" s="75"/>
+      <c r="R1" s="75"/>
+      <c r="S1" s="75"/>
+      <c r="T1" s="75"/>
+      <c r="U1" s="75"/>
+      <c r="V1" s="75"/>
+      <c r="W1" s="75"/>
+      <c r="X1" s="75"/>
+      <c r="Y1" s="75"/>
+      <c r="Z1" s="75"/>
+      <c r="AA1" s="75"/>
+      <c r="AB1" s="75"/>
+      <c r="AC1" s="75"/>
+      <c r="AD1" s="75"/>
     </row>
     <row r="2" spans="1:30" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="55" t="s">
@@ -3795,120 +3811,120 @@
       <c r="C2" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="89" t="s">
+      <c r="D2" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="91"/>
-      <c r="H2" s="74" t="s">
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="76" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="75"/>
-      <c r="J2" s="75"/>
-      <c r="K2" s="75"/>
-      <c r="L2" s="75"/>
-      <c r="M2" s="75"/>
-      <c r="N2" s="75"/>
-      <c r="O2" s="75"/>
-      <c r="P2" s="76"/>
-      <c r="Q2" s="83" t="s">
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
+      <c r="L2" s="77"/>
+      <c r="M2" s="77"/>
+      <c r="N2" s="77"/>
+      <c r="O2" s="77"/>
+      <c r="P2" s="78"/>
+      <c r="Q2" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="84"/>
-      <c r="S2" s="84"/>
-      <c r="T2" s="84"/>
-      <c r="U2" s="84"/>
-      <c r="V2" s="84"/>
-      <c r="W2" s="84"/>
-      <c r="X2" s="84"/>
-      <c r="Y2" s="85"/>
-      <c r="Z2" s="66" t="s">
+      <c r="R2" s="86"/>
+      <c r="S2" s="86"/>
+      <c r="T2" s="86"/>
+      <c r="U2" s="86"/>
+      <c r="V2" s="86"/>
+      <c r="W2" s="86"/>
+      <c r="X2" s="86"/>
+      <c r="Y2" s="87"/>
+      <c r="Z2" s="68" t="s">
         <v>21</v>
       </c>
-      <c r="AA2" s="67"/>
-      <c r="AB2" s="67"/>
-      <c r="AC2" s="67"/>
-      <c r="AD2" s="68"/>
+      <c r="AA2" s="69"/>
+      <c r="AB2" s="69"/>
+      <c r="AC2" s="69"/>
+      <c r="AD2" s="70"/>
     </row>
     <row r="3" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="56"/>
       <c r="B3" s="54"/>
       <c r="C3" s="56"/>
-      <c r="D3" s="92" t="s">
+      <c r="D3" s="94" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="94"/>
-      <c r="H3" s="77" t="s">
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="78"/>
-      <c r="J3" s="78"/>
-      <c r="K3" s="78"/>
-      <c r="L3" s="78"/>
-      <c r="M3" s="78"/>
-      <c r="N3" s="78"/>
-      <c r="O3" s="78"/>
-      <c r="P3" s="79"/>
-      <c r="Q3" s="86" t="s">
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="81"/>
+      <c r="Q3" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="R3" s="87"/>
-      <c r="S3" s="87"/>
-      <c r="T3" s="87"/>
-      <c r="U3" s="87"/>
-      <c r="V3" s="87"/>
-      <c r="W3" s="87"/>
-      <c r="X3" s="87"/>
-      <c r="Y3" s="88"/>
-      <c r="Z3" s="69" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="70"/>
-      <c r="AB3" s="70"/>
-      <c r="AC3" s="70"/>
-      <c r="AD3" s="71"/>
+      <c r="R3" s="89"/>
+      <c r="S3" s="89"/>
+      <c r="T3" s="89"/>
+      <c r="U3" s="89"/>
+      <c r="V3" s="89"/>
+      <c r="W3" s="89"/>
+      <c r="X3" s="89"/>
+      <c r="Y3" s="90"/>
+      <c r="Z3" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="72"/>
+      <c r="AB3" s="72"/>
+      <c r="AC3" s="72"/>
+      <c r="AD3" s="73"/>
     </row>
     <row r="4" spans="1:30" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="56"/>
       <c r="B4" s="54"/>
       <c r="C4" s="56"/>
-      <c r="D4" s="95" t="s">
+      <c r="D4" s="97" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="81"/>
-      <c r="F4" s="81"/>
+      <c r="E4" s="83"/>
+      <c r="F4" s="83"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="80" t="s">
+      <c r="H4" s="82" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="81"/>
-      <c r="J4" s="81"/>
-      <c r="K4" s="81"/>
-      <c r="L4" s="81"/>
-      <c r="M4" s="81"/>
-      <c r="N4" s="81"/>
-      <c r="O4" s="82"/>
+      <c r="I4" s="83"/>
+      <c r="J4" s="83"/>
+      <c r="K4" s="83"/>
+      <c r="L4" s="83"/>
+      <c r="M4" s="83"/>
+      <c r="N4" s="83"/>
+      <c r="O4" s="84"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="80" t="s">
+      <c r="Q4" s="82" t="s">
         <v>24</v>
       </c>
-      <c r="R4" s="81"/>
-      <c r="S4" s="81"/>
-      <c r="T4" s="81"/>
-      <c r="U4" s="81"/>
-      <c r="V4" s="81"/>
-      <c r="W4" s="81"/>
-      <c r="X4" s="82"/>
+      <c r="R4" s="83"/>
+      <c r="S4" s="83"/>
+      <c r="T4" s="83"/>
+      <c r="U4" s="83"/>
+      <c r="V4" s="83"/>
+      <c r="W4" s="83"/>
+      <c r="X4" s="84"/>
       <c r="Y4" s="13"/>
-      <c r="Z4" s="72" t="s">
+      <c r="Z4" s="74" t="s">
         <v>24</v>
       </c>
-      <c r="AA4" s="72"/>
-      <c r="AB4" s="72"/>
-      <c r="AC4" s="72"/>
+      <c r="AA4" s="74"/>
+      <c r="AB4" s="74"/>
+      <c r="AC4" s="74"/>
       <c r="AD4" s="3"/>
     </row>
     <row r="5" spans="1:30" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -3928,8 +3944,12 @@
         <v>19</v>
       </c>
       <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="29"/>
+      <c r="I5" s="29" t="s">
+        <v>248</v>
+      </c>
+      <c r="J5" s="29" t="s">
+        <v>249</v>
+      </c>
       <c r="K5" s="29"/>
       <c r="L5" s="29"/>
       <c r="M5" s="29"/>
@@ -4012,7 +4032,7 @@
       <c r="A7" s="21">
         <v>2</v>
       </c>
-      <c r="B7" s="60" t="str">
+      <c r="B7" s="19" t="str">
         <f>+Inscritos!B5</f>
         <v>ANALÍA APARICIO HOYOS</v>
       </c>
@@ -4065,7 +4085,7 @@
       <c r="A8" s="21">
         <v>3</v>
       </c>
-      <c r="B8" s="60" t="str">
+      <c r="B8" s="19" t="str">
         <f>+Inscritos!B6</f>
         <v xml:space="preserve">ANDREA CAROLINA ACUÑA CORONADO </v>
       </c>
@@ -4118,7 +4138,7 @@
       <c r="A9" s="21">
         <v>4</v>
       </c>
-      <c r="B9" s="60" t="str">
+      <c r="B9" s="19" t="str">
         <f>+Inscritos!B7</f>
         <v xml:space="preserve">ANDREA CAROLINA TRUJILLO HERRERA </v>
       </c>
@@ -4133,7 +4153,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I9" s="39"/>
       <c r="J9" s="39"/>
@@ -4144,7 +4164,7 @@
       <c r="O9" s="39"/>
       <c r="P9" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Q9" s="39"/>
       <c r="R9" s="39"/>
@@ -4171,7 +4191,7 @@
       <c r="A10" s="21">
         <v>5</v>
       </c>
-      <c r="B10" s="60" t="str">
+      <c r="B10" s="19" t="str">
         <f>+Inscritos!B8</f>
         <v xml:space="preserve">ANDRÉS DAVID OSUNA ALVAREZ </v>
       </c>
@@ -4224,7 +4244,7 @@
       <c r="A11" s="21">
         <v>6</v>
       </c>
-      <c r="B11" s="60" t="str">
+      <c r="B11" s="19" t="str">
         <f>+Inscritos!B9</f>
         <v xml:space="preserve">ANDRES EDUARDO CISNEROS MARTINEZ </v>
       </c>
@@ -4277,7 +4297,7 @@
       <c r="A12" s="21">
         <v>7</v>
       </c>
-      <c r="B12" s="60" t="str">
+      <c r="B12" s="19" t="str">
         <f>+Inscritos!B10</f>
         <v>ANGEL GABRIEL ARROYO ARRIETA</v>
       </c>
@@ -4330,7 +4350,7 @@
       <c r="A13" s="21">
         <v>8</v>
       </c>
-      <c r="B13" s="19" t="str">
+      <c r="B13" s="62" t="str">
         <f>+Inscritos!B11</f>
         <v xml:space="preserve">ANGELINA MARIA OYÓLA HERRERA </v>
       </c>
@@ -4383,7 +4403,7 @@
       <c r="A14" s="21">
         <v>9</v>
       </c>
-      <c r="B14" s="19" t="str">
+      <c r="B14" s="63" t="str">
         <f>+Inscritos!B12</f>
         <v xml:space="preserve">CELENY LUZ ACOSTA MONTERROSA </v>
       </c>
@@ -4436,7 +4456,7 @@
       <c r="A15" s="21">
         <v>10</v>
       </c>
-      <c r="B15" s="19" t="str">
+      <c r="B15" s="63" t="str">
         <f>+Inscritos!B13</f>
         <v xml:space="preserve">DARLENE TRUJILLO </v>
       </c>
@@ -4489,7 +4509,7 @@
       <c r="A16" s="21">
         <v>11</v>
       </c>
-      <c r="B16" s="19" t="str">
+      <c r="B16" s="63" t="str">
         <f>+Inscritos!B14</f>
         <v xml:space="preserve">DAYANA MARÍA ARGUMEDO ARRIETA </v>
       </c>
@@ -4542,7 +4562,7 @@
       <c r="A17" s="21">
         <v>12</v>
       </c>
-      <c r="B17" s="19" t="str">
+      <c r="B17" s="63" t="str">
         <f>+Inscritos!B15</f>
         <v>DEIVER DAVID FLORES LOPEZ</v>
       </c>
@@ -4557,7 +4577,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" s="39"/>
       <c r="J17" s="39"/>
@@ -4568,7 +4588,7 @@
       <c r="O17" s="40"/>
       <c r="P17" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q17" s="39"/>
       <c r="R17" s="39"/>
@@ -4595,7 +4615,7 @@
       <c r="A18" s="21">
         <v>13</v>
       </c>
-      <c r="B18" s="19" t="str">
+      <c r="B18" s="63" t="str">
         <f>+Inscritos!B16</f>
         <v xml:space="preserve">DUBERNEY JARAMILLO CAPACHERO </v>
       </c>
@@ -4663,7 +4683,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I19" s="39"/>
       <c r="J19" s="39"/>
@@ -4674,7 +4694,7 @@
       <c r="O19" s="40"/>
       <c r="P19" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q19" s="39"/>
       <c r="R19" s="39"/>
@@ -4822,7 +4842,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I22" s="39"/>
       <c r="J22" s="39"/>
@@ -4833,7 +4853,7 @@
       <c r="O22" s="40"/>
       <c r="P22" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q22" s="39"/>
       <c r="R22" s="39"/>
@@ -4928,7 +4948,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I24" s="39"/>
       <c r="J24" s="39"/>
@@ -4939,7 +4959,7 @@
       <c r="O24" s="40"/>
       <c r="P24" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.375</v>
       </c>
       <c r="Q24" s="39"/>
       <c r="R24" s="39"/>
@@ -5034,7 +5054,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I26" s="39"/>
       <c r="J26" s="39"/>
@@ -5045,7 +5065,7 @@
       <c r="O26" s="40"/>
       <c r="P26" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.375</v>
       </c>
       <c r="Q26" s="39"/>
       <c r="R26" s="39"/>
@@ -5193,7 +5213,7 @@
         <v>0</v>
       </c>
       <c r="H29" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" s="39"/>
       <c r="J29" s="39"/>
@@ -5204,7 +5224,7 @@
       <c r="O29" s="40"/>
       <c r="P29" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q29" s="39"/>
       <c r="R29" s="39"/>
@@ -5352,7 +5372,7 @@
         <v>0</v>
       </c>
       <c r="H32" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" s="39"/>
       <c r="J32" s="39"/>
@@ -5363,7 +5383,7 @@
       <c r="O32" s="40"/>
       <c r="P32" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q32" s="39"/>
       <c r="R32" s="39"/>
@@ -5564,7 +5584,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36" s="39"/>
       <c r="J36" s="39"/>
@@ -5575,7 +5595,7 @@
       <c r="O36" s="39"/>
       <c r="P36" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q36" s="39"/>
       <c r="R36" s="39"/>
@@ -5617,7 +5637,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" s="39"/>
       <c r="J37" s="39"/>
@@ -5628,7 +5648,7 @@
       <c r="O37" s="40"/>
       <c r="P37" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q37" s="39"/>
       <c r="R37" s="39"/>
@@ -5723,7 +5743,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I39" s="39"/>
       <c r="J39" s="39"/>
@@ -5734,7 +5754,7 @@
       <c r="O39" s="40"/>
       <c r="P39" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Q39" s="39"/>
       <c r="R39" s="39"/>
@@ -5776,7 +5796,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I40" s="39"/>
       <c r="J40" s="39"/>
@@ -5787,7 +5807,7 @@
       <c r="O40" s="39"/>
       <c r="P40" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.375</v>
       </c>
       <c r="Q40" s="39"/>
       <c r="R40" s="39"/>
@@ -6041,7 +6061,7 @@
         <v>0</v>
       </c>
       <c r="H45" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I45" s="39"/>
       <c r="J45" s="39"/>
@@ -6052,7 +6072,7 @@
       <c r="O45" s="40"/>
       <c r="P45" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q45" s="39"/>
       <c r="R45" s="39"/>
@@ -6147,7 +6167,7 @@
         <v>0</v>
       </c>
       <c r="H47" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I47" s="39"/>
       <c r="J47" s="39"/>
@@ -6158,7 +6178,7 @@
       <c r="O47" s="40"/>
       <c r="P47" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q47" s="39"/>
       <c r="R47" s="39"/>
@@ -6412,7 +6432,7 @@
         <v>0</v>
       </c>
       <c r="H52" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" s="39"/>
       <c r="J52" s="39"/>
@@ -6423,7 +6443,7 @@
       <c r="O52" s="40"/>
       <c r="P52" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q52" s="39"/>
       <c r="R52" s="39"/>
@@ -6465,7 +6485,7 @@
         <v>0</v>
       </c>
       <c r="H53" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I53" s="39"/>
       <c r="J53" s="39"/>
@@ -6476,7 +6496,7 @@
       <c r="O53" s="40"/>
       <c r="P53" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q53" s="39"/>
       <c r="R53" s="39"/>
@@ -6518,7 +6538,9 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="H54" s="39"/>
+      <c r="H54" s="39">
+        <v>2</v>
+      </c>
       <c r="I54" s="39"/>
       <c r="J54" s="39"/>
       <c r="K54" s="39"/>
@@ -6528,7 +6550,7 @@
       <c r="O54" s="40"/>
       <c r="P54" s="38">
         <f t="shared" ref="P54" si="4">+SUM(H54:O54)/8</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="Q54" s="39"/>
       <c r="R54" s="39"/>
@@ -6555,14 +6577,8 @@
       <c r="A55" s="21">
         <v>50</v>
       </c>
-      <c r="B55" s="19">
-        <f>+Inscritos!B53</f>
-        <v>0</v>
-      </c>
-      <c r="C55" s="22">
-        <f>+Inscritos!D53</f>
-        <v>0</v>
-      </c>
+      <c r="B55" s="19"/>
+      <c r="C55" s="22"/>
       <c r="D55" s="14"/>
       <c r="E55" s="14"/>
       <c r="F55" s="14"/>
@@ -6607,14 +6623,8 @@
       <c r="A56" s="21">
         <v>51</v>
       </c>
-      <c r="B56" s="19">
-        <f>+Inscritos!B54</f>
-        <v>0</v>
-      </c>
-      <c r="C56" s="22">
-        <f>+Inscritos!D54</f>
-        <v>0</v>
-      </c>
+      <c r="B56" s="19"/>
+      <c r="C56" s="22"/>
       <c r="D56" s="14"/>
       <c r="E56" s="14"/>
       <c r="F56" s="14"/>
@@ -6659,14 +6669,8 @@
       <c r="A57" s="21">
         <v>52</v>
       </c>
-      <c r="B57" s="19">
-        <f>+Inscritos!B55</f>
-        <v>0</v>
-      </c>
-      <c r="C57" s="22">
-        <f>+Inscritos!D55</f>
-        <v>0</v>
-      </c>
+      <c r="B57" s="19"/>
+      <c r="C57" s="22"/>
       <c r="D57" s="14"/>
       <c r="E57" s="14"/>
       <c r="F57" s="14"/>
@@ -7023,10 +7027,7 @@
       <c r="A64" s="21">
         <v>59</v>
       </c>
-      <c r="B64" s="19">
-        <f>+Inscritos!B62</f>
-        <v>0</v>
-      </c>
+      <c r="B64" s="19"/>
       <c r="C64" s="22">
         <f>+Inscritos!D62</f>
         <v>0</v>
@@ -7117,123 +7118,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="128" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="126"/>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
-      <c r="F1" s="126"/>
-      <c r="G1" s="126"/>
-      <c r="H1" s="126"/>
-      <c r="I1" s="126"/>
-      <c r="J1" s="126"/>
-      <c r="K1" s="126"/>
-      <c r="L1" s="126"/>
-      <c r="M1" s="126"/>
-      <c r="N1" s="126"/>
-      <c r="O1" s="126"/>
-      <c r="P1" s="126"/>
-      <c r="Q1" s="126"/>
-      <c r="R1" s="126"/>
-      <c r="S1" s="126"/>
-      <c r="T1" s="126"/>
+      <c r="C1" s="128"/>
+      <c r="D1" s="128"/>
+      <c r="E1" s="128"/>
+      <c r="F1" s="128"/>
+      <c r="G1" s="128"/>
+      <c r="H1" s="128"/>
+      <c r="I1" s="128"/>
+      <c r="J1" s="128"/>
+      <c r="K1" s="128"/>
+      <c r="L1" s="128"/>
+      <c r="M1" s="128"/>
+      <c r="N1" s="128"/>
+      <c r="O1" s="128"/>
+      <c r="P1" s="128"/>
+      <c r="Q1" s="128"/>
+      <c r="R1" s="128"/>
+      <c r="S1" s="128"/>
+      <c r="T1" s="128"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="110" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="122" t="s">
+      <c r="B2" s="124" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="124" t="s">
+      <c r="C2" s="126" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="96" t="str">
+      <c r="D2" s="98" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="97"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="96" t="str">
+      <c r="E2" s="99"/>
+      <c r="F2" s="100"/>
+      <c r="G2" s="98" t="str">
         <f>Asistencia!H2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="97"/>
-      <c r="I2" s="97"/>
-      <c r="J2" s="97"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="96" t="s">
+      <c r="H2" s="99"/>
+      <c r="I2" s="99"/>
+      <c r="J2" s="99"/>
+      <c r="K2" s="100"/>
+      <c r="L2" s="98" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="97"/>
-      <c r="N2" s="97"/>
-      <c r="O2" s="97"/>
-      <c r="P2" s="98"/>
-      <c r="Q2" s="96" t="str">
+      <c r="M2" s="99"/>
+      <c r="N2" s="99"/>
+      <c r="O2" s="99"/>
+      <c r="P2" s="100"/>
+      <c r="Q2" s="98" t="str">
         <f>Asistencia!Z2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="97"/>
-      <c r="S2" s="97"/>
-      <c r="T2" s="98"/>
+      <c r="R2" s="99"/>
+      <c r="S2" s="99"/>
+      <c r="T2" s="100"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="109"/>
-      <c r="B3" s="123"/>
-      <c r="C3" s="125"/>
-      <c r="D3" s="116" t="s">
+      <c r="A3" s="111"/>
+      <c r="B3" s="125"/>
+      <c r="C3" s="127"/>
+      <c r="D3" s="118" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="117"/>
-      <c r="F3" s="118"/>
-      <c r="G3" s="110" t="s">
+      <c r="E3" s="119"/>
+      <c r="F3" s="120"/>
+      <c r="G3" s="112" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="112"/>
-      <c r="L3" s="145" t="s">
+      <c r="H3" s="113"/>
+      <c r="I3" s="113"/>
+      <c r="J3" s="113"/>
+      <c r="K3" s="114"/>
+      <c r="L3" s="147" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="146"/>
-      <c r="N3" s="146"/>
-      <c r="O3" s="146"/>
-      <c r="P3" s="147"/>
-      <c r="Q3" s="99" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="100"/>
-      <c r="S3" s="100"/>
-      <c r="T3" s="101"/>
+      <c r="M3" s="148"/>
+      <c r="N3" s="148"/>
+      <c r="O3" s="148"/>
+      <c r="P3" s="149"/>
+      <c r="Q3" s="101" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="102"/>
+      <c r="S3" s="102"/>
+      <c r="T3" s="103"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="109"/>
-      <c r="B4" s="123"/>
-      <c r="C4" s="125"/>
-      <c r="D4" s="119"/>
-      <c r="E4" s="120"/>
-      <c r="F4" s="121"/>
-      <c r="G4" s="113"/>
-      <c r="H4" s="114"/>
-      <c r="I4" s="114"/>
-      <c r="J4" s="114"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="148"/>
-      <c r="M4" s="149"/>
-      <c r="N4" s="149"/>
-      <c r="O4" s="149"/>
-      <c r="P4" s="150"/>
-      <c r="Q4" s="102"/>
-      <c r="R4" s="103"/>
-      <c r="S4" s="103"/>
-      <c r="T4" s="104"/>
+      <c r="A4" s="111"/>
+      <c r="B4" s="125"/>
+      <c r="C4" s="127"/>
+      <c r="D4" s="121"/>
+      <c r="E4" s="122"/>
+      <c r="F4" s="123"/>
+      <c r="G4" s="115"/>
+      <c r="H4" s="116"/>
+      <c r="I4" s="116"/>
+      <c r="J4" s="116"/>
+      <c r="K4" s="117"/>
+      <c r="L4" s="150"/>
+      <c r="M4" s="151"/>
+      <c r="N4" s="151"/>
+      <c r="O4" s="151"/>
+      <c r="P4" s="152"/>
+      <c r="Q4" s="104"/>
+      <c r="R4" s="105"/>
+      <c r="S4" s="105"/>
+      <c r="T4" s="106"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="109"/>
-      <c r="B5" s="123"/>
-      <c r="C5" s="125"/>
+      <c r="A5" s="111"/>
+      <c r="B5" s="125"/>
+      <c r="C5" s="127"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -9765,180 +9766,180 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D65" s="130" t="s">
+      <c r="D65" s="132" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="133" t="s">
+      <c r="E65" s="135" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="127" t="s">
+      <c r="G65" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="139" t="s">
+      <c r="H65" s="141" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="139" t="s">
+      <c r="I65" s="141" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="127" t="s">
+      <c r="J65" s="129" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="105" t="s">
+      <c r="L65" s="107" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="136" t="s">
+      <c r="M65" s="138" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="136" t="s">
+      <c r="N65" s="138" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="105" t="s">
+      <c r="O65" s="107" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="142" t="s">
+      <c r="Q65" s="144" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="142" t="s">
+      <c r="R65" s="144" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="142" t="s">
+      <c r="S65" s="144" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D66" s="131"/>
-      <c r="E66" s="134"/>
-      <c r="G66" s="128"/>
-      <c r="H66" s="140"/>
-      <c r="I66" s="140"/>
-      <c r="J66" s="128"/>
-      <c r="L66" s="106"/>
-      <c r="M66" s="137"/>
-      <c r="N66" s="137"/>
-      <c r="O66" s="106"/>
-      <c r="Q66" s="143"/>
-      <c r="R66" s="143"/>
-      <c r="S66" s="143"/>
+      <c r="D66" s="133"/>
+      <c r="E66" s="136"/>
+      <c r="G66" s="130"/>
+      <c r="H66" s="142"/>
+      <c r="I66" s="142"/>
+      <c r="J66" s="130"/>
+      <c r="L66" s="108"/>
+      <c r="M66" s="139"/>
+      <c r="N66" s="139"/>
+      <c r="O66" s="108"/>
+      <c r="Q66" s="145"/>
+      <c r="R66" s="145"/>
+      <c r="S66" s="145"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D67" s="131"/>
-      <c r="E67" s="134"/>
-      <c r="G67" s="128"/>
-      <c r="H67" s="140"/>
-      <c r="I67" s="140"/>
-      <c r="J67" s="128"/>
-      <c r="L67" s="106"/>
-      <c r="M67" s="137"/>
-      <c r="N67" s="137"/>
-      <c r="O67" s="106"/>
-      <c r="Q67" s="143"/>
-      <c r="R67" s="143"/>
-      <c r="S67" s="143"/>
+      <c r="D67" s="133"/>
+      <c r="E67" s="136"/>
+      <c r="G67" s="130"/>
+      <c r="H67" s="142"/>
+      <c r="I67" s="142"/>
+      <c r="J67" s="130"/>
+      <c r="L67" s="108"/>
+      <c r="M67" s="139"/>
+      <c r="N67" s="139"/>
+      <c r="O67" s="108"/>
+      <c r="Q67" s="145"/>
+      <c r="R67" s="145"/>
+      <c r="S67" s="145"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D68" s="131"/>
-      <c r="E68" s="134"/>
-      <c r="G68" s="128"/>
-      <c r="H68" s="140"/>
-      <c r="I68" s="140"/>
-      <c r="J68" s="128"/>
-      <c r="L68" s="106"/>
-      <c r="M68" s="137"/>
-      <c r="N68" s="137"/>
-      <c r="O68" s="106"/>
-      <c r="Q68" s="143"/>
-      <c r="R68" s="143"/>
-      <c r="S68" s="143"/>
+      <c r="D68" s="133"/>
+      <c r="E68" s="136"/>
+      <c r="G68" s="130"/>
+      <c r="H68" s="142"/>
+      <c r="I68" s="142"/>
+      <c r="J68" s="130"/>
+      <c r="L68" s="108"/>
+      <c r="M68" s="139"/>
+      <c r="N68" s="139"/>
+      <c r="O68" s="108"/>
+      <c r="Q68" s="145"/>
+      <c r="R68" s="145"/>
+      <c r="S68" s="145"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D69" s="131"/>
-      <c r="E69" s="134"/>
-      <c r="G69" s="128"/>
-      <c r="H69" s="140"/>
-      <c r="I69" s="140"/>
-      <c r="J69" s="128"/>
-      <c r="L69" s="106"/>
-      <c r="M69" s="137"/>
-      <c r="N69" s="137"/>
-      <c r="O69" s="106"/>
-      <c r="Q69" s="143"/>
-      <c r="R69" s="143"/>
-      <c r="S69" s="143"/>
+      <c r="D69" s="133"/>
+      <c r="E69" s="136"/>
+      <c r="G69" s="130"/>
+      <c r="H69" s="142"/>
+      <c r="I69" s="142"/>
+      <c r="J69" s="130"/>
+      <c r="L69" s="108"/>
+      <c r="M69" s="139"/>
+      <c r="N69" s="139"/>
+      <c r="O69" s="108"/>
+      <c r="Q69" s="145"/>
+      <c r="R69" s="145"/>
+      <c r="S69" s="145"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D70" s="131"/>
-      <c r="E70" s="134"/>
-      <c r="G70" s="128"/>
-      <c r="H70" s="140"/>
-      <c r="I70" s="140"/>
-      <c r="J70" s="128"/>
-      <c r="L70" s="106"/>
-      <c r="M70" s="137"/>
-      <c r="N70" s="137"/>
-      <c r="O70" s="106"/>
-      <c r="Q70" s="143"/>
-      <c r="R70" s="143"/>
-      <c r="S70" s="143"/>
+      <c r="D70" s="133"/>
+      <c r="E70" s="136"/>
+      <c r="G70" s="130"/>
+      <c r="H70" s="142"/>
+      <c r="I70" s="142"/>
+      <c r="J70" s="130"/>
+      <c r="L70" s="108"/>
+      <c r="M70" s="139"/>
+      <c r="N70" s="139"/>
+      <c r="O70" s="108"/>
+      <c r="Q70" s="145"/>
+      <c r="R70" s="145"/>
+      <c r="S70" s="145"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D71" s="131"/>
-      <c r="E71" s="134"/>
-      <c r="G71" s="128"/>
-      <c r="H71" s="140"/>
-      <c r="I71" s="140"/>
-      <c r="J71" s="128"/>
-      <c r="L71" s="106"/>
-      <c r="M71" s="137"/>
-      <c r="N71" s="137"/>
-      <c r="O71" s="106"/>
-      <c r="Q71" s="143"/>
-      <c r="R71" s="143"/>
-      <c r="S71" s="143"/>
+      <c r="D71" s="133"/>
+      <c r="E71" s="136"/>
+      <c r="G71" s="130"/>
+      <c r="H71" s="142"/>
+      <c r="I71" s="142"/>
+      <c r="J71" s="130"/>
+      <c r="L71" s="108"/>
+      <c r="M71" s="139"/>
+      <c r="N71" s="139"/>
+      <c r="O71" s="108"/>
+      <c r="Q71" s="145"/>
+      <c r="R71" s="145"/>
+      <c r="S71" s="145"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D72" s="131"/>
-      <c r="E72" s="134"/>
-      <c r="G72" s="128"/>
-      <c r="H72" s="140"/>
-      <c r="I72" s="140"/>
-      <c r="J72" s="128"/>
-      <c r="L72" s="106"/>
-      <c r="M72" s="137"/>
-      <c r="N72" s="137"/>
-      <c r="O72" s="106"/>
-      <c r="Q72" s="143"/>
-      <c r="R72" s="143"/>
-      <c r="S72" s="143"/>
+      <c r="D72" s="133"/>
+      <c r="E72" s="136"/>
+      <c r="G72" s="130"/>
+      <c r="H72" s="142"/>
+      <c r="I72" s="142"/>
+      <c r="J72" s="130"/>
+      <c r="L72" s="108"/>
+      <c r="M72" s="139"/>
+      <c r="N72" s="139"/>
+      <c r="O72" s="108"/>
+      <c r="Q72" s="145"/>
+      <c r="R72" s="145"/>
+      <c r="S72" s="145"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D73" s="131"/>
-      <c r="E73" s="134"/>
-      <c r="G73" s="128"/>
-      <c r="H73" s="140"/>
-      <c r="I73" s="140"/>
-      <c r="J73" s="128"/>
-      <c r="L73" s="106"/>
-      <c r="M73" s="137"/>
-      <c r="N73" s="137"/>
-      <c r="O73" s="106"/>
-      <c r="Q73" s="143"/>
-      <c r="R73" s="143"/>
-      <c r="S73" s="143"/>
+      <c r="D73" s="133"/>
+      <c r="E73" s="136"/>
+      <c r="G73" s="130"/>
+      <c r="H73" s="142"/>
+      <c r="I73" s="142"/>
+      <c r="J73" s="130"/>
+      <c r="L73" s="108"/>
+      <c r="M73" s="139"/>
+      <c r="N73" s="139"/>
+      <c r="O73" s="108"/>
+      <c r="Q73" s="145"/>
+      <c r="R73" s="145"/>
+      <c r="S73" s="145"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D74" s="132"/>
-      <c r="E74" s="135"/>
-      <c r="G74" s="129"/>
-      <c r="H74" s="141"/>
-      <c r="I74" s="141"/>
-      <c r="J74" s="129"/>
-      <c r="L74" s="107"/>
-      <c r="M74" s="138"/>
-      <c r="N74" s="138"/>
-      <c r="O74" s="107"/>
-      <c r="Q74" s="144"/>
-      <c r="R74" s="144"/>
-      <c r="S74" s="144"/>
+      <c r="D74" s="134"/>
+      <c r="E74" s="137"/>
+      <c r="G74" s="131"/>
+      <c r="H74" s="143"/>
+      <c r="I74" s="143"/>
+      <c r="J74" s="131"/>
+      <c r="L74" s="109"/>
+      <c r="M74" s="140"/>
+      <c r="N74" s="140"/>
+      <c r="O74" s="109"/>
+      <c r="Q74" s="146"/>
+      <c r="R74" s="146"/>
+      <c r="S74" s="146"/>
     </row>
   </sheetData>
   <mergeCells count="25">

</xml_diff>

<commit_message>
agregué los ejercicios de entrenamiento para el tema 9
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACEE989-BB64-45A9-B5A8-6795D148C788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D45624-519C-4EB7-942C-9FC67C968710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="252">
   <si>
     <t>METODOLOGÍA DE ESTUDIO</t>
   </si>
@@ -791,6 +791,9 @@
   </si>
   <si>
     <t>elkinq719@gmail.com</t>
+  </si>
+  <si>
+    <t>1|</t>
   </si>
 </sst>
 </file>
@@ -1259,7 +1262,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="154">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1438,11 +1441,95 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1456,94 +1543,88 @@
     <xf numFmtId="0" fontId="19" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1573,15 +1654,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1636,80 +1708,14 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2217,28 +2223,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="93" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="67"/>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="95"/>
     </row>
     <row r="2" spans="1:8" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -3769,37 +3775,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="75" t="s">
+      <c r="B1" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
-      <c r="R1" s="75"/>
-      <c r="S1" s="75"/>
-      <c r="T1" s="75"/>
-      <c r="U1" s="75"/>
-      <c r="V1" s="75"/>
-      <c r="W1" s="75"/>
-      <c r="X1" s="75"/>
-      <c r="Y1" s="75"/>
-      <c r="Z1" s="75"/>
-      <c r="AA1" s="75"/>
-      <c r="AB1" s="75"/>
-      <c r="AC1" s="75"/>
-      <c r="AD1" s="75"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
     </row>
     <row r="2" spans="1:30" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="55" t="s">
@@ -3811,120 +3817,120 @@
       <c r="C2" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="91" t="s">
+      <c r="D2" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="92"/>
-      <c r="F2" s="92"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="76" t="s">
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="77"/>
-      <c r="J2" s="77"/>
-      <c r="K2" s="77"/>
-      <c r="L2" s="77"/>
-      <c r="M2" s="77"/>
-      <c r="N2" s="77"/>
-      <c r="O2" s="77"/>
-      <c r="P2" s="78"/>
-      <c r="Q2" s="85" t="s">
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+      <c r="P2" s="72"/>
+      <c r="Q2" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="86"/>
-      <c r="S2" s="86"/>
-      <c r="T2" s="86"/>
-      <c r="U2" s="86"/>
-      <c r="V2" s="86"/>
-      <c r="W2" s="86"/>
-      <c r="X2" s="86"/>
-      <c r="Y2" s="87"/>
-      <c r="Z2" s="68" t="s">
+      <c r="R2" s="80"/>
+      <c r="S2" s="80"/>
+      <c r="T2" s="80"/>
+      <c r="U2" s="80"/>
+      <c r="V2" s="80"/>
+      <c r="W2" s="80"/>
+      <c r="X2" s="80"/>
+      <c r="Y2" s="81"/>
+      <c r="Z2" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="AA2" s="69"/>
-      <c r="AB2" s="69"/>
-      <c r="AC2" s="69"/>
-      <c r="AD2" s="70"/>
+      <c r="AA2" s="63"/>
+      <c r="AB2" s="63"/>
+      <c r="AC2" s="63"/>
+      <c r="AD2" s="64"/>
     </row>
     <row r="3" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="56"/>
       <c r="B3" s="54"/>
       <c r="C3" s="56"/>
-      <c r="D3" s="94" t="s">
+      <c r="D3" s="88" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="79" t="s">
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="80"/>
-      <c r="J3" s="80"/>
-      <c r="K3" s="80"/>
-      <c r="L3" s="80"/>
-      <c r="M3" s="80"/>
-      <c r="N3" s="80"/>
-      <c r="O3" s="80"/>
-      <c r="P3" s="81"/>
-      <c r="Q3" s="88" t="s">
+      <c r="I3" s="74"/>
+      <c r="J3" s="74"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="74"/>
+      <c r="M3" s="74"/>
+      <c r="N3" s="74"/>
+      <c r="O3" s="74"/>
+      <c r="P3" s="75"/>
+      <c r="Q3" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="R3" s="89"/>
-      <c r="S3" s="89"/>
-      <c r="T3" s="89"/>
-      <c r="U3" s="89"/>
-      <c r="V3" s="89"/>
-      <c r="W3" s="89"/>
-      <c r="X3" s="89"/>
-      <c r="Y3" s="90"/>
-      <c r="Z3" s="71" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="72"/>
-      <c r="AB3" s="72"/>
-      <c r="AC3" s="72"/>
-      <c r="AD3" s="73"/>
+      <c r="R3" s="83"/>
+      <c r="S3" s="83"/>
+      <c r="T3" s="83"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="83"/>
+      <c r="W3" s="83"/>
+      <c r="X3" s="83"/>
+      <c r="Y3" s="84"/>
+      <c r="Z3" s="65" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="66"/>
+      <c r="AB3" s="66"/>
+      <c r="AC3" s="66"/>
+      <c r="AD3" s="67"/>
     </row>
     <row r="4" spans="1:30" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="56"/>
       <c r="B4" s="54"/>
       <c r="C4" s="56"/>
-      <c r="D4" s="97" t="s">
+      <c r="D4" s="91" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="82" t="s">
+      <c r="H4" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="83"/>
-      <c r="J4" s="83"/>
-      <c r="K4" s="83"/>
-      <c r="L4" s="83"/>
-      <c r="M4" s="83"/>
-      <c r="N4" s="83"/>
-      <c r="O4" s="84"/>
+      <c r="I4" s="77"/>
+      <c r="J4" s="77"/>
+      <c r="K4" s="77"/>
+      <c r="L4" s="77"/>
+      <c r="M4" s="77"/>
+      <c r="N4" s="77"/>
+      <c r="O4" s="78"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="82" t="s">
+      <c r="Q4" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="R4" s="83"/>
-      <c r="S4" s="83"/>
-      <c r="T4" s="83"/>
-      <c r="U4" s="83"/>
-      <c r="V4" s="83"/>
-      <c r="W4" s="83"/>
-      <c r="X4" s="84"/>
+      <c r="R4" s="77"/>
+      <c r="S4" s="77"/>
+      <c r="T4" s="77"/>
+      <c r="U4" s="77"/>
+      <c r="V4" s="77"/>
+      <c r="W4" s="77"/>
+      <c r="X4" s="78"/>
       <c r="Y4" s="13"/>
-      <c r="Z4" s="74" t="s">
+      <c r="Z4" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="AA4" s="74"/>
-      <c r="AB4" s="74"/>
-      <c r="AC4" s="74"/>
+      <c r="AA4" s="68"/>
+      <c r="AB4" s="68"/>
+      <c r="AC4" s="68"/>
       <c r="AD4" s="3"/>
     </row>
     <row r="5" spans="1:30" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -3997,7 +4003,9 @@
       </c>
       <c r="H6" s="14"/>
       <c r="I6" s="39"/>
-      <c r="J6" s="39"/>
+      <c r="J6" s="39" t="s">
+        <v>251</v>
+      </c>
       <c r="K6" s="39"/>
       <c r="L6" s="39"/>
       <c r="M6" s="39"/>
@@ -4050,7 +4058,9 @@
         <v>0</v>
       </c>
       <c r="I7" s="39"/>
-      <c r="J7" s="39"/>
+      <c r="J7" s="39">
+        <v>1</v>
+      </c>
       <c r="K7" s="39"/>
       <c r="L7" s="39"/>
       <c r="M7" s="39"/>
@@ -4058,7 +4068,7 @@
       <c r="O7" s="40"/>
       <c r="P7" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q7" s="39"/>
       <c r="R7" s="39"/>
@@ -4103,7 +4113,9 @@
         <v>0</v>
       </c>
       <c r="I8" s="39"/>
-      <c r="J8" s="39"/>
+      <c r="J8" s="39">
+        <v>0</v>
+      </c>
       <c r="K8" s="39"/>
       <c r="L8" s="39"/>
       <c r="M8" s="39"/>
@@ -4156,7 +4168,9 @@
         <v>2</v>
       </c>
       <c r="I9" s="39"/>
-      <c r="J9" s="39"/>
+      <c r="J9" s="39">
+        <v>1</v>
+      </c>
       <c r="K9" s="39"/>
       <c r="L9" s="39"/>
       <c r="M9" s="39"/>
@@ -4164,7 +4178,7 @@
       <c r="O9" s="39"/>
       <c r="P9" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q9" s="39"/>
       <c r="R9" s="39"/>
@@ -4209,7 +4223,9 @@
         <v>1</v>
       </c>
       <c r="I10" s="39"/>
-      <c r="J10" s="39"/>
+      <c r="J10" s="39">
+        <v>1</v>
+      </c>
       <c r="K10" s="39"/>
       <c r="L10" s="39"/>
       <c r="M10" s="39"/>
@@ -4217,7 +4233,7 @@
       <c r="O10" s="39"/>
       <c r="P10" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q10" s="39"/>
       <c r="R10" s="39"/>
@@ -4262,7 +4278,9 @@
         <v>0</v>
       </c>
       <c r="I11" s="39"/>
-      <c r="J11" s="39"/>
+      <c r="J11" s="39">
+        <v>1</v>
+      </c>
       <c r="K11" s="39"/>
       <c r="L11" s="39"/>
       <c r="M11" s="39"/>
@@ -4270,7 +4288,7 @@
       <c r="O11" s="40"/>
       <c r="P11" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q11" s="39"/>
       <c r="R11" s="39"/>
@@ -4315,7 +4333,9 @@
         <v>1</v>
       </c>
       <c r="I12" s="39"/>
-      <c r="J12" s="39"/>
+      <c r="J12" s="39">
+        <v>1</v>
+      </c>
       <c r="K12" s="39"/>
       <c r="L12" s="39"/>
       <c r="M12" s="39"/>
@@ -4323,7 +4343,7 @@
       <c r="O12" s="40"/>
       <c r="P12" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q12" s="39"/>
       <c r="R12" s="39"/>
@@ -4350,7 +4370,7 @@
       <c r="A13" s="21">
         <v>8</v>
       </c>
-      <c r="B13" s="62" t="str">
+      <c r="B13" s="153" t="str">
         <f>+Inscritos!B11</f>
         <v xml:space="preserve">ANGELINA MARIA OYÓLA HERRERA </v>
       </c>
@@ -4368,7 +4388,9 @@
         <v>0</v>
       </c>
       <c r="I13" s="39"/>
-      <c r="J13" s="39"/>
+      <c r="J13" s="39">
+        <v>0</v>
+      </c>
       <c r="K13" s="39"/>
       <c r="L13" s="39"/>
       <c r="M13" s="39"/>
@@ -4403,7 +4425,7 @@
       <c r="A14" s="21">
         <v>9</v>
       </c>
-      <c r="B14" s="63" t="str">
+      <c r="B14" s="152" t="str">
         <f>+Inscritos!B12</f>
         <v xml:space="preserve">CELENY LUZ ACOSTA MONTERROSA </v>
       </c>
@@ -4421,7 +4443,9 @@
         <v>1</v>
       </c>
       <c r="I14" s="39"/>
-      <c r="J14" s="39"/>
+      <c r="J14" s="39">
+        <v>1</v>
+      </c>
       <c r="K14" s="39"/>
       <c r="L14" s="39"/>
       <c r="M14" s="39"/>
@@ -4429,7 +4453,7 @@
       <c r="O14" s="40"/>
       <c r="P14" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q14" s="39"/>
       <c r="R14" s="39"/>
@@ -4456,7 +4480,7 @@
       <c r="A15" s="21">
         <v>10</v>
       </c>
-      <c r="B15" s="63" t="str">
+      <c r="B15" s="152" t="str">
         <f>+Inscritos!B13</f>
         <v xml:space="preserve">DARLENE TRUJILLO </v>
       </c>
@@ -4474,7 +4498,9 @@
         <v>0</v>
       </c>
       <c r="I15" s="39"/>
-      <c r="J15" s="39"/>
+      <c r="J15" s="39">
+        <v>1</v>
+      </c>
       <c r="K15" s="39"/>
       <c r="L15" s="39"/>
       <c r="M15" s="39"/>
@@ -4482,7 +4508,7 @@
       <c r="O15" s="40"/>
       <c r="P15" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q15" s="39"/>
       <c r="R15" s="39"/>
@@ -4509,7 +4535,7 @@
       <c r="A16" s="21">
         <v>11</v>
       </c>
-      <c r="B16" s="63" t="str">
+      <c r="B16" s="152" t="str">
         <f>+Inscritos!B14</f>
         <v xml:space="preserve">DAYANA MARÍA ARGUMEDO ARRIETA </v>
       </c>
@@ -4527,7 +4553,9 @@
         <v>0</v>
       </c>
       <c r="I16" s="39"/>
-      <c r="J16" s="39"/>
+      <c r="J16" s="39">
+        <v>0</v>
+      </c>
       <c r="K16" s="39"/>
       <c r="L16" s="39"/>
       <c r="M16" s="39"/>
@@ -4562,7 +4590,7 @@
       <c r="A17" s="21">
         <v>12</v>
       </c>
-      <c r="B17" s="63" t="str">
+      <c r="B17" s="152" t="str">
         <f>+Inscritos!B15</f>
         <v>DEIVER DAVID FLORES LOPEZ</v>
       </c>
@@ -4580,7 +4608,9 @@
         <v>1</v>
       </c>
       <c r="I17" s="39"/>
-      <c r="J17" s="39"/>
+      <c r="J17" s="39">
+        <v>1</v>
+      </c>
       <c r="K17" s="39"/>
       <c r="L17" s="39"/>
       <c r="M17" s="39"/>
@@ -4588,7 +4618,7 @@
       <c r="O17" s="40"/>
       <c r="P17" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q17" s="39"/>
       <c r="R17" s="39"/>
@@ -4615,7 +4645,7 @@
       <c r="A18" s="21">
         <v>13</v>
       </c>
-      <c r="B18" s="63" t="str">
+      <c r="B18" s="152" t="str">
         <f>+Inscritos!B16</f>
         <v xml:space="preserve">DUBERNEY JARAMILLO CAPACHERO </v>
       </c>
@@ -4633,7 +4663,9 @@
         <v>0</v>
       </c>
       <c r="I18" s="39"/>
-      <c r="J18" s="39"/>
+      <c r="J18" s="39">
+        <v>1</v>
+      </c>
       <c r="K18" s="39"/>
       <c r="L18" s="39"/>
       <c r="M18" s="39"/>
@@ -4641,7 +4673,7 @@
       <c r="O18" s="40"/>
       <c r="P18" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q18" s="39"/>
       <c r="R18" s="39"/>
@@ -4668,7 +4700,7 @@
       <c r="A19" s="21">
         <v>14</v>
       </c>
-      <c r="B19" s="19" t="str">
+      <c r="B19" s="151" t="str">
         <f>+Inscritos!B17</f>
         <v>ELKIN DARIO QUITERO URANGO</v>
       </c>
@@ -4686,7 +4718,9 @@
         <v>2</v>
       </c>
       <c r="I19" s="39"/>
-      <c r="J19" s="39"/>
+      <c r="J19" s="39">
+        <v>1</v>
+      </c>
       <c r="K19" s="39"/>
       <c r="L19" s="39"/>
       <c r="M19" s="39"/>
@@ -4694,7 +4728,7 @@
       <c r="O19" s="40"/>
       <c r="P19" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q19" s="39"/>
       <c r="R19" s="39"/>
@@ -4721,7 +4755,7 @@
       <c r="A20" s="21">
         <v>15</v>
       </c>
-      <c r="B20" s="19" t="str">
+      <c r="B20" s="151" t="str">
         <f>+Inscritos!B18</f>
         <v xml:space="preserve">EMILYS PATRICIA OVIEDO ROMERO </v>
       </c>
@@ -4739,7 +4773,9 @@
         <v>0</v>
       </c>
       <c r="I20" s="39"/>
-      <c r="J20" s="39"/>
+      <c r="J20" s="39">
+        <v>0</v>
+      </c>
       <c r="K20" s="39"/>
       <c r="L20" s="39"/>
       <c r="M20" s="39"/>
@@ -4774,7 +4810,7 @@
       <c r="A21" s="21">
         <v>16</v>
       </c>
-      <c r="B21" s="19" t="str">
+      <c r="B21" s="151" t="str">
         <f>+Inscritos!B19</f>
         <v>HEELEN DANIELA PÉREZ JIMÉNEZ.</v>
       </c>
@@ -4792,7 +4828,9 @@
         <v>0</v>
       </c>
       <c r="I21" s="39"/>
-      <c r="J21" s="39"/>
+      <c r="J21" s="39">
+        <v>1</v>
+      </c>
       <c r="K21" s="39"/>
       <c r="L21" s="39"/>
       <c r="M21" s="39"/>
@@ -4800,7 +4838,7 @@
       <c r="O21" s="39"/>
       <c r="P21" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q21" s="39"/>
       <c r="R21" s="39"/>
@@ -4827,7 +4865,7 @@
       <c r="A22" s="21">
         <v>17</v>
       </c>
-      <c r="B22" s="19" t="str">
+      <c r="B22" s="151" t="str">
         <f>+Inscritos!B20</f>
         <v>ISABELA ALVARADO JULIO</v>
       </c>
@@ -4845,7 +4883,9 @@
         <v>2</v>
       </c>
       <c r="I22" s="39"/>
-      <c r="J22" s="39"/>
+      <c r="J22" s="39">
+        <v>1</v>
+      </c>
       <c r="K22" s="39"/>
       <c r="L22" s="39"/>
       <c r="M22" s="39"/>
@@ -4853,7 +4893,7 @@
       <c r="O22" s="40"/>
       <c r="P22" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q22" s="39"/>
       <c r="R22" s="39"/>
@@ -4880,7 +4920,7 @@
       <c r="A23" s="21">
         <v>18</v>
       </c>
-      <c r="B23" s="19" t="str">
+      <c r="B23" s="151" t="str">
         <f>+Inscritos!B21</f>
         <v xml:space="preserve">ISABELA CUITIVA ALFARO </v>
       </c>
@@ -4898,7 +4938,9 @@
         <v>0</v>
       </c>
       <c r="I23" s="39"/>
-      <c r="J23" s="39"/>
+      <c r="J23" s="39">
+        <v>1</v>
+      </c>
       <c r="K23" s="39"/>
       <c r="L23" s="39"/>
       <c r="M23" s="39"/>
@@ -4906,7 +4948,7 @@
       <c r="O23" s="40"/>
       <c r="P23" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q23" s="39"/>
       <c r="R23" s="39"/>
@@ -4933,7 +4975,7 @@
       <c r="A24" s="21">
         <v>19</v>
       </c>
-      <c r="B24" s="19" t="str">
+      <c r="B24" s="151" t="str">
         <f>+Inscritos!B22</f>
         <v xml:space="preserve">ISLENE TEIRUMA LOBO HERNÁNDEZ </v>
       </c>
@@ -4951,7 +4993,9 @@
         <v>3</v>
       </c>
       <c r="I24" s="39"/>
-      <c r="J24" s="39"/>
+      <c r="J24" s="39">
+        <v>0</v>
+      </c>
       <c r="K24" s="39"/>
       <c r="L24" s="39"/>
       <c r="M24" s="39"/>
@@ -5004,7 +5048,9 @@
         <v>0</v>
       </c>
       <c r="I25" s="39"/>
-      <c r="J25" s="39"/>
+      <c r="J25" s="39">
+        <v>1</v>
+      </c>
       <c r="K25" s="39"/>
       <c r="L25" s="39"/>
       <c r="M25" s="39"/>
@@ -5012,7 +5058,7 @@
       <c r="O25" s="39"/>
       <c r="P25" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q25" s="39"/>
       <c r="R25" s="39"/>
@@ -5057,7 +5103,9 @@
         <v>3</v>
       </c>
       <c r="I26" s="39"/>
-      <c r="J26" s="39"/>
+      <c r="J26" s="39">
+        <v>0</v>
+      </c>
       <c r="K26" s="39"/>
       <c r="L26" s="39"/>
       <c r="M26" s="39"/>
@@ -5110,7 +5158,9 @@
         <v>0</v>
       </c>
       <c r="I27" s="39"/>
-      <c r="J27" s="39"/>
+      <c r="J27" s="39">
+        <v>1</v>
+      </c>
       <c r="K27" s="39"/>
       <c r="L27" s="39"/>
       <c r="M27" s="39"/>
@@ -5118,7 +5168,7 @@
       <c r="O27" s="40"/>
       <c r="P27" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q27" s="39"/>
       <c r="R27" s="39"/>
@@ -5163,7 +5213,9 @@
         <v>0</v>
       </c>
       <c r="I28" s="39"/>
-      <c r="J28" s="39"/>
+      <c r="J28" s="39">
+        <v>1</v>
+      </c>
       <c r="K28" s="39"/>
       <c r="L28" s="39"/>
       <c r="M28" s="39"/>
@@ -5171,7 +5223,7 @@
       <c r="O28" s="40"/>
       <c r="P28" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q28" s="39"/>
       <c r="R28" s="39"/>
@@ -5216,7 +5268,9 @@
         <v>1</v>
       </c>
       <c r="I29" s="39"/>
-      <c r="J29" s="39"/>
+      <c r="J29" s="39">
+        <v>1</v>
+      </c>
       <c r="K29" s="39"/>
       <c r="L29" s="39"/>
       <c r="M29" s="39"/>
@@ -5224,7 +5278,7 @@
       <c r="O29" s="40"/>
       <c r="P29" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q29" s="39"/>
       <c r="R29" s="39"/>
@@ -5269,7 +5323,9 @@
         <v>0</v>
       </c>
       <c r="I30" s="39"/>
-      <c r="J30" s="39"/>
+      <c r="J30" s="39">
+        <v>1</v>
+      </c>
       <c r="K30" s="39"/>
       <c r="L30" s="39"/>
       <c r="M30" s="39"/>
@@ -5277,7 +5333,7 @@
       <c r="O30" s="39"/>
       <c r="P30" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q30" s="39"/>
       <c r="R30" s="39"/>
@@ -5322,7 +5378,9 @@
         <v>1</v>
       </c>
       <c r="I31" s="39"/>
-      <c r="J31" s="39"/>
+      <c r="J31" s="39">
+        <v>1</v>
+      </c>
       <c r="K31" s="39"/>
       <c r="L31" s="39"/>
       <c r="M31" s="39"/>
@@ -5330,7 +5388,7 @@
       <c r="O31" s="40"/>
       <c r="P31" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q31" s="39"/>
       <c r="R31" s="39"/>
@@ -5375,7 +5433,9 @@
         <v>1</v>
       </c>
       <c r="I32" s="39"/>
-      <c r="J32" s="39"/>
+      <c r="J32" s="39">
+        <v>1</v>
+      </c>
       <c r="K32" s="39"/>
       <c r="L32" s="39"/>
       <c r="M32" s="39"/>
@@ -5383,7 +5443,7 @@
       <c r="O32" s="40"/>
       <c r="P32" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q32" s="39"/>
       <c r="R32" s="39"/>
@@ -5428,7 +5488,9 @@
         <v>1</v>
       </c>
       <c r="I33" s="39"/>
-      <c r="J33" s="39"/>
+      <c r="J33" s="39">
+        <v>1</v>
+      </c>
       <c r="K33" s="39"/>
       <c r="L33" s="39"/>
       <c r="M33" s="39"/>
@@ -5436,7 +5498,7 @@
       <c r="O33" s="40"/>
       <c r="P33" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q33" s="39"/>
       <c r="R33" s="39"/>
@@ -5481,7 +5543,9 @@
         <v>0</v>
       </c>
       <c r="I34" s="39"/>
-      <c r="J34" s="39"/>
+      <c r="J34" s="39">
+        <v>0</v>
+      </c>
       <c r="K34" s="39"/>
       <c r="L34" s="39"/>
       <c r="M34" s="39"/>
@@ -5534,7 +5598,9 @@
         <v>0</v>
       </c>
       <c r="I35" s="39"/>
-      <c r="J35" s="39"/>
+      <c r="J35" s="39">
+        <v>1</v>
+      </c>
       <c r="K35" s="39"/>
       <c r="L35" s="39"/>
       <c r="M35" s="39"/>
@@ -5542,7 +5608,7 @@
       <c r="O35" s="40"/>
       <c r="P35" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q35" s="39"/>
       <c r="R35" s="39"/>
@@ -5587,7 +5653,9 @@
         <v>1</v>
       </c>
       <c r="I36" s="39"/>
-      <c r="J36" s="39"/>
+      <c r="J36" s="39">
+        <v>1</v>
+      </c>
       <c r="K36" s="39"/>
       <c r="L36" s="39"/>
       <c r="M36" s="39"/>
@@ -5595,7 +5663,7 @@
       <c r="O36" s="39"/>
       <c r="P36" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q36" s="39"/>
       <c r="R36" s="39"/>
@@ -5640,7 +5708,9 @@
         <v>1</v>
       </c>
       <c r="I37" s="39"/>
-      <c r="J37" s="39"/>
+      <c r="J37" s="39">
+        <v>1</v>
+      </c>
       <c r="K37" s="39"/>
       <c r="L37" s="39"/>
       <c r="M37" s="39"/>
@@ -5648,7 +5718,7 @@
       <c r="O37" s="40"/>
       <c r="P37" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q37" s="39"/>
       <c r="R37" s="39"/>
@@ -5693,7 +5763,9 @@
         <v>1</v>
       </c>
       <c r="I38" s="39"/>
-      <c r="J38" s="39"/>
+      <c r="J38" s="39">
+        <v>1</v>
+      </c>
       <c r="K38" s="39"/>
       <c r="L38" s="39"/>
       <c r="M38" s="39"/>
@@ -5701,7 +5773,7 @@
       <c r="O38" s="40"/>
       <c r="P38" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q38" s="39"/>
       <c r="R38" s="39"/>
@@ -5746,7 +5818,9 @@
         <v>2</v>
       </c>
       <c r="I39" s="39"/>
-      <c r="J39" s="39"/>
+      <c r="J39" s="39">
+        <v>1</v>
+      </c>
       <c r="K39" s="39"/>
       <c r="L39" s="39"/>
       <c r="M39" s="39"/>
@@ -5754,7 +5828,7 @@
       <c r="O39" s="40"/>
       <c r="P39" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q39" s="39"/>
       <c r="R39" s="39"/>
@@ -5799,7 +5873,9 @@
         <v>3</v>
       </c>
       <c r="I40" s="39"/>
-      <c r="J40" s="39"/>
+      <c r="J40" s="39">
+        <v>0</v>
+      </c>
       <c r="K40" s="39"/>
       <c r="L40" s="39"/>
       <c r="M40" s="39"/>
@@ -5852,7 +5928,9 @@
         <v>0</v>
       </c>
       <c r="I41" s="39"/>
-      <c r="J41" s="39"/>
+      <c r="J41" s="39">
+        <v>1</v>
+      </c>
       <c r="K41" s="39"/>
       <c r="L41" s="39"/>
       <c r="M41" s="39"/>
@@ -5860,7 +5938,7 @@
       <c r="O41" s="39"/>
       <c r="P41" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q41" s="39"/>
       <c r="R41" s="39"/>
@@ -5905,7 +5983,9 @@
         <v>0</v>
       </c>
       <c r="I42" s="39"/>
-      <c r="J42" s="39"/>
+      <c r="J42" s="39">
+        <v>0</v>
+      </c>
       <c r="K42" s="39"/>
       <c r="L42" s="39"/>
       <c r="M42" s="39"/>
@@ -5958,7 +6038,9 @@
         <v>0</v>
       </c>
       <c r="I43" s="39"/>
-      <c r="J43" s="39"/>
+      <c r="J43" s="39">
+        <v>0</v>
+      </c>
       <c r="K43" s="39"/>
       <c r="L43" s="39"/>
       <c r="M43" s="39"/>
@@ -6011,7 +6093,9 @@
         <v>1</v>
       </c>
       <c r="I44" s="39"/>
-      <c r="J44" s="39"/>
+      <c r="J44" s="39">
+        <v>0</v>
+      </c>
       <c r="K44" s="39"/>
       <c r="L44" s="39"/>
       <c r="M44" s="39"/>
@@ -6064,7 +6148,9 @@
         <v>1</v>
       </c>
       <c r="I45" s="39"/>
-      <c r="J45" s="39"/>
+      <c r="J45" s="39">
+        <v>0</v>
+      </c>
       <c r="K45" s="39"/>
       <c r="L45" s="39"/>
       <c r="M45" s="39"/>
@@ -6117,7 +6203,9 @@
         <v>0</v>
       </c>
       <c r="I46" s="39"/>
-      <c r="J46" s="39"/>
+      <c r="J46" s="39">
+        <v>1</v>
+      </c>
       <c r="K46" s="39"/>
       <c r="L46" s="39"/>
       <c r="M46" s="39"/>
@@ -6125,7 +6213,7 @@
       <c r="O46" s="39"/>
       <c r="P46" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q46" s="39"/>
       <c r="R46" s="39"/>
@@ -6170,7 +6258,9 @@
         <v>1</v>
       </c>
       <c r="I47" s="39"/>
-      <c r="J47" s="39"/>
+      <c r="J47" s="39">
+        <v>1</v>
+      </c>
       <c r="K47" s="39"/>
       <c r="L47" s="39"/>
       <c r="M47" s="39"/>
@@ -6178,7 +6268,7 @@
       <c r="O47" s="40"/>
       <c r="P47" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q47" s="39"/>
       <c r="R47" s="39"/>
@@ -6223,7 +6313,9 @@
         <v>0</v>
       </c>
       <c r="I48" s="39"/>
-      <c r="J48" s="39"/>
+      <c r="J48" s="39">
+        <v>1</v>
+      </c>
       <c r="K48" s="39"/>
       <c r="L48" s="39"/>
       <c r="M48" s="39"/>
@@ -6231,7 +6323,7 @@
       <c r="O48" s="40"/>
       <c r="P48" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q48" s="39"/>
       <c r="R48" s="39"/>
@@ -6276,7 +6368,9 @@
         <v>0</v>
       </c>
       <c r="I49" s="39"/>
-      <c r="J49" s="39"/>
+      <c r="J49" s="39">
+        <v>1</v>
+      </c>
       <c r="K49" s="39"/>
       <c r="L49" s="39"/>
       <c r="M49" s="39"/>
@@ -6284,7 +6378,7 @@
       <c r="O49" s="40"/>
       <c r="P49" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q49" s="39"/>
       <c r="R49" s="39"/>
@@ -6329,7 +6423,9 @@
         <v>0</v>
       </c>
       <c r="I50" s="39"/>
-      <c r="J50" s="39"/>
+      <c r="J50" s="39">
+        <v>0</v>
+      </c>
       <c r="K50" s="39"/>
       <c r="L50" s="39"/>
       <c r="M50" s="39"/>
@@ -6382,7 +6478,9 @@
         <v>0</v>
       </c>
       <c r="I51" s="39"/>
-      <c r="J51" s="39"/>
+      <c r="J51" s="39">
+        <v>1</v>
+      </c>
       <c r="K51" s="39"/>
       <c r="L51" s="39"/>
       <c r="M51" s="39"/>
@@ -6390,7 +6488,7 @@
       <c r="O51" s="40"/>
       <c r="P51" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q51" s="39"/>
       <c r="R51" s="39"/>
@@ -6435,7 +6533,9 @@
         <v>1</v>
       </c>
       <c r="I52" s="39"/>
-      <c r="J52" s="39"/>
+      <c r="J52" s="39">
+        <v>1</v>
+      </c>
       <c r="K52" s="39"/>
       <c r="L52" s="39"/>
       <c r="M52" s="39"/>
@@ -6443,7 +6543,7 @@
       <c r="O52" s="40"/>
       <c r="P52" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q52" s="39"/>
       <c r="R52" s="39"/>
@@ -6488,7 +6588,9 @@
         <v>1</v>
       </c>
       <c r="I53" s="39"/>
-      <c r="J53" s="39"/>
+      <c r="J53" s="39">
+        <v>1</v>
+      </c>
       <c r="K53" s="39"/>
       <c r="L53" s="39"/>
       <c r="M53" s="39"/>
@@ -6496,7 +6598,7 @@
       <c r="O53" s="40"/>
       <c r="P53" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q53" s="39"/>
       <c r="R53" s="39"/>
@@ -6542,7 +6644,9 @@
         <v>2</v>
       </c>
       <c r="I54" s="39"/>
-      <c r="J54" s="39"/>
+      <c r="J54" s="39">
+        <v>0</v>
+      </c>
       <c r="K54" s="39"/>
       <c r="L54" s="39"/>
       <c r="M54" s="39"/>
@@ -7118,123 +7222,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="128" t="s">
+      <c r="B1" s="96" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="128"/>
-      <c r="D1" s="128"/>
-      <c r="E1" s="128"/>
-      <c r="F1" s="128"/>
-      <c r="G1" s="128"/>
-      <c r="H1" s="128"/>
-      <c r="I1" s="128"/>
-      <c r="J1" s="128"/>
-      <c r="K1" s="128"/>
-      <c r="L1" s="128"/>
-      <c r="M1" s="128"/>
-      <c r="N1" s="128"/>
-      <c r="O1" s="128"/>
-      <c r="P1" s="128"/>
-      <c r="Q1" s="128"/>
-      <c r="R1" s="128"/>
-      <c r="S1" s="128"/>
-      <c r="T1" s="128"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="96"/>
+      <c r="J1" s="96"/>
+      <c r="K1" s="96"/>
+      <c r="L1" s="96"/>
+      <c r="M1" s="96"/>
+      <c r="N1" s="96"/>
+      <c r="O1" s="96"/>
+      <c r="P1" s="96"/>
+      <c r="Q1" s="96"/>
+      <c r="R1" s="96"/>
+      <c r="S1" s="96"/>
+      <c r="T1" s="96"/>
     </row>
     <row r="2" spans="1:20" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="110" t="s">
+      <c r="A2" s="133" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="124" t="s">
+      <c r="B2" s="147" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="126" t="s">
+      <c r="C2" s="149" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="98" t="str">
+      <c r="D2" s="124" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="99"/>
-      <c r="F2" s="100"/>
-      <c r="G2" s="98" t="str">
+      <c r="E2" s="125"/>
+      <c r="F2" s="126"/>
+      <c r="G2" s="124" t="str">
         <f>Asistencia!H2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="99"/>
-      <c r="I2" s="99"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="100"/>
-      <c r="L2" s="98" t="s">
+      <c r="H2" s="125"/>
+      <c r="I2" s="125"/>
+      <c r="J2" s="125"/>
+      <c r="K2" s="126"/>
+      <c r="L2" s="124" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="99"/>
-      <c r="N2" s="99"/>
-      <c r="O2" s="99"/>
-      <c r="P2" s="100"/>
-      <c r="Q2" s="98" t="str">
+      <c r="M2" s="125"/>
+      <c r="N2" s="125"/>
+      <c r="O2" s="125"/>
+      <c r="P2" s="126"/>
+      <c r="Q2" s="124" t="str">
         <f>Asistencia!Z2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="99"/>
-      <c r="S2" s="99"/>
-      <c r="T2" s="100"/>
+      <c r="R2" s="125"/>
+      <c r="S2" s="125"/>
+      <c r="T2" s="126"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="111"/>
-      <c r="B3" s="125"/>
-      <c r="C3" s="127"/>
-      <c r="D3" s="118" t="s">
+      <c r="A3" s="134"/>
+      <c r="B3" s="148"/>
+      <c r="C3" s="150"/>
+      <c r="D3" s="141" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="119"/>
-      <c r="F3" s="120"/>
-      <c r="G3" s="112" t="s">
+      <c r="E3" s="142"/>
+      <c r="F3" s="143"/>
+      <c r="G3" s="135" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="113"/>
-      <c r="I3" s="113"/>
-      <c r="J3" s="113"/>
-      <c r="K3" s="114"/>
-      <c r="L3" s="147" t="s">
+      <c r="H3" s="136"/>
+      <c r="I3" s="136"/>
+      <c r="J3" s="136"/>
+      <c r="K3" s="137"/>
+      <c r="L3" s="118" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="148"/>
-      <c r="N3" s="148"/>
-      <c r="O3" s="148"/>
-      <c r="P3" s="149"/>
-      <c r="Q3" s="101" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="102"/>
-      <c r="S3" s="102"/>
-      <c r="T3" s="103"/>
+      <c r="M3" s="119"/>
+      <c r="N3" s="119"/>
+      <c r="O3" s="119"/>
+      <c r="P3" s="120"/>
+      <c r="Q3" s="127" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="128"/>
+      <c r="S3" s="128"/>
+      <c r="T3" s="129"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="111"/>
-      <c r="B4" s="125"/>
-      <c r="C4" s="127"/>
-      <c r="D4" s="121"/>
-      <c r="E4" s="122"/>
-      <c r="F4" s="123"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="116"/>
-      <c r="I4" s="116"/>
-      <c r="J4" s="116"/>
-      <c r="K4" s="117"/>
-      <c r="L4" s="150"/>
-      <c r="M4" s="151"/>
-      <c r="N4" s="151"/>
-      <c r="O4" s="151"/>
-      <c r="P4" s="152"/>
-      <c r="Q4" s="104"/>
-      <c r="R4" s="105"/>
-      <c r="S4" s="105"/>
-      <c r="T4" s="106"/>
+      <c r="A4" s="134"/>
+      <c r="B4" s="148"/>
+      <c r="C4" s="150"/>
+      <c r="D4" s="144"/>
+      <c r="E4" s="145"/>
+      <c r="F4" s="146"/>
+      <c r="G4" s="138"/>
+      <c r="H4" s="139"/>
+      <c r="I4" s="139"/>
+      <c r="J4" s="139"/>
+      <c r="K4" s="140"/>
+      <c r="L4" s="121"/>
+      <c r="M4" s="122"/>
+      <c r="N4" s="122"/>
+      <c r="O4" s="122"/>
+      <c r="P4" s="123"/>
+      <c r="Q4" s="130"/>
+      <c r="R4" s="131"/>
+      <c r="S4" s="131"/>
+      <c r="T4" s="132"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="111"/>
-      <c r="B5" s="125"/>
-      <c r="C5" s="127"/>
+      <c r="A5" s="134"/>
+      <c r="B5" s="148"/>
+      <c r="C5" s="150"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -9766,183 +9870,192 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D65" s="132" t="s">
+      <c r="D65" s="100" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="135" t="s">
+      <c r="E65" s="103" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="129" t="s">
+      <c r="G65" s="97" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="141" t="s">
+      <c r="H65" s="112" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="141" t="s">
+      <c r="I65" s="112" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="129" t="s">
+      <c r="J65" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="107" t="s">
+      <c r="L65" s="106" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="138" t="s">
+      <c r="M65" s="109" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="138" t="s">
+      <c r="N65" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="107" t="s">
+      <c r="O65" s="106" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="144" t="s">
+      <c r="Q65" s="115" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="144" t="s">
+      <c r="R65" s="115" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="144" t="s">
+      <c r="S65" s="115" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D66" s="133"/>
-      <c r="E66" s="136"/>
-      <c r="G66" s="130"/>
-      <c r="H66" s="142"/>
-      <c r="I66" s="142"/>
-      <c r="J66" s="130"/>
-      <c r="L66" s="108"/>
-      <c r="M66" s="139"/>
-      <c r="N66" s="139"/>
-      <c r="O66" s="108"/>
-      <c r="Q66" s="145"/>
-      <c r="R66" s="145"/>
-      <c r="S66" s="145"/>
+      <c r="D66" s="101"/>
+      <c r="E66" s="104"/>
+      <c r="G66" s="98"/>
+      <c r="H66" s="113"/>
+      <c r="I66" s="113"/>
+      <c r="J66" s="98"/>
+      <c r="L66" s="107"/>
+      <c r="M66" s="110"/>
+      <c r="N66" s="110"/>
+      <c r="O66" s="107"/>
+      <c r="Q66" s="116"/>
+      <c r="R66" s="116"/>
+      <c r="S66" s="116"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D67" s="133"/>
-      <c r="E67" s="136"/>
-      <c r="G67" s="130"/>
-      <c r="H67" s="142"/>
-      <c r="I67" s="142"/>
-      <c r="J67" s="130"/>
-      <c r="L67" s="108"/>
-      <c r="M67" s="139"/>
-      <c r="N67" s="139"/>
-      <c r="O67" s="108"/>
-      <c r="Q67" s="145"/>
-      <c r="R67" s="145"/>
-      <c r="S67" s="145"/>
+      <c r="D67" s="101"/>
+      <c r="E67" s="104"/>
+      <c r="G67" s="98"/>
+      <c r="H67" s="113"/>
+      <c r="I67" s="113"/>
+      <c r="J67" s="98"/>
+      <c r="L67" s="107"/>
+      <c r="M67" s="110"/>
+      <c r="N67" s="110"/>
+      <c r="O67" s="107"/>
+      <c r="Q67" s="116"/>
+      <c r="R67" s="116"/>
+      <c r="S67" s="116"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D68" s="133"/>
-      <c r="E68" s="136"/>
-      <c r="G68" s="130"/>
-      <c r="H68" s="142"/>
-      <c r="I68" s="142"/>
-      <c r="J68" s="130"/>
-      <c r="L68" s="108"/>
-      <c r="M68" s="139"/>
-      <c r="N68" s="139"/>
-      <c r="O68" s="108"/>
-      <c r="Q68" s="145"/>
-      <c r="R68" s="145"/>
-      <c r="S68" s="145"/>
+      <c r="D68" s="101"/>
+      <c r="E68" s="104"/>
+      <c r="G68" s="98"/>
+      <c r="H68" s="113"/>
+      <c r="I68" s="113"/>
+      <c r="J68" s="98"/>
+      <c r="L68" s="107"/>
+      <c r="M68" s="110"/>
+      <c r="N68" s="110"/>
+      <c r="O68" s="107"/>
+      <c r="Q68" s="116"/>
+      <c r="R68" s="116"/>
+      <c r="S68" s="116"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D69" s="133"/>
-      <c r="E69" s="136"/>
-      <c r="G69" s="130"/>
-      <c r="H69" s="142"/>
-      <c r="I69" s="142"/>
-      <c r="J69" s="130"/>
-      <c r="L69" s="108"/>
-      <c r="M69" s="139"/>
-      <c r="N69" s="139"/>
-      <c r="O69" s="108"/>
-      <c r="Q69" s="145"/>
-      <c r="R69" s="145"/>
-      <c r="S69" s="145"/>
+      <c r="D69" s="101"/>
+      <c r="E69" s="104"/>
+      <c r="G69" s="98"/>
+      <c r="H69" s="113"/>
+      <c r="I69" s="113"/>
+      <c r="J69" s="98"/>
+      <c r="L69" s="107"/>
+      <c r="M69" s="110"/>
+      <c r="N69" s="110"/>
+      <c r="O69" s="107"/>
+      <c r="Q69" s="116"/>
+      <c r="R69" s="116"/>
+      <c r="S69" s="116"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D70" s="133"/>
-      <c r="E70" s="136"/>
-      <c r="G70" s="130"/>
-      <c r="H70" s="142"/>
-      <c r="I70" s="142"/>
-      <c r="J70" s="130"/>
-      <c r="L70" s="108"/>
-      <c r="M70" s="139"/>
-      <c r="N70" s="139"/>
-      <c r="O70" s="108"/>
-      <c r="Q70" s="145"/>
-      <c r="R70" s="145"/>
-      <c r="S70" s="145"/>
+      <c r="D70" s="101"/>
+      <c r="E70" s="104"/>
+      <c r="G70" s="98"/>
+      <c r="H70" s="113"/>
+      <c r="I70" s="113"/>
+      <c r="J70" s="98"/>
+      <c r="L70" s="107"/>
+      <c r="M70" s="110"/>
+      <c r="N70" s="110"/>
+      <c r="O70" s="107"/>
+      <c r="Q70" s="116"/>
+      <c r="R70" s="116"/>
+      <c r="S70" s="116"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D71" s="133"/>
-      <c r="E71" s="136"/>
-      <c r="G71" s="130"/>
-      <c r="H71" s="142"/>
-      <c r="I71" s="142"/>
-      <c r="J71" s="130"/>
-      <c r="L71" s="108"/>
-      <c r="M71" s="139"/>
-      <c r="N71" s="139"/>
-      <c r="O71" s="108"/>
-      <c r="Q71" s="145"/>
-      <c r="R71" s="145"/>
-      <c r="S71" s="145"/>
+      <c r="D71" s="101"/>
+      <c r="E71" s="104"/>
+      <c r="G71" s="98"/>
+      <c r="H71" s="113"/>
+      <c r="I71" s="113"/>
+      <c r="J71" s="98"/>
+      <c r="L71" s="107"/>
+      <c r="M71" s="110"/>
+      <c r="N71" s="110"/>
+      <c r="O71" s="107"/>
+      <c r="Q71" s="116"/>
+      <c r="R71" s="116"/>
+      <c r="S71" s="116"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D72" s="133"/>
-      <c r="E72" s="136"/>
-      <c r="G72" s="130"/>
-      <c r="H72" s="142"/>
-      <c r="I72" s="142"/>
-      <c r="J72" s="130"/>
-      <c r="L72" s="108"/>
-      <c r="M72" s="139"/>
-      <c r="N72" s="139"/>
-      <c r="O72" s="108"/>
-      <c r="Q72" s="145"/>
-      <c r="R72" s="145"/>
-      <c r="S72" s="145"/>
+      <c r="D72" s="101"/>
+      <c r="E72" s="104"/>
+      <c r="G72" s="98"/>
+      <c r="H72" s="113"/>
+      <c r="I72" s="113"/>
+      <c r="J72" s="98"/>
+      <c r="L72" s="107"/>
+      <c r="M72" s="110"/>
+      <c r="N72" s="110"/>
+      <c r="O72" s="107"/>
+      <c r="Q72" s="116"/>
+      <c r="R72" s="116"/>
+      <c r="S72" s="116"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.3">
-      <c r="D73" s="133"/>
-      <c r="E73" s="136"/>
-      <c r="G73" s="130"/>
-      <c r="H73" s="142"/>
-      <c r="I73" s="142"/>
-      <c r="J73" s="130"/>
-      <c r="L73" s="108"/>
-      <c r="M73" s="139"/>
-      <c r="N73" s="139"/>
-      <c r="O73" s="108"/>
-      <c r="Q73" s="145"/>
-      <c r="R73" s="145"/>
-      <c r="S73" s="145"/>
+      <c r="D73" s="101"/>
+      <c r="E73" s="104"/>
+      <c r="G73" s="98"/>
+      <c r="H73" s="113"/>
+      <c r="I73" s="113"/>
+      <c r="J73" s="98"/>
+      <c r="L73" s="107"/>
+      <c r="M73" s="110"/>
+      <c r="N73" s="110"/>
+      <c r="O73" s="107"/>
+      <c r="Q73" s="116"/>
+      <c r="R73" s="116"/>
+      <c r="S73" s="116"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D74" s="134"/>
-      <c r="E74" s="137"/>
-      <c r="G74" s="131"/>
-      <c r="H74" s="143"/>
-      <c r="I74" s="143"/>
-      <c r="J74" s="131"/>
-      <c r="L74" s="109"/>
-      <c r="M74" s="140"/>
-      <c r="N74" s="140"/>
-      <c r="O74" s="109"/>
-      <c r="Q74" s="146"/>
-      <c r="R74" s="146"/>
-      <c r="S74" s="146"/>
+      <c r="D74" s="102"/>
+      <c r="E74" s="105"/>
+      <c r="G74" s="99"/>
+      <c r="H74" s="114"/>
+      <c r="I74" s="114"/>
+      <c r="J74" s="99"/>
+      <c r="L74" s="108"/>
+      <c r="M74" s="111"/>
+      <c r="N74" s="111"/>
+      <c r="O74" s="108"/>
+      <c r="Q74" s="117"/>
+      <c r="R74" s="117"/>
+      <c r="S74" s="117"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -9959,15 +10072,6 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
ya terminé de preparar el tema 15
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5F5D48-2978-40B9-953A-2AF1117E4D14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F77E93-A66C-41CA-8940-D108B37648BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
@@ -1262,7 +1262,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1441,8 +1441,95 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1456,94 +1543,94 @@
     <xf numFmtId="0" fontId="19" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1576,15 +1663,6 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1630,86 +1708,11 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2217,28 +2220,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="93" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="66"/>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="94"/>
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="94"/>
+      <c r="H1" s="95"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="92"/>
+      <c r="D2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="92"/>
+      <c r="G2" s="92"/>
+      <c r="H2" s="92"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
@@ -3769,37 +3772,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="74" t="s">
+      <c r="B1" s="69" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
-      <c r="I1" s="74"/>
-      <c r="J1" s="74"/>
-      <c r="K1" s="74"/>
-      <c r="L1" s="74"/>
-      <c r="M1" s="74"/>
-      <c r="N1" s="74"/>
-      <c r="O1" s="74"/>
-      <c r="P1" s="74"/>
-      <c r="Q1" s="74"/>
-      <c r="R1" s="74"/>
-      <c r="S1" s="74"/>
-      <c r="T1" s="74"/>
-      <c r="U1" s="74"/>
-      <c r="V1" s="74"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="69"/>
+      <c r="Z1" s="69"/>
+      <c r="AA1" s="69"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="69"/>
+      <c r="AD1" s="69"/>
     </row>
     <row r="2" spans="1:30" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="55" t="s">
@@ -3811,120 +3814,120 @@
       <c r="C2" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="90" t="s">
+      <c r="D2" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="92"/>
-      <c r="H2" s="75" t="s">
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="70" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="76"/>
-      <c r="N2" s="76"/>
-      <c r="O2" s="76"/>
-      <c r="P2" s="77"/>
-      <c r="Q2" s="84" t="s">
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
+      <c r="M2" s="71"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="71"/>
+      <c r="P2" s="72"/>
+      <c r="Q2" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="85"/>
-      <c r="S2" s="85"/>
-      <c r="T2" s="85"/>
-      <c r="U2" s="85"/>
-      <c r="V2" s="85"/>
-      <c r="W2" s="85"/>
-      <c r="X2" s="85"/>
-      <c r="Y2" s="86"/>
-      <c r="Z2" s="67" t="s">
+      <c r="R2" s="80"/>
+      <c r="S2" s="80"/>
+      <c r="T2" s="80"/>
+      <c r="U2" s="80"/>
+      <c r="V2" s="80"/>
+      <c r="W2" s="80"/>
+      <c r="X2" s="80"/>
+      <c r="Y2" s="81"/>
+      <c r="Z2" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="AA2" s="68"/>
-      <c r="AB2" s="68"/>
-      <c r="AC2" s="68"/>
-      <c r="AD2" s="69"/>
+      <c r="AA2" s="63"/>
+      <c r="AB2" s="63"/>
+      <c r="AC2" s="63"/>
+      <c r="AD2" s="64"/>
     </row>
     <row r="3" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="56"/>
       <c r="B3" s="54"/>
       <c r="C3" s="56"/>
-      <c r="D3" s="93" t="s">
+      <c r="D3" s="88" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="94"/>
-      <c r="F3" s="94"/>
-      <c r="G3" s="95"/>
-      <c r="H3" s="78" t="s">
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="79"/>
-      <c r="J3" s="79"/>
-      <c r="K3" s="79"/>
-      <c r="L3" s="79"/>
-      <c r="M3" s="79"/>
-      <c r="N3" s="79"/>
-      <c r="O3" s="79"/>
-      <c r="P3" s="80"/>
-      <c r="Q3" s="87" t="s">
+      <c r="I3" s="74"/>
+      <c r="J3" s="74"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="74"/>
+      <c r="M3" s="74"/>
+      <c r="N3" s="74"/>
+      <c r="O3" s="74"/>
+      <c r="P3" s="75"/>
+      <c r="Q3" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="R3" s="88"/>
-      <c r="S3" s="88"/>
-      <c r="T3" s="88"/>
-      <c r="U3" s="88"/>
-      <c r="V3" s="88"/>
-      <c r="W3" s="88"/>
-      <c r="X3" s="88"/>
-      <c r="Y3" s="89"/>
-      <c r="Z3" s="70" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="71"/>
-      <c r="AB3" s="71"/>
-      <c r="AC3" s="71"/>
-      <c r="AD3" s="72"/>
+      <c r="R3" s="83"/>
+      <c r="S3" s="83"/>
+      <c r="T3" s="83"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="83"/>
+      <c r="W3" s="83"/>
+      <c r="X3" s="83"/>
+      <c r="Y3" s="84"/>
+      <c r="Z3" s="65" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="66"/>
+      <c r="AB3" s="66"/>
+      <c r="AC3" s="66"/>
+      <c r="AD3" s="67"/>
     </row>
     <row r="4" spans="1:30" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="56"/>
       <c r="B4" s="54"/>
       <c r="C4" s="56"/>
-      <c r="D4" s="96" t="s">
+      <c r="D4" s="91" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="82"/>
-      <c r="F4" s="82"/>
+      <c r="E4" s="77"/>
+      <c r="F4" s="77"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="81" t="s">
+      <c r="H4" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="82"/>
-      <c r="J4" s="82"/>
-      <c r="K4" s="82"/>
-      <c r="L4" s="82"/>
-      <c r="M4" s="82"/>
-      <c r="N4" s="82"/>
-      <c r="O4" s="83"/>
+      <c r="I4" s="77"/>
+      <c r="J4" s="77"/>
+      <c r="K4" s="77"/>
+      <c r="L4" s="77"/>
+      <c r="M4" s="77"/>
+      <c r="N4" s="77"/>
+      <c r="O4" s="78"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="81" t="s">
+      <c r="Q4" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="R4" s="82"/>
-      <c r="S4" s="82"/>
-      <c r="T4" s="82"/>
-      <c r="U4" s="82"/>
-      <c r="V4" s="82"/>
-      <c r="W4" s="82"/>
-      <c r="X4" s="83"/>
+      <c r="R4" s="77"/>
+      <c r="S4" s="77"/>
+      <c r="T4" s="77"/>
+      <c r="U4" s="77"/>
+      <c r="V4" s="77"/>
+      <c r="W4" s="77"/>
+      <c r="X4" s="78"/>
       <c r="Y4" s="13"/>
-      <c r="Z4" s="73" t="s">
+      <c r="Z4" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="AA4" s="73"/>
-      <c r="AB4" s="73"/>
-      <c r="AC4" s="73"/>
+      <c r="AA4" s="68"/>
+      <c r="AB4" s="68"/>
+      <c r="AC4" s="68"/>
       <c r="AD4" s="3"/>
     </row>
     <row r="5" spans="1:30" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -4969,7 +4972,7 @@
       <c r="A24" s="21">
         <v>19</v>
       </c>
-      <c r="B24" s="62" t="str">
+      <c r="B24" s="152" t="str">
         <f>+Inscritos!B22</f>
         <v xml:space="preserve">ISLENE TEIRUMA LOBO HERNÁNDEZ </v>
       </c>
@@ -5024,7 +5027,7 @@
       <c r="A25" s="21">
         <v>20</v>
       </c>
-      <c r="B25" s="62" t="str">
+      <c r="B25" s="152" t="str">
         <f>+Inscritos!B23</f>
         <v xml:space="preserve">JEAN CARLOS QUIÑONES HOYOS </v>
       </c>
@@ -5079,7 +5082,7 @@
       <c r="A26" s="21">
         <v>21</v>
       </c>
-      <c r="B26" s="62" t="str">
+      <c r="B26" s="152" t="str">
         <f>+Inscritos!B24</f>
         <v>JORGE ANDRES ARRIETA GARCIA</v>
       </c>
@@ -5134,7 +5137,7 @@
       <c r="A27" s="21">
         <v>22</v>
       </c>
-      <c r="B27" s="62" t="str">
+      <c r="B27" s="152" t="str">
         <f>+Inscritos!B25</f>
         <v>JULIAN ANDRES SAENZ MOLINA</v>
       </c>
@@ -5189,7 +5192,7 @@
       <c r="A28" s="21">
         <v>23</v>
       </c>
-      <c r="B28" s="62" t="str">
+      <c r="B28" s="152" t="str">
         <f>+Inscritos!B26</f>
         <v>JUNIOR ANDRES CALLE SAMARRA</v>
       </c>
@@ -5244,7 +5247,7 @@
       <c r="A29" s="21">
         <v>24</v>
       </c>
-      <c r="B29" s="62" t="str">
+      <c r="B29" s="152" t="str">
         <f>+Inscritos!B27</f>
         <v xml:space="preserve">KAREN NOEMITH NIETO DE AGUAS </v>
       </c>
@@ -5299,7 +5302,7 @@
       <c r="A30" s="21">
         <v>25</v>
       </c>
-      <c r="B30" s="62" t="str">
+      <c r="B30" s="152" t="str">
         <f>+Inscritos!B28</f>
         <v xml:space="preserve">KATERINE HOLGUIN BENAVIDES </v>
       </c>
@@ -5354,7 +5357,7 @@
       <c r="A31" s="21">
         <v>26</v>
       </c>
-      <c r="B31" s="62" t="str">
+      <c r="B31" s="152" t="str">
         <f>+Inscritos!B29</f>
         <v xml:space="preserve">KATIA ANDREA FERNÁNDEZ RAMOS </v>
       </c>
@@ -5409,7 +5412,7 @@
       <c r="A32" s="21">
         <v>27</v>
       </c>
-      <c r="B32" s="19" t="str">
+      <c r="B32" s="151" t="str">
         <f>+Inscritos!B30</f>
         <v xml:space="preserve">KEIDER LUIS SUAREZ CALDEÑO </v>
       </c>
@@ -5464,7 +5467,7 @@
       <c r="A33" s="21">
         <v>28</v>
       </c>
-      <c r="B33" s="19" t="str">
+      <c r="B33" s="151" t="str">
         <f>+Inscritos!B31</f>
         <v xml:space="preserve">KEINER NICK TUIRAN CUITIVA </v>
       </c>
@@ -5519,7 +5522,7 @@
       <c r="A34" s="21">
         <v>29</v>
       </c>
-      <c r="B34" s="19" t="str">
+      <c r="B34" s="151" t="str">
         <f>+Inscritos!B32</f>
         <v xml:space="preserve">KENDIS ESTER MONTIEL VILLALOBOS </v>
       </c>
@@ -5574,7 +5577,7 @@
       <c r="A35" s="21">
         <v>30</v>
       </c>
-      <c r="B35" s="19" t="str">
+      <c r="B35" s="151" t="str">
         <f>+Inscritos!B33</f>
         <v xml:space="preserve">KEVIN DAVID ACOSTA RAMOS </v>
       </c>
@@ -5629,7 +5632,7 @@
       <c r="A36" s="21">
         <v>31</v>
       </c>
-      <c r="B36" s="19" t="str">
+      <c r="B36" s="151" t="str">
         <f>+Inscritos!B34</f>
         <v xml:space="preserve">LENIS ENITH ORTEGA FUENTES </v>
       </c>
@@ -5684,7 +5687,7 @@
       <c r="A37" s="21">
         <v>32</v>
       </c>
-      <c r="B37" s="19" t="str">
+      <c r="B37" s="151" t="str">
         <f>+Inscritos!B35</f>
         <v xml:space="preserve">LILIANA ÁLVAREZ FLÓREZ </v>
       </c>
@@ -7216,123 +7219,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="97" t="s">
+      <c r="B1" s="126" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="97"/>
-      <c r="D1" s="97"/>
-      <c r="E1" s="97"/>
-      <c r="F1" s="97"/>
-      <c r="G1" s="97"/>
-      <c r="H1" s="97"/>
-      <c r="I1" s="97"/>
-      <c r="J1" s="97"/>
-      <c r="K1" s="97"/>
-      <c r="L1" s="97"/>
-      <c r="M1" s="97"/>
-      <c r="N1" s="97"/>
-      <c r="O1" s="97"/>
-      <c r="P1" s="97"/>
-      <c r="Q1" s="97"/>
-      <c r="R1" s="97"/>
-      <c r="S1" s="97"/>
-      <c r="T1" s="97"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
+      <c r="G1" s="126"/>
+      <c r="H1" s="126"/>
+      <c r="I1" s="126"/>
+      <c r="J1" s="126"/>
+      <c r="K1" s="126"/>
+      <c r="L1" s="126"/>
+      <c r="M1" s="126"/>
+      <c r="N1" s="126"/>
+      <c r="O1" s="126"/>
+      <c r="P1" s="126"/>
+      <c r="Q1" s="126"/>
+      <c r="R1" s="126"/>
+      <c r="S1" s="126"/>
+      <c r="T1" s="126"/>
     </row>
     <row r="2" spans="1:20" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="134" t="s">
+      <c r="A2" s="108" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="148" t="s">
+      <c r="B2" s="122" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="150" t="s">
+      <c r="C2" s="124" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="125" t="str">
+      <c r="D2" s="96" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="126"/>
-      <c r="F2" s="127"/>
-      <c r="G2" s="125" t="str">
+      <c r="E2" s="97"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="96" t="str">
         <f>Asistencia!H2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="127"/>
-      <c r="L2" s="125" t="s">
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="98"/>
+      <c r="L2" s="96" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
-      <c r="Q2" s="125" t="str">
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
+      <c r="P2" s="98"/>
+      <c r="Q2" s="96" t="str">
         <f>Asistencia!Z2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="126"/>
-      <c r="S2" s="126"/>
-      <c r="T2" s="127"/>
+      <c r="R2" s="97"/>
+      <c r="S2" s="97"/>
+      <c r="T2" s="98"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="135"/>
-      <c r="B3" s="149"/>
-      <c r="C3" s="151"/>
-      <c r="D3" s="142" t="s">
+      <c r="A3" s="109"/>
+      <c r="B3" s="123"/>
+      <c r="C3" s="125"/>
+      <c r="D3" s="116" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="143"/>
-      <c r="F3" s="144"/>
-      <c r="G3" s="136" t="s">
+      <c r="E3" s="117"/>
+      <c r="F3" s="118"/>
+      <c r="G3" s="110" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="137"/>
-      <c r="I3" s="137"/>
-      <c r="J3" s="137"/>
-      <c r="K3" s="138"/>
-      <c r="L3" s="119" t="s">
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="112"/>
+      <c r="L3" s="145" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="120"/>
-      <c r="N3" s="120"/>
-      <c r="O3" s="120"/>
-      <c r="P3" s="121"/>
-      <c r="Q3" s="128" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="129"/>
-      <c r="S3" s="129"/>
-      <c r="T3" s="130"/>
+      <c r="M3" s="146"/>
+      <c r="N3" s="146"/>
+      <c r="O3" s="146"/>
+      <c r="P3" s="147"/>
+      <c r="Q3" s="99" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="100"/>
+      <c r="S3" s="100"/>
+      <c r="T3" s="101"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="135"/>
-      <c r="B4" s="149"/>
-      <c r="C4" s="151"/>
-      <c r="D4" s="145"/>
-      <c r="E4" s="146"/>
-      <c r="F4" s="147"/>
-      <c r="G4" s="139"/>
-      <c r="H4" s="140"/>
-      <c r="I4" s="140"/>
-      <c r="J4" s="140"/>
-      <c r="K4" s="141"/>
-      <c r="L4" s="122"/>
-      <c r="M4" s="123"/>
-      <c r="N4" s="123"/>
-      <c r="O4" s="123"/>
-      <c r="P4" s="124"/>
-      <c r="Q4" s="131"/>
-      <c r="R4" s="132"/>
-      <c r="S4" s="132"/>
-      <c r="T4" s="133"/>
+      <c r="A4" s="109"/>
+      <c r="B4" s="123"/>
+      <c r="C4" s="125"/>
+      <c r="D4" s="119"/>
+      <c r="E4" s="120"/>
+      <c r="F4" s="121"/>
+      <c r="G4" s="113"/>
+      <c r="H4" s="114"/>
+      <c r="I4" s="114"/>
+      <c r="J4" s="114"/>
+      <c r="K4" s="115"/>
+      <c r="L4" s="148"/>
+      <c r="M4" s="149"/>
+      <c r="N4" s="149"/>
+      <c r="O4" s="149"/>
+      <c r="P4" s="150"/>
+      <c r="Q4" s="102"/>
+      <c r="R4" s="103"/>
+      <c r="S4" s="103"/>
+      <c r="T4" s="104"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="135"/>
-      <c r="B5" s="149"/>
-      <c r="C5" s="151"/>
+      <c r="A5" s="109"/>
+      <c r="B5" s="123"/>
+      <c r="C5" s="125"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -9864,192 +9867,183 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D65" s="101" t="s">
+      <c r="D65" s="130" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="104" t="s">
+      <c r="E65" s="133" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="98" t="s">
+      <c r="G65" s="127" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="113" t="s">
+      <c r="H65" s="139" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="113" t="s">
+      <c r="I65" s="139" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="98" t="s">
+      <c r="J65" s="127" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="107" t="s">
+      <c r="L65" s="105" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="110" t="s">
+      <c r="M65" s="136" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="110" t="s">
+      <c r="N65" s="136" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="107" t="s">
+      <c r="O65" s="105" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="116" t="s">
+      <c r="Q65" s="142" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="116" t="s">
+      <c r="R65" s="142" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="116" t="s">
+      <c r="S65" s="142" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D66" s="102"/>
-      <c r="E66" s="105"/>
-      <c r="G66" s="99"/>
-      <c r="H66" s="114"/>
-      <c r="I66" s="114"/>
-      <c r="J66" s="99"/>
-      <c r="L66" s="108"/>
-      <c r="M66" s="111"/>
-      <c r="N66" s="111"/>
-      <c r="O66" s="108"/>
-      <c r="Q66" s="117"/>
-      <c r="R66" s="117"/>
-      <c r="S66" s="117"/>
+      <c r="D66" s="131"/>
+      <c r="E66" s="134"/>
+      <c r="G66" s="128"/>
+      <c r="H66" s="140"/>
+      <c r="I66" s="140"/>
+      <c r="J66" s="128"/>
+      <c r="L66" s="106"/>
+      <c r="M66" s="137"/>
+      <c r="N66" s="137"/>
+      <c r="O66" s="106"/>
+      <c r="Q66" s="143"/>
+      <c r="R66" s="143"/>
+      <c r="S66" s="143"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D67" s="102"/>
-      <c r="E67" s="105"/>
-      <c r="G67" s="99"/>
-      <c r="H67" s="114"/>
-      <c r="I67" s="114"/>
-      <c r="J67" s="99"/>
-      <c r="L67" s="108"/>
-      <c r="M67" s="111"/>
-      <c r="N67" s="111"/>
-      <c r="O67" s="108"/>
-      <c r="Q67" s="117"/>
-      <c r="R67" s="117"/>
-      <c r="S67" s="117"/>
+      <c r="D67" s="131"/>
+      <c r="E67" s="134"/>
+      <c r="G67" s="128"/>
+      <c r="H67" s="140"/>
+      <c r="I67" s="140"/>
+      <c r="J67" s="128"/>
+      <c r="L67" s="106"/>
+      <c r="M67" s="137"/>
+      <c r="N67" s="137"/>
+      <c r="O67" s="106"/>
+      <c r="Q67" s="143"/>
+      <c r="R67" s="143"/>
+      <c r="S67" s="143"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D68" s="102"/>
-      <c r="E68" s="105"/>
-      <c r="G68" s="99"/>
-      <c r="H68" s="114"/>
-      <c r="I68" s="114"/>
-      <c r="J68" s="99"/>
-      <c r="L68" s="108"/>
-      <c r="M68" s="111"/>
-      <c r="N68" s="111"/>
-      <c r="O68" s="108"/>
-      <c r="Q68" s="117"/>
-      <c r="R68" s="117"/>
-      <c r="S68" s="117"/>
+      <c r="D68" s="131"/>
+      <c r="E68" s="134"/>
+      <c r="G68" s="128"/>
+      <c r="H68" s="140"/>
+      <c r="I68" s="140"/>
+      <c r="J68" s="128"/>
+      <c r="L68" s="106"/>
+      <c r="M68" s="137"/>
+      <c r="N68" s="137"/>
+      <c r="O68" s="106"/>
+      <c r="Q68" s="143"/>
+      <c r="R68" s="143"/>
+      <c r="S68" s="143"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D69" s="102"/>
-      <c r="E69" s="105"/>
-      <c r="G69" s="99"/>
-      <c r="H69" s="114"/>
-      <c r="I69" s="114"/>
-      <c r="J69" s="99"/>
-      <c r="L69" s="108"/>
-      <c r="M69" s="111"/>
-      <c r="N69" s="111"/>
-      <c r="O69" s="108"/>
-      <c r="Q69" s="117"/>
-      <c r="R69" s="117"/>
-      <c r="S69" s="117"/>
+      <c r="D69" s="131"/>
+      <c r="E69" s="134"/>
+      <c r="G69" s="128"/>
+      <c r="H69" s="140"/>
+      <c r="I69" s="140"/>
+      <c r="J69" s="128"/>
+      <c r="L69" s="106"/>
+      <c r="M69" s="137"/>
+      <c r="N69" s="137"/>
+      <c r="O69" s="106"/>
+      <c r="Q69" s="143"/>
+      <c r="R69" s="143"/>
+      <c r="S69" s="143"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D70" s="102"/>
-      <c r="E70" s="105"/>
-      <c r="G70" s="99"/>
-      <c r="H70" s="114"/>
-      <c r="I70" s="114"/>
-      <c r="J70" s="99"/>
-      <c r="L70" s="108"/>
-      <c r="M70" s="111"/>
-      <c r="N70" s="111"/>
-      <c r="O70" s="108"/>
-      <c r="Q70" s="117"/>
-      <c r="R70" s="117"/>
-      <c r="S70" s="117"/>
+      <c r="D70" s="131"/>
+      <c r="E70" s="134"/>
+      <c r="G70" s="128"/>
+      <c r="H70" s="140"/>
+      <c r="I70" s="140"/>
+      <c r="J70" s="128"/>
+      <c r="L70" s="106"/>
+      <c r="M70" s="137"/>
+      <c r="N70" s="137"/>
+      <c r="O70" s="106"/>
+      <c r="Q70" s="143"/>
+      <c r="R70" s="143"/>
+      <c r="S70" s="143"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D71" s="102"/>
-      <c r="E71" s="105"/>
-      <c r="G71" s="99"/>
-      <c r="H71" s="114"/>
-      <c r="I71" s="114"/>
-      <c r="J71" s="99"/>
-      <c r="L71" s="108"/>
-      <c r="M71" s="111"/>
-      <c r="N71" s="111"/>
-      <c r="O71" s="108"/>
-      <c r="Q71" s="117"/>
-      <c r="R71" s="117"/>
-      <c r="S71" s="117"/>
+      <c r="D71" s="131"/>
+      <c r="E71" s="134"/>
+      <c r="G71" s="128"/>
+      <c r="H71" s="140"/>
+      <c r="I71" s="140"/>
+      <c r="J71" s="128"/>
+      <c r="L71" s="106"/>
+      <c r="M71" s="137"/>
+      <c r="N71" s="137"/>
+      <c r="O71" s="106"/>
+      <c r="Q71" s="143"/>
+      <c r="R71" s="143"/>
+      <c r="S71" s="143"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D72" s="102"/>
-      <c r="E72" s="105"/>
-      <c r="G72" s="99"/>
-      <c r="H72" s="114"/>
-      <c r="I72" s="114"/>
-      <c r="J72" s="99"/>
-      <c r="L72" s="108"/>
-      <c r="M72" s="111"/>
-      <c r="N72" s="111"/>
-      <c r="O72" s="108"/>
-      <c r="Q72" s="117"/>
-      <c r="R72" s="117"/>
-      <c r="S72" s="117"/>
+      <c r="D72" s="131"/>
+      <c r="E72" s="134"/>
+      <c r="G72" s="128"/>
+      <c r="H72" s="140"/>
+      <c r="I72" s="140"/>
+      <c r="J72" s="128"/>
+      <c r="L72" s="106"/>
+      <c r="M72" s="137"/>
+      <c r="N72" s="137"/>
+      <c r="O72" s="106"/>
+      <c r="Q72" s="143"/>
+      <c r="R72" s="143"/>
+      <c r="S72" s="143"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D73" s="102"/>
-      <c r="E73" s="105"/>
-      <c r="G73" s="99"/>
-      <c r="H73" s="114"/>
-      <c r="I73" s="114"/>
-      <c r="J73" s="99"/>
-      <c r="L73" s="108"/>
-      <c r="M73" s="111"/>
-      <c r="N73" s="111"/>
-      <c r="O73" s="108"/>
-      <c r="Q73" s="117"/>
-      <c r="R73" s="117"/>
-      <c r="S73" s="117"/>
+      <c r="D73" s="131"/>
+      <c r="E73" s="134"/>
+      <c r="G73" s="128"/>
+      <c r="H73" s="140"/>
+      <c r="I73" s="140"/>
+      <c r="J73" s="128"/>
+      <c r="L73" s="106"/>
+      <c r="M73" s="137"/>
+      <c r="N73" s="137"/>
+      <c r="O73" s="106"/>
+      <c r="Q73" s="143"/>
+      <c r="R73" s="143"/>
+      <c r="S73" s="143"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D74" s="103"/>
-      <c r="E74" s="106"/>
-      <c r="G74" s="100"/>
-      <c r="H74" s="115"/>
-      <c r="I74" s="115"/>
-      <c r="J74" s="100"/>
-      <c r="L74" s="109"/>
-      <c r="M74" s="112"/>
-      <c r="N74" s="112"/>
-      <c r="O74" s="109"/>
-      <c r="Q74" s="118"/>
-      <c r="R74" s="118"/>
-      <c r="S74" s="118"/>
+      <c r="D74" s="132"/>
+      <c r="E74" s="135"/>
+      <c r="G74" s="129"/>
+      <c r="H74" s="141"/>
+      <c r="I74" s="141"/>
+      <c r="J74" s="129"/>
+      <c r="L74" s="107"/>
+      <c r="M74" s="138"/>
+      <c r="N74" s="138"/>
+      <c r="O74" s="107"/>
+      <c r="Q74" s="144"/>
+      <c r="R74" s="144"/>
+      <c r="S74" s="144"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -10066,6 +10060,15 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
se agregó la presentación del concepto de progresión aritmética.
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35F77E93-A66C-41CA-8940-D108B37648BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6BCE4C-DB6B-44AA-952F-A7F76EA7F6A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inscritos" sheetId="2" r:id="rId1"/>
     <sheet name="Asistencia" sheetId="1" r:id="rId2"/>
-    <sheet name="Notas" sheetId="4" r:id="rId3"/>
+    <sheet name="Hoja1" sheetId="5" r:id="rId3"/>
+    <sheet name="Notas" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Inscritos!$1:$3</definedName>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="260">
   <si>
     <t>METODOLOGÍA DE ESTUDIO</t>
   </si>
@@ -794,6 +795,30 @@
   </si>
   <si>
     <t>mariaisabelquiñoneshernandez9@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 de Julio </t>
+  </si>
+  <si>
+    <t>Despedida</t>
+  </si>
+  <si>
+    <t>Lenis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yeris </t>
+  </si>
+  <si>
+    <t>Sofia Salcedo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isabela Cuitiva </t>
+  </si>
+  <si>
+    <t>Verónica Arrieta</t>
+  </si>
+  <si>
+    <t>Aporte Artístico</t>
   </si>
 </sst>
 </file>
@@ -1441,6 +1466,9 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1708,12 +1736,7 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="3" builtinId="8"/>
@@ -2220,28 +2243,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="93" t="s">
+      <c r="A1" s="94" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="94"/>
-      <c r="D1" s="94"/>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="95"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="96"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="93" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="92"/>
-      <c r="C2" s="92"/>
-      <c r="D2" s="92"/>
-      <c r="E2" s="92"/>
-      <c r="F2" s="92"/>
-      <c r="G2" s="92"/>
-      <c r="H2" s="92"/>
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
@@ -3755,7 +3778,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="34.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.6328125" customWidth="1"/>
+    <col min="3" max="3" width="8.6328125" customWidth="1"/>
     <col min="4" max="4" width="10.90625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
@@ -3763,7 +3786,9 @@
     <col min="8" max="8" width="7.36328125" customWidth="1"/>
     <col min="9" max="9" width="11.36328125" customWidth="1"/>
     <col min="10" max="10" width="10.6328125" customWidth="1"/>
-    <col min="11" max="15" width="7.36328125" customWidth="1"/>
+    <col min="11" max="13" width="7.36328125" customWidth="1"/>
+    <col min="14" max="14" width="10.08984375" customWidth="1"/>
+    <col min="15" max="15" width="7.36328125" customWidth="1"/>
     <col min="16" max="16" width="7.36328125" style="2" customWidth="1"/>
     <col min="17" max="24" width="7.36328125" customWidth="1"/>
     <col min="25" max="25" width="7.36328125" style="2" customWidth="1"/>
@@ -3772,37 +3797,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="69" t="s">
+      <c r="B1" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="69"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
-      <c r="S1" s="69"/>
-      <c r="T1" s="69"/>
-      <c r="U1" s="69"/>
-      <c r="V1" s="69"/>
-      <c r="W1" s="69"/>
-      <c r="X1" s="69"/>
-      <c r="Y1" s="69"/>
-      <c r="Z1" s="69"/>
-      <c r="AA1" s="69"/>
-      <c r="AB1" s="69"/>
-      <c r="AC1" s="69"/>
-      <c r="AD1" s="69"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
+      <c r="Q1" s="70"/>
+      <c r="R1" s="70"/>
+      <c r="S1" s="70"/>
+      <c r="T1" s="70"/>
+      <c r="U1" s="70"/>
+      <c r="V1" s="70"/>
+      <c r="W1" s="70"/>
+      <c r="X1" s="70"/>
+      <c r="Y1" s="70"/>
+      <c r="Z1" s="70"/>
+      <c r="AA1" s="70"/>
+      <c r="AB1" s="70"/>
+      <c r="AC1" s="70"/>
+      <c r="AD1" s="70"/>
     </row>
     <row r="2" spans="1:30" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="55" t="s">
@@ -3814,120 +3839,120 @@
       <c r="C2" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="85" t="s">
+      <c r="D2" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="87"/>
-      <c r="H2" s="70" t="s">
+      <c r="E2" s="87"/>
+      <c r="F2" s="87"/>
+      <c r="G2" s="88"/>
+      <c r="H2" s="71" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="71"/>
-      <c r="M2" s="71"/>
-      <c r="N2" s="71"/>
-      <c r="O2" s="71"/>
-      <c r="P2" s="72"/>
-      <c r="Q2" s="79" t="s">
+      <c r="I2" s="72"/>
+      <c r="J2" s="72"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="72"/>
+      <c r="M2" s="72"/>
+      <c r="N2" s="72"/>
+      <c r="O2" s="72"/>
+      <c r="P2" s="73"/>
+      <c r="Q2" s="80" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="80"/>
-      <c r="S2" s="80"/>
-      <c r="T2" s="80"/>
-      <c r="U2" s="80"/>
-      <c r="V2" s="80"/>
-      <c r="W2" s="80"/>
-      <c r="X2" s="80"/>
-      <c r="Y2" s="81"/>
-      <c r="Z2" s="62" t="s">
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="81"/>
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="81"/>
+      <c r="Y2" s="82"/>
+      <c r="Z2" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="AA2" s="63"/>
-      <c r="AB2" s="63"/>
-      <c r="AC2" s="63"/>
-      <c r="AD2" s="64"/>
+      <c r="AA2" s="64"/>
+      <c r="AB2" s="64"/>
+      <c r="AC2" s="64"/>
+      <c r="AD2" s="65"/>
     </row>
     <row r="3" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="56"/>
       <c r="B3" s="54"/>
       <c r="C3" s="56"/>
-      <c r="D3" s="88" t="s">
+      <c r="D3" s="89" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="73" t="s">
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="74"/>
-      <c r="J3" s="74"/>
-      <c r="K3" s="74"/>
-      <c r="L3" s="74"/>
-      <c r="M3" s="74"/>
-      <c r="N3" s="74"/>
-      <c r="O3" s="74"/>
-      <c r="P3" s="75"/>
-      <c r="Q3" s="82" t="s">
+      <c r="I3" s="75"/>
+      <c r="J3" s="75"/>
+      <c r="K3" s="75"/>
+      <c r="L3" s="75"/>
+      <c r="M3" s="75"/>
+      <c r="N3" s="75"/>
+      <c r="O3" s="75"/>
+      <c r="P3" s="76"/>
+      <c r="Q3" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="R3" s="83"/>
-      <c r="S3" s="83"/>
-      <c r="T3" s="83"/>
-      <c r="U3" s="83"/>
-      <c r="V3" s="83"/>
-      <c r="W3" s="83"/>
-      <c r="X3" s="83"/>
-      <c r="Y3" s="84"/>
-      <c r="Z3" s="65" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="66"/>
-      <c r="AB3" s="66"/>
-      <c r="AC3" s="66"/>
-      <c r="AD3" s="67"/>
+      <c r="R3" s="84"/>
+      <c r="S3" s="84"/>
+      <c r="T3" s="84"/>
+      <c r="U3" s="84"/>
+      <c r="V3" s="84"/>
+      <c r="W3" s="84"/>
+      <c r="X3" s="84"/>
+      <c r="Y3" s="85"/>
+      <c r="Z3" s="66" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="67"/>
+      <c r="AB3" s="67"/>
+      <c r="AC3" s="67"/>
+      <c r="AD3" s="68"/>
     </row>
     <row r="4" spans="1:30" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="56"/>
       <c r="B4" s="54"/>
       <c r="C4" s="56"/>
-      <c r="D4" s="91" t="s">
+      <c r="D4" s="92" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="77"/>
-      <c r="F4" s="77"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="76" t="s">
+      <c r="H4" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="77"/>
-      <c r="J4" s="77"/>
-      <c r="K4" s="77"/>
-      <c r="L4" s="77"/>
-      <c r="M4" s="77"/>
-      <c r="N4" s="77"/>
-      <c r="O4" s="78"/>
+      <c r="I4" s="78"/>
+      <c r="J4" s="78"/>
+      <c r="K4" s="78"/>
+      <c r="L4" s="78"/>
+      <c r="M4" s="78"/>
+      <c r="N4" s="78"/>
+      <c r="O4" s="79"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="76" t="s">
+      <c r="Q4" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="R4" s="77"/>
-      <c r="S4" s="77"/>
-      <c r="T4" s="77"/>
-      <c r="U4" s="77"/>
-      <c r="V4" s="77"/>
-      <c r="W4" s="77"/>
-      <c r="X4" s="78"/>
+      <c r="R4" s="78"/>
+      <c r="S4" s="78"/>
+      <c r="T4" s="78"/>
+      <c r="U4" s="78"/>
+      <c r="V4" s="78"/>
+      <c r="W4" s="78"/>
+      <c r="X4" s="79"/>
       <c r="Y4" s="13"/>
-      <c r="Z4" s="68" t="s">
+      <c r="Z4" s="69" t="s">
         <v>24</v>
       </c>
-      <c r="AA4" s="68"/>
-      <c r="AB4" s="68"/>
-      <c r="AC4" s="68"/>
+      <c r="AA4" s="69"/>
+      <c r="AB4" s="69"/>
+      <c r="AC4" s="69"/>
       <c r="AD4" s="3"/>
     </row>
     <row r="5" spans="1:30" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3956,7 +3981,9 @@
       <c r="K5" s="29"/>
       <c r="L5" s="29"/>
       <c r="M5" s="29"/>
-      <c r="N5" s="29"/>
+      <c r="N5" s="29" t="s">
+        <v>252</v>
+      </c>
       <c r="O5" s="29"/>
       <c r="P5" s="12" t="s">
         <v>19</v>
@@ -3980,7 +4007,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A6" s="21">
         <v>1</v>
       </c>
@@ -4006,11 +4033,13 @@
       <c r="K6" s="39"/>
       <c r="L6" s="39"/>
       <c r="M6" s="39"/>
-      <c r="N6" s="39"/>
+      <c r="N6" s="39">
+        <v>1</v>
+      </c>
       <c r="O6" s="40"/>
       <c r="P6" s="38">
         <f t="shared" ref="P6:P53" si="0">+SUM(H6:O6)/8</f>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q6" s="39"/>
       <c r="R6" s="39"/>
@@ -4033,7 +4062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A7" s="21">
         <v>2</v>
       </c>
@@ -4061,11 +4090,13 @@
       <c r="K7" s="39"/>
       <c r="L7" s="39"/>
       <c r="M7" s="39"/>
-      <c r="N7" s="39"/>
+      <c r="N7" s="39">
+        <v>1</v>
+      </c>
       <c r="O7" s="40"/>
       <c r="P7" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q7" s="39"/>
       <c r="R7" s="39"/>
@@ -4088,7 +4119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A8" s="21">
         <v>3</v>
       </c>
@@ -4116,11 +4147,13 @@
       <c r="K8" s="39"/>
       <c r="L8" s="39"/>
       <c r="M8" s="39"/>
-      <c r="N8" s="39"/>
+      <c r="N8" s="39">
+        <v>1</v>
+      </c>
       <c r="O8" s="40"/>
       <c r="P8" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q8" s="39"/>
       <c r="R8" s="39"/>
@@ -4171,7 +4204,9 @@
       <c r="K9" s="39"/>
       <c r="L9" s="39"/>
       <c r="M9" s="39"/>
-      <c r="N9" s="39"/>
+      <c r="N9" s="39">
+        <v>0</v>
+      </c>
       <c r="O9" s="39"/>
       <c r="P9" s="38">
         <f t="shared" si="0"/>
@@ -4226,11 +4261,13 @@
       <c r="K10" s="39"/>
       <c r="L10" s="39"/>
       <c r="M10" s="39"/>
-      <c r="N10" s="39"/>
+      <c r="N10" s="39">
+        <v>1</v>
+      </c>
       <c r="O10" s="39"/>
       <c r="P10" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q10" s="39"/>
       <c r="R10" s="39"/>
@@ -4281,11 +4318,13 @@
       <c r="K11" s="39"/>
       <c r="L11" s="39"/>
       <c r="M11" s="39"/>
-      <c r="N11" s="39"/>
+      <c r="N11" s="39">
+        <v>1</v>
+      </c>
       <c r="O11" s="40"/>
       <c r="P11" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q11" s="39"/>
       <c r="R11" s="39"/>
@@ -4336,7 +4375,9 @@
       <c r="K12" s="39"/>
       <c r="L12" s="39"/>
       <c r="M12" s="39"/>
-      <c r="N12" s="39"/>
+      <c r="N12" s="39">
+        <v>0</v>
+      </c>
       <c r="O12" s="40"/>
       <c r="P12" s="38">
         <f t="shared" si="0"/>
@@ -4363,7 +4404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A13" s="21">
         <v>8</v>
       </c>
@@ -4391,11 +4432,13 @@
       <c r="K13" s="39"/>
       <c r="L13" s="39"/>
       <c r="M13" s="39"/>
-      <c r="N13" s="39"/>
+      <c r="N13" s="39">
+        <v>1</v>
+      </c>
       <c r="O13" s="39"/>
       <c r="P13" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q13" s="39"/>
       <c r="R13" s="39"/>
@@ -4446,11 +4489,13 @@
       <c r="K14" s="39"/>
       <c r="L14" s="39"/>
       <c r="M14" s="39"/>
-      <c r="N14" s="39"/>
+      <c r="N14" s="39">
+        <v>1</v>
+      </c>
       <c r="O14" s="40"/>
       <c r="P14" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q14" s="39"/>
       <c r="R14" s="39"/>
@@ -4501,11 +4546,13 @@
       <c r="K15" s="39"/>
       <c r="L15" s="39"/>
       <c r="M15" s="39"/>
-      <c r="N15" s="39"/>
+      <c r="N15" s="39">
+        <v>1</v>
+      </c>
       <c r="O15" s="40"/>
       <c r="P15" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q15" s="39"/>
       <c r="R15" s="39"/>
@@ -4528,7 +4575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A16" s="21">
         <v>11</v>
       </c>
@@ -4556,11 +4603,13 @@
       <c r="K16" s="39"/>
       <c r="L16" s="39"/>
       <c r="M16" s="39"/>
-      <c r="N16" s="39"/>
+      <c r="N16" s="39">
+        <v>1</v>
+      </c>
       <c r="O16" s="40"/>
       <c r="P16" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q16" s="39"/>
       <c r="R16" s="39"/>
@@ -4611,11 +4660,13 @@
       <c r="K17" s="39"/>
       <c r="L17" s="39"/>
       <c r="M17" s="39"/>
-      <c r="N17" s="39"/>
+      <c r="N17" s="39">
+        <v>1</v>
+      </c>
       <c r="O17" s="40"/>
       <c r="P17" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q17" s="39"/>
       <c r="R17" s="39"/>
@@ -4666,11 +4717,13 @@
       <c r="K18" s="39"/>
       <c r="L18" s="39"/>
       <c r="M18" s="39"/>
-      <c r="N18" s="39"/>
+      <c r="N18" s="39">
+        <v>1</v>
+      </c>
       <c r="O18" s="40"/>
       <c r="P18" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q18" s="39"/>
       <c r="R18" s="39"/>
@@ -4721,11 +4774,13 @@
       <c r="K19" s="39"/>
       <c r="L19" s="39"/>
       <c r="M19" s="39"/>
-      <c r="N19" s="39"/>
+      <c r="N19" s="39">
+        <v>1</v>
+      </c>
       <c r="O19" s="40"/>
       <c r="P19" s="38">
         <f t="shared" si="0"/>
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
       <c r="Q19" s="39"/>
       <c r="R19" s="39"/>
@@ -4776,11 +4831,13 @@
       <c r="K20" s="39"/>
       <c r="L20" s="39"/>
       <c r="M20" s="39"/>
-      <c r="N20" s="39"/>
+      <c r="N20" s="39">
+        <v>1</v>
+      </c>
       <c r="O20" s="40"/>
       <c r="P20" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q20" s="39"/>
       <c r="R20" s="39"/>
@@ -4803,7 +4860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A21" s="21">
         <v>16</v>
       </c>
@@ -4831,11 +4888,13 @@
       <c r="K21" s="39"/>
       <c r="L21" s="39"/>
       <c r="M21" s="39"/>
-      <c r="N21" s="39"/>
+      <c r="N21" s="39">
+        <v>1</v>
+      </c>
       <c r="O21" s="39"/>
       <c r="P21" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q21" s="39"/>
       <c r="R21" s="39"/>
@@ -4886,11 +4945,13 @@
       <c r="K22" s="39"/>
       <c r="L22" s="39"/>
       <c r="M22" s="39"/>
-      <c r="N22" s="39"/>
+      <c r="N22" s="39">
+        <v>1</v>
+      </c>
       <c r="O22" s="40"/>
       <c r="P22" s="38">
         <f t="shared" si="0"/>
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
       <c r="Q22" s="39"/>
       <c r="R22" s="39"/>
@@ -4941,11 +5002,13 @@
       <c r="K23" s="39"/>
       <c r="L23" s="39"/>
       <c r="M23" s="39"/>
-      <c r="N23" s="39"/>
+      <c r="N23" s="39">
+        <v>1</v>
+      </c>
       <c r="O23" s="40"/>
       <c r="P23" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q23" s="39"/>
       <c r="R23" s="39"/>
@@ -4968,11 +5031,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A24" s="21">
         <v>19</v>
       </c>
-      <c r="B24" s="152" t="str">
+      <c r="B24" s="19" t="str">
         <f>+Inscritos!B22</f>
         <v xml:space="preserve">ISLENE TEIRUMA LOBO HERNÁNDEZ </v>
       </c>
@@ -4996,7 +5059,9 @@
       <c r="K24" s="39"/>
       <c r="L24" s="39"/>
       <c r="M24" s="39"/>
-      <c r="N24" s="39"/>
+      <c r="N24" s="39">
+        <v>0</v>
+      </c>
       <c r="O24" s="40"/>
       <c r="P24" s="38">
         <f t="shared" si="0"/>
@@ -5023,11 +5088,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:30" s="20" customFormat="1" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:30" s="20" customFormat="1" ht="26" x14ac:dyDescent="0.35">
       <c r="A25" s="21">
         <v>20</v>
       </c>
-      <c r="B25" s="152" t="str">
+      <c r="B25" s="19" t="str">
         <f>+Inscritos!B23</f>
         <v xml:space="preserve">JEAN CARLOS QUIÑONES HOYOS </v>
       </c>
@@ -5051,11 +5116,13 @@
       <c r="K25" s="39"/>
       <c r="L25" s="39"/>
       <c r="M25" s="39"/>
-      <c r="N25" s="39"/>
+      <c r="N25" s="39">
+        <v>1</v>
+      </c>
       <c r="O25" s="39"/>
       <c r="P25" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q25" s="39"/>
       <c r="R25" s="39"/>
@@ -5082,7 +5149,7 @@
       <c r="A26" s="21">
         <v>21</v>
       </c>
-      <c r="B26" s="152" t="str">
+      <c r="B26" s="19" t="str">
         <f>+Inscritos!B24</f>
         <v>JORGE ANDRES ARRIETA GARCIA</v>
       </c>
@@ -5106,7 +5173,9 @@
       <c r="K26" s="39"/>
       <c r="L26" s="39"/>
       <c r="M26" s="39"/>
-      <c r="N26" s="39"/>
+      <c r="N26" s="39">
+        <v>0</v>
+      </c>
       <c r="O26" s="40"/>
       <c r="P26" s="38">
         <f t="shared" si="0"/>
@@ -5137,7 +5206,7 @@
       <c r="A27" s="21">
         <v>22</v>
       </c>
-      <c r="B27" s="152" t="str">
+      <c r="B27" s="19" t="str">
         <f>+Inscritos!B25</f>
         <v>JULIAN ANDRES SAENZ MOLINA</v>
       </c>
@@ -5161,7 +5230,9 @@
       <c r="K27" s="39"/>
       <c r="L27" s="39"/>
       <c r="M27" s="39"/>
-      <c r="N27" s="39"/>
+      <c r="N27" s="39">
+        <v>0</v>
+      </c>
       <c r="O27" s="40"/>
       <c r="P27" s="38">
         <f t="shared" si="0"/>
@@ -5192,7 +5263,7 @@
       <c r="A28" s="21">
         <v>23</v>
       </c>
-      <c r="B28" s="152" t="str">
+      <c r="B28" s="19" t="str">
         <f>+Inscritos!B26</f>
         <v>JUNIOR ANDRES CALLE SAMARRA</v>
       </c>
@@ -5216,7 +5287,9 @@
       <c r="K28" s="39"/>
       <c r="L28" s="39"/>
       <c r="M28" s="39"/>
-      <c r="N28" s="39"/>
+      <c r="N28" s="39">
+        <v>0</v>
+      </c>
       <c r="O28" s="40"/>
       <c r="P28" s="38">
         <f t="shared" si="0"/>
@@ -5247,7 +5320,7 @@
       <c r="A29" s="21">
         <v>24</v>
       </c>
-      <c r="B29" s="152" t="str">
+      <c r="B29" s="19" t="str">
         <f>+Inscritos!B27</f>
         <v xml:space="preserve">KAREN NOEMITH NIETO DE AGUAS </v>
       </c>
@@ -5271,11 +5344,13 @@
       <c r="K29" s="39"/>
       <c r="L29" s="39"/>
       <c r="M29" s="39"/>
-      <c r="N29" s="39"/>
+      <c r="N29" s="39">
+        <v>1</v>
+      </c>
       <c r="O29" s="40"/>
       <c r="P29" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q29" s="39"/>
       <c r="R29" s="39"/>
@@ -5302,7 +5377,7 @@
       <c r="A30" s="21">
         <v>25</v>
       </c>
-      <c r="B30" s="152" t="str">
+      <c r="B30" s="19" t="str">
         <f>+Inscritos!B28</f>
         <v xml:space="preserve">KATERINE HOLGUIN BENAVIDES </v>
       </c>
@@ -5326,11 +5401,13 @@
       <c r="K30" s="39"/>
       <c r="L30" s="39"/>
       <c r="M30" s="39"/>
-      <c r="N30" s="39"/>
+      <c r="N30" s="39">
+        <v>1</v>
+      </c>
       <c r="O30" s="39"/>
       <c r="P30" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q30" s="39"/>
       <c r="R30" s="39"/>
@@ -5353,11 +5430,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A31" s="21">
         <v>26</v>
       </c>
-      <c r="B31" s="152" t="str">
+      <c r="B31" s="19" t="str">
         <f>+Inscritos!B29</f>
         <v xml:space="preserve">KATIA ANDREA FERNÁNDEZ RAMOS </v>
       </c>
@@ -5381,7 +5458,9 @@
       <c r="K31" s="39"/>
       <c r="L31" s="39"/>
       <c r="M31" s="39"/>
-      <c r="N31" s="39"/>
+      <c r="N31" s="39">
+        <v>0</v>
+      </c>
       <c r="O31" s="40"/>
       <c r="P31" s="38">
         <f t="shared" si="0"/>
@@ -5408,11 +5487,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A32" s="21">
         <v>27</v>
       </c>
-      <c r="B32" s="151" t="str">
+      <c r="B32" s="62" t="str">
         <f>+Inscritos!B30</f>
         <v xml:space="preserve">KEIDER LUIS SUAREZ CALDEÑO </v>
       </c>
@@ -5436,11 +5515,13 @@
       <c r="K32" s="39"/>
       <c r="L32" s="39"/>
       <c r="M32" s="39"/>
-      <c r="N32" s="39"/>
+      <c r="N32" s="39">
+        <v>1</v>
+      </c>
       <c r="O32" s="40"/>
       <c r="P32" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q32" s="39"/>
       <c r="R32" s="39"/>
@@ -5467,7 +5548,7 @@
       <c r="A33" s="21">
         <v>28</v>
       </c>
-      <c r="B33" s="151" t="str">
+      <c r="B33" s="62" t="str">
         <f>+Inscritos!B31</f>
         <v xml:space="preserve">KEINER NICK TUIRAN CUITIVA </v>
       </c>
@@ -5491,11 +5572,13 @@
       <c r="K33" s="39"/>
       <c r="L33" s="39"/>
       <c r="M33" s="39"/>
-      <c r="N33" s="39"/>
+      <c r="N33" s="39">
+        <v>1</v>
+      </c>
       <c r="O33" s="40"/>
       <c r="P33" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q33" s="39"/>
       <c r="R33" s="39"/>
@@ -5522,7 +5605,7 @@
       <c r="A34" s="21">
         <v>29</v>
       </c>
-      <c r="B34" s="151" t="str">
+      <c r="B34" s="62" t="str">
         <f>+Inscritos!B32</f>
         <v xml:space="preserve">KENDIS ESTER MONTIEL VILLALOBOS </v>
       </c>
@@ -5546,11 +5629,13 @@
       <c r="K34" s="39"/>
       <c r="L34" s="39"/>
       <c r="M34" s="39"/>
-      <c r="N34" s="39"/>
+      <c r="N34" s="39">
+        <v>1</v>
+      </c>
       <c r="O34" s="40"/>
       <c r="P34" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q34" s="39"/>
       <c r="R34" s="39"/>
@@ -5577,7 +5662,7 @@
       <c r="A35" s="21">
         <v>30</v>
       </c>
-      <c r="B35" s="151" t="str">
+      <c r="B35" s="62" t="str">
         <f>+Inscritos!B33</f>
         <v xml:space="preserve">KEVIN DAVID ACOSTA RAMOS </v>
       </c>
@@ -5601,11 +5686,13 @@
       <c r="K35" s="39"/>
       <c r="L35" s="39"/>
       <c r="M35" s="39"/>
-      <c r="N35" s="39"/>
+      <c r="N35" s="39">
+        <v>1</v>
+      </c>
       <c r="O35" s="40"/>
       <c r="P35" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q35" s="39"/>
       <c r="R35" s="39"/>
@@ -5632,7 +5719,7 @@
       <c r="A36" s="21">
         <v>31</v>
       </c>
-      <c r="B36" s="151" t="str">
+      <c r="B36" s="62" t="str">
         <f>+Inscritos!B34</f>
         <v xml:space="preserve">LENIS ENITH ORTEGA FUENTES </v>
       </c>
@@ -5656,11 +5743,13 @@
       <c r="K36" s="39"/>
       <c r="L36" s="39"/>
       <c r="M36" s="39"/>
-      <c r="N36" s="39"/>
+      <c r="N36" s="39">
+        <v>1</v>
+      </c>
       <c r="O36" s="39"/>
       <c r="P36" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q36" s="39"/>
       <c r="R36" s="39"/>
@@ -5683,11 +5772,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A37" s="21">
         <v>32</v>
       </c>
-      <c r="B37" s="151" t="str">
+      <c r="B37" s="62" t="str">
         <f>+Inscritos!B35</f>
         <v xml:space="preserve">LILIANA ÁLVAREZ FLÓREZ </v>
       </c>
@@ -5711,11 +5800,13 @@
       <c r="K37" s="39"/>
       <c r="L37" s="39"/>
       <c r="M37" s="39"/>
-      <c r="N37" s="39"/>
+      <c r="N37" s="39">
+        <v>1</v>
+      </c>
       <c r="O37" s="40"/>
       <c r="P37" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q37" s="39"/>
       <c r="R37" s="39"/>
@@ -5766,7 +5857,9 @@
       <c r="K38" s="39"/>
       <c r="L38" s="39"/>
       <c r="M38" s="39"/>
-      <c r="N38" s="39"/>
+      <c r="N38" s="39">
+        <v>0</v>
+      </c>
       <c r="O38" s="40"/>
       <c r="P38" s="38">
         <f t="shared" si="0"/>
@@ -5793,7 +5886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A39" s="21">
         <v>34</v>
       </c>
@@ -5821,11 +5914,13 @@
       <c r="K39" s="39"/>
       <c r="L39" s="39"/>
       <c r="M39" s="39"/>
-      <c r="N39" s="39"/>
+      <c r="N39" s="39">
+        <v>1</v>
+      </c>
       <c r="O39" s="40"/>
       <c r="P39" s="38">
         <f t="shared" si="0"/>
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
       <c r="Q39" s="39"/>
       <c r="R39" s="39"/>
@@ -5848,7 +5943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A40" s="21">
         <v>35</v>
       </c>
@@ -5876,7 +5971,9 @@
       <c r="K40" s="39"/>
       <c r="L40" s="39"/>
       <c r="M40" s="39"/>
-      <c r="N40" s="39"/>
+      <c r="N40" s="39">
+        <v>0</v>
+      </c>
       <c r="O40" s="39"/>
       <c r="P40" s="38">
         <f t="shared" si="0"/>
@@ -5931,11 +6028,13 @@
       <c r="K41" s="39"/>
       <c r="L41" s="39"/>
       <c r="M41" s="39"/>
-      <c r="N41" s="39"/>
+      <c r="N41" s="39">
+        <v>1</v>
+      </c>
       <c r="O41" s="39"/>
       <c r="P41" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q41" s="39"/>
       <c r="R41" s="39"/>
@@ -5986,11 +6085,13 @@
       <c r="K42" s="39"/>
       <c r="L42" s="39"/>
       <c r="M42" s="39"/>
-      <c r="N42" s="39"/>
+      <c r="N42" s="39">
+        <v>1</v>
+      </c>
       <c r="O42" s="40"/>
       <c r="P42" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q42" s="39"/>
       <c r="R42" s="39"/>
@@ -6013,7 +6114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A43" s="21">
         <v>38</v>
       </c>
@@ -6041,7 +6142,9 @@
       <c r="K43" s="39"/>
       <c r="L43" s="39"/>
       <c r="M43" s="39"/>
-      <c r="N43" s="39"/>
+      <c r="N43" s="39">
+        <v>0</v>
+      </c>
       <c r="O43" s="40"/>
       <c r="P43" s="38">
         <f t="shared" si="0"/>
@@ -6068,7 +6171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A44" s="21">
         <v>39</v>
       </c>
@@ -6096,7 +6199,9 @@
       <c r="K44" s="39"/>
       <c r="L44" s="39"/>
       <c r="M44" s="39"/>
-      <c r="N44" s="39"/>
+      <c r="N44" s="39">
+        <v>0</v>
+      </c>
       <c r="O44" s="40"/>
       <c r="P44" s="38">
         <f t="shared" si="0"/>
@@ -6151,11 +6256,13 @@
       <c r="K45" s="39"/>
       <c r="L45" s="39"/>
       <c r="M45" s="39"/>
-      <c r="N45" s="39"/>
+      <c r="N45" s="39">
+        <v>1</v>
+      </c>
       <c r="O45" s="40"/>
       <c r="P45" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q45" s="39"/>
       <c r="R45" s="39"/>
@@ -6178,7 +6285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A46" s="21">
         <v>41</v>
       </c>
@@ -6206,11 +6313,13 @@
       <c r="K46" s="39"/>
       <c r="L46" s="39"/>
       <c r="M46" s="39"/>
-      <c r="N46" s="39"/>
+      <c r="N46" s="39">
+        <v>1</v>
+      </c>
       <c r="O46" s="39"/>
       <c r="P46" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q46" s="39"/>
       <c r="R46" s="39"/>
@@ -6233,7 +6342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A47" s="21">
         <v>42</v>
       </c>
@@ -6261,11 +6370,13 @@
       <c r="K47" s="39"/>
       <c r="L47" s="39"/>
       <c r="M47" s="39"/>
-      <c r="N47" s="39"/>
+      <c r="N47" s="39">
+        <v>1</v>
+      </c>
       <c r="O47" s="40"/>
       <c r="P47" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q47" s="39"/>
       <c r="R47" s="39"/>
@@ -6288,7 +6399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A48" s="21">
         <v>43</v>
       </c>
@@ -6316,11 +6427,13 @@
       <c r="K48" s="39"/>
       <c r="L48" s="39"/>
       <c r="M48" s="39"/>
-      <c r="N48" s="39"/>
+      <c r="N48" s="39">
+        <v>1</v>
+      </c>
       <c r="O48" s="40"/>
       <c r="P48" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q48" s="39"/>
       <c r="R48" s="39"/>
@@ -6343,7 +6456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A49" s="21">
         <v>44</v>
       </c>
@@ -6371,11 +6484,13 @@
       <c r="K49" s="39"/>
       <c r="L49" s="39"/>
       <c r="M49" s="39"/>
-      <c r="N49" s="39"/>
+      <c r="N49" s="39">
+        <v>1</v>
+      </c>
       <c r="O49" s="40"/>
       <c r="P49" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q49" s="39"/>
       <c r="R49" s="39"/>
@@ -6398,7 +6513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A50" s="21">
         <v>45</v>
       </c>
@@ -6426,11 +6541,13 @@
       <c r="K50" s="39"/>
       <c r="L50" s="39"/>
       <c r="M50" s="39"/>
-      <c r="N50" s="39"/>
+      <c r="N50" s="39">
+        <v>1</v>
+      </c>
       <c r="O50" s="39"/>
       <c r="P50" s="38">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.125</v>
       </c>
       <c r="Q50" s="39"/>
       <c r="R50" s="39"/>
@@ -6453,7 +6570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A51" s="21">
         <v>46</v>
       </c>
@@ -6481,11 +6598,13 @@
       <c r="K51" s="39"/>
       <c r="L51" s="39"/>
       <c r="M51" s="39"/>
-      <c r="N51" s="39"/>
+      <c r="N51" s="39">
+        <v>1</v>
+      </c>
       <c r="O51" s="40"/>
       <c r="P51" s="38">
         <f t="shared" si="0"/>
-        <v>0.125</v>
+        <v>0.25</v>
       </c>
       <c r="Q51" s="39"/>
       <c r="R51" s="39"/>
@@ -6508,7 +6627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A52" s="21">
         <v>47</v>
       </c>
@@ -6536,11 +6655,13 @@
       <c r="K52" s="39"/>
       <c r="L52" s="39"/>
       <c r="M52" s="39"/>
-      <c r="N52" s="39"/>
+      <c r="N52" s="39">
+        <v>1</v>
+      </c>
       <c r="O52" s="40"/>
       <c r="P52" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q52" s="39"/>
       <c r="R52" s="39"/>
@@ -6563,7 +6684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:30" ht="19.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:30" ht="26" x14ac:dyDescent="0.35">
       <c r="A53" s="21">
         <v>48</v>
       </c>
@@ -6591,11 +6712,13 @@
       <c r="K53" s="39"/>
       <c r="L53" s="39"/>
       <c r="M53" s="39"/>
-      <c r="N53" s="39"/>
+      <c r="N53" s="39">
+        <v>1</v>
+      </c>
       <c r="O53" s="40"/>
       <c r="P53" s="38">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.375</v>
       </c>
       <c r="Q53" s="39"/>
       <c r="R53" s="39"/>
@@ -6647,7 +6770,9 @@
       <c r="K54" s="39"/>
       <c r="L54" s="39"/>
       <c r="M54" s="39"/>
-      <c r="N54" s="39"/>
+      <c r="N54" s="39">
+        <v>0</v>
+      </c>
       <c r="O54" s="40"/>
       <c r="P54" s="38">
         <f t="shared" ref="P54" si="4">+SUM(H54:O54)/8</f>
@@ -7197,6 +7322,55 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFBB87D3-4E21-4E9F-BAA0-8671330E309C}">
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" s="152" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" s="152" t="s">
+        <v>259</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:T74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -7219,123 +7393,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="126" t="s">
+      <c r="B1" s="127" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="126"/>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
-      <c r="F1" s="126"/>
-      <c r="G1" s="126"/>
-      <c r="H1" s="126"/>
-      <c r="I1" s="126"/>
-      <c r="J1" s="126"/>
-      <c r="K1" s="126"/>
-      <c r="L1" s="126"/>
-      <c r="M1" s="126"/>
-      <c r="N1" s="126"/>
-      <c r="O1" s="126"/>
-      <c r="P1" s="126"/>
-      <c r="Q1" s="126"/>
-      <c r="R1" s="126"/>
-      <c r="S1" s="126"/>
-      <c r="T1" s="126"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
+      <c r="I1" s="127"/>
+      <c r="J1" s="127"/>
+      <c r="K1" s="127"/>
+      <c r="L1" s="127"/>
+      <c r="M1" s="127"/>
+      <c r="N1" s="127"/>
+      <c r="O1" s="127"/>
+      <c r="P1" s="127"/>
+      <c r="Q1" s="127"/>
+      <c r="R1" s="127"/>
+      <c r="S1" s="127"/>
+      <c r="T1" s="127"/>
     </row>
     <row r="2" spans="1:20" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="108" t="s">
+      <c r="A2" s="109" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="122" t="s">
+      <c r="B2" s="123" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="124" t="s">
+      <c r="C2" s="125" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="96" t="str">
+      <c r="D2" s="97" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="97"/>
-      <c r="F2" s="98"/>
-      <c r="G2" s="96" t="str">
+      <c r="E2" s="98"/>
+      <c r="F2" s="99"/>
+      <c r="G2" s="97" t="str">
         <f>Asistencia!H2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="97"/>
-      <c r="I2" s="97"/>
-      <c r="J2" s="97"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="96" t="s">
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="99"/>
+      <c r="L2" s="97" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="97"/>
-      <c r="N2" s="97"/>
-      <c r="O2" s="97"/>
-      <c r="P2" s="98"/>
-      <c r="Q2" s="96" t="str">
+      <c r="M2" s="98"/>
+      <c r="N2" s="98"/>
+      <c r="O2" s="98"/>
+      <c r="P2" s="99"/>
+      <c r="Q2" s="97" t="str">
         <f>Asistencia!Z2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="97"/>
-      <c r="S2" s="97"/>
-      <c r="T2" s="98"/>
+      <c r="R2" s="98"/>
+      <c r="S2" s="98"/>
+      <c r="T2" s="99"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="109"/>
-      <c r="B3" s="123"/>
-      <c r="C3" s="125"/>
-      <c r="D3" s="116" t="s">
+      <c r="A3" s="110"/>
+      <c r="B3" s="124"/>
+      <c r="C3" s="126"/>
+      <c r="D3" s="117" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="117"/>
-      <c r="F3" s="118"/>
-      <c r="G3" s="110" t="s">
+      <c r="E3" s="118"/>
+      <c r="F3" s="119"/>
+      <c r="G3" s="111" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="112"/>
-      <c r="L3" s="145" t="s">
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="112"/>
+      <c r="K3" s="113"/>
+      <c r="L3" s="146" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="146"/>
-      <c r="N3" s="146"/>
-      <c r="O3" s="146"/>
-      <c r="P3" s="147"/>
-      <c r="Q3" s="99" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="100"/>
-      <c r="S3" s="100"/>
-      <c r="T3" s="101"/>
+      <c r="M3" s="147"/>
+      <c r="N3" s="147"/>
+      <c r="O3" s="147"/>
+      <c r="P3" s="148"/>
+      <c r="Q3" s="100" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="101"/>
+      <c r="S3" s="101"/>
+      <c r="T3" s="102"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="109"/>
-      <c r="B4" s="123"/>
-      <c r="C4" s="125"/>
-      <c r="D4" s="119"/>
-      <c r="E4" s="120"/>
-      <c r="F4" s="121"/>
-      <c r="G4" s="113"/>
-      <c r="H4" s="114"/>
-      <c r="I4" s="114"/>
-      <c r="J4" s="114"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="148"/>
-      <c r="M4" s="149"/>
-      <c r="N4" s="149"/>
-      <c r="O4" s="149"/>
-      <c r="P4" s="150"/>
-      <c r="Q4" s="102"/>
-      <c r="R4" s="103"/>
-      <c r="S4" s="103"/>
-      <c r="T4" s="104"/>
+      <c r="A4" s="110"/>
+      <c r="B4" s="124"/>
+      <c r="C4" s="126"/>
+      <c r="D4" s="120"/>
+      <c r="E4" s="121"/>
+      <c r="F4" s="122"/>
+      <c r="G4" s="114"/>
+      <c r="H4" s="115"/>
+      <c r="I4" s="115"/>
+      <c r="J4" s="115"/>
+      <c r="K4" s="116"/>
+      <c r="L4" s="149"/>
+      <c r="M4" s="150"/>
+      <c r="N4" s="150"/>
+      <c r="O4" s="150"/>
+      <c r="P4" s="151"/>
+      <c r="Q4" s="103"/>
+      <c r="R4" s="104"/>
+      <c r="S4" s="104"/>
+      <c r="T4" s="105"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="109"/>
-      <c r="B5" s="123"/>
-      <c r="C5" s="125"/>
+      <c r="A5" s="110"/>
+      <c r="B5" s="124"/>
+      <c r="C5" s="126"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -9867,180 +10041,180 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D65" s="130" t="s">
+      <c r="D65" s="131" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="133" t="s">
+      <c r="E65" s="134" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="127" t="s">
+      <c r="G65" s="128" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="139" t="s">
+      <c r="H65" s="140" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="139" t="s">
+      <c r="I65" s="140" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="127" t="s">
+      <c r="J65" s="128" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="105" t="s">
+      <c r="L65" s="106" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="136" t="s">
+      <c r="M65" s="137" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="136" t="s">
+      <c r="N65" s="137" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="105" t="s">
+      <c r="O65" s="106" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="142" t="s">
+      <c r="Q65" s="143" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="142" t="s">
+      <c r="R65" s="143" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="142" t="s">
+      <c r="S65" s="143" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D66" s="131"/>
-      <c r="E66" s="134"/>
-      <c r="G66" s="128"/>
-      <c r="H66" s="140"/>
-      <c r="I66" s="140"/>
-      <c r="J66" s="128"/>
-      <c r="L66" s="106"/>
-      <c r="M66" s="137"/>
-      <c r="N66" s="137"/>
-      <c r="O66" s="106"/>
-      <c r="Q66" s="143"/>
-      <c r="R66" s="143"/>
-      <c r="S66" s="143"/>
+      <c r="D66" s="132"/>
+      <c r="E66" s="135"/>
+      <c r="G66" s="129"/>
+      <c r="H66" s="141"/>
+      <c r="I66" s="141"/>
+      <c r="J66" s="129"/>
+      <c r="L66" s="107"/>
+      <c r="M66" s="138"/>
+      <c r="N66" s="138"/>
+      <c r="O66" s="107"/>
+      <c r="Q66" s="144"/>
+      <c r="R66" s="144"/>
+      <c r="S66" s="144"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D67" s="131"/>
-      <c r="E67" s="134"/>
-      <c r="G67" s="128"/>
-      <c r="H67" s="140"/>
-      <c r="I67" s="140"/>
-      <c r="J67" s="128"/>
-      <c r="L67" s="106"/>
-      <c r="M67" s="137"/>
-      <c r="N67" s="137"/>
-      <c r="O67" s="106"/>
-      <c r="Q67" s="143"/>
-      <c r="R67" s="143"/>
-      <c r="S67" s="143"/>
+      <c r="D67" s="132"/>
+      <c r="E67" s="135"/>
+      <c r="G67" s="129"/>
+      <c r="H67" s="141"/>
+      <c r="I67" s="141"/>
+      <c r="J67" s="129"/>
+      <c r="L67" s="107"/>
+      <c r="M67" s="138"/>
+      <c r="N67" s="138"/>
+      <c r="O67" s="107"/>
+      <c r="Q67" s="144"/>
+      <c r="R67" s="144"/>
+      <c r="S67" s="144"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D68" s="131"/>
-      <c r="E68" s="134"/>
-      <c r="G68" s="128"/>
-      <c r="H68" s="140"/>
-      <c r="I68" s="140"/>
-      <c r="J68" s="128"/>
-      <c r="L68" s="106"/>
-      <c r="M68" s="137"/>
-      <c r="N68" s="137"/>
-      <c r="O68" s="106"/>
-      <c r="Q68" s="143"/>
-      <c r="R68" s="143"/>
-      <c r="S68" s="143"/>
+      <c r="D68" s="132"/>
+      <c r="E68" s="135"/>
+      <c r="G68" s="129"/>
+      <c r="H68" s="141"/>
+      <c r="I68" s="141"/>
+      <c r="J68" s="129"/>
+      <c r="L68" s="107"/>
+      <c r="M68" s="138"/>
+      <c r="N68" s="138"/>
+      <c r="O68" s="107"/>
+      <c r="Q68" s="144"/>
+      <c r="R68" s="144"/>
+      <c r="S68" s="144"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D69" s="131"/>
-      <c r="E69" s="134"/>
-      <c r="G69" s="128"/>
-      <c r="H69" s="140"/>
-      <c r="I69" s="140"/>
-      <c r="J69" s="128"/>
-      <c r="L69" s="106"/>
-      <c r="M69" s="137"/>
-      <c r="N69" s="137"/>
-      <c r="O69" s="106"/>
-      <c r="Q69" s="143"/>
-      <c r="R69" s="143"/>
-      <c r="S69" s="143"/>
+      <c r="D69" s="132"/>
+      <c r="E69" s="135"/>
+      <c r="G69" s="129"/>
+      <c r="H69" s="141"/>
+      <c r="I69" s="141"/>
+      <c r="J69" s="129"/>
+      <c r="L69" s="107"/>
+      <c r="M69" s="138"/>
+      <c r="N69" s="138"/>
+      <c r="O69" s="107"/>
+      <c r="Q69" s="144"/>
+      <c r="R69" s="144"/>
+      <c r="S69" s="144"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D70" s="131"/>
-      <c r="E70" s="134"/>
-      <c r="G70" s="128"/>
-      <c r="H70" s="140"/>
-      <c r="I70" s="140"/>
-      <c r="J70" s="128"/>
-      <c r="L70" s="106"/>
-      <c r="M70" s="137"/>
-      <c r="N70" s="137"/>
-      <c r="O70" s="106"/>
-      <c r="Q70" s="143"/>
-      <c r="R70" s="143"/>
-      <c r="S70" s="143"/>
+      <c r="D70" s="132"/>
+      <c r="E70" s="135"/>
+      <c r="G70" s="129"/>
+      <c r="H70" s="141"/>
+      <c r="I70" s="141"/>
+      <c r="J70" s="129"/>
+      <c r="L70" s="107"/>
+      <c r="M70" s="138"/>
+      <c r="N70" s="138"/>
+      <c r="O70" s="107"/>
+      <c r="Q70" s="144"/>
+      <c r="R70" s="144"/>
+      <c r="S70" s="144"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D71" s="131"/>
-      <c r="E71" s="134"/>
-      <c r="G71" s="128"/>
-      <c r="H71" s="140"/>
-      <c r="I71" s="140"/>
-      <c r="J71" s="128"/>
-      <c r="L71" s="106"/>
-      <c r="M71" s="137"/>
-      <c r="N71" s="137"/>
-      <c r="O71" s="106"/>
-      <c r="Q71" s="143"/>
-      <c r="R71" s="143"/>
-      <c r="S71" s="143"/>
+      <c r="D71" s="132"/>
+      <c r="E71" s="135"/>
+      <c r="G71" s="129"/>
+      <c r="H71" s="141"/>
+      <c r="I71" s="141"/>
+      <c r="J71" s="129"/>
+      <c r="L71" s="107"/>
+      <c r="M71" s="138"/>
+      <c r="N71" s="138"/>
+      <c r="O71" s="107"/>
+      <c r="Q71" s="144"/>
+      <c r="R71" s="144"/>
+      <c r="S71" s="144"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D72" s="131"/>
-      <c r="E72" s="134"/>
-      <c r="G72" s="128"/>
-      <c r="H72" s="140"/>
-      <c r="I72" s="140"/>
-      <c r="J72" s="128"/>
-      <c r="L72" s="106"/>
-      <c r="M72" s="137"/>
-      <c r="N72" s="137"/>
-      <c r="O72" s="106"/>
-      <c r="Q72" s="143"/>
-      <c r="R72" s="143"/>
-      <c r="S72" s="143"/>
+      <c r="D72" s="132"/>
+      <c r="E72" s="135"/>
+      <c r="G72" s="129"/>
+      <c r="H72" s="141"/>
+      <c r="I72" s="141"/>
+      <c r="J72" s="129"/>
+      <c r="L72" s="107"/>
+      <c r="M72" s="138"/>
+      <c r="N72" s="138"/>
+      <c r="O72" s="107"/>
+      <c r="Q72" s="144"/>
+      <c r="R72" s="144"/>
+      <c r="S72" s="144"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D73" s="131"/>
-      <c r="E73" s="134"/>
-      <c r="G73" s="128"/>
-      <c r="H73" s="140"/>
-      <c r="I73" s="140"/>
-      <c r="J73" s="128"/>
-      <c r="L73" s="106"/>
-      <c r="M73" s="137"/>
-      <c r="N73" s="137"/>
-      <c r="O73" s="106"/>
-      <c r="Q73" s="143"/>
-      <c r="R73" s="143"/>
-      <c r="S73" s="143"/>
+      <c r="D73" s="132"/>
+      <c r="E73" s="135"/>
+      <c r="G73" s="129"/>
+      <c r="H73" s="141"/>
+      <c r="I73" s="141"/>
+      <c r="J73" s="129"/>
+      <c r="L73" s="107"/>
+      <c r="M73" s="138"/>
+      <c r="N73" s="138"/>
+      <c r="O73" s="107"/>
+      <c r="Q73" s="144"/>
+      <c r="R73" s="144"/>
+      <c r="S73" s="144"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D74" s="132"/>
-      <c r="E74" s="135"/>
-      <c r="G74" s="129"/>
-      <c r="H74" s="141"/>
-      <c r="I74" s="141"/>
-      <c r="J74" s="129"/>
-      <c r="L74" s="107"/>
-      <c r="M74" s="138"/>
-      <c r="N74" s="138"/>
-      <c r="O74" s="107"/>
-      <c r="Q74" s="144"/>
-      <c r="R74" s="144"/>
-      <c r="S74" s="144"/>
+      <c r="D74" s="133"/>
+      <c r="E74" s="136"/>
+      <c r="G74" s="130"/>
+      <c r="H74" s="142"/>
+      <c r="I74" s="142"/>
+      <c r="J74" s="130"/>
+      <c r="L74" s="108"/>
+      <c r="M74" s="139"/>
+      <c r="N74" s="139"/>
+      <c r="O74" s="108"/>
+      <c r="Q74" s="145"/>
+      <c r="R74" s="145"/>
+      <c r="S74" s="145"/>
     </row>
   </sheetData>
   <mergeCells count="25">

</xml_diff>

<commit_message>
preguntas 1 y 2 del tema 1 con los ejesrciocios de entrenamiento
</commit_message>
<xml_diff>
--- a/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
+++ b/9_asistencia_evaluacion/pivu_bijao_grupo_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\extension\camino-udea\9_asistencia_evaluacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6BCE4C-DB6B-44AA-952F-A7F76EA7F6A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F81FD6F-BBED-4E81-94ED-E319A7DD949C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -794,9 +794,6 @@
     <t>1|</t>
   </si>
   <si>
-    <t>mariaisabelquiñoneshernandez9@gmail.com</t>
-  </si>
-  <si>
     <t xml:space="preserve">18 de Julio </t>
   </si>
   <si>
@@ -819,6 +816,9 @@
   </si>
   <si>
     <t>Aporte Artístico</t>
+  </si>
+  <si>
+    <t>quinoneshernandezmariaisabel9@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -829,7 +829,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -998,8 +998,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF00B050"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1069,6 +1083,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1287,7 +1307,7 @@
     <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1469,6 +1489,7 @@
     <xf numFmtId="0" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1571,6 +1592,90 @@
     <xf numFmtId="0" fontId="19" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1598,15 +1703,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1661,82 +1757,18 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hipervínculo" xfId="3" builtinId="8"/>
@@ -2243,28 +2275,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="72" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="95" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="95"/>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="96"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
+      <c r="E1" s="96"/>
+      <c r="F1" s="96"/>
+      <c r="G1" s="96"/>
+      <c r="H1" s="97"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="93" t="s">
+      <c r="A2" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="93"/>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="93"/>
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="94"/>
+      <c r="H2" s="94"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
@@ -3203,7 +3235,7 @@
         <v>175</v>
       </c>
       <c r="G37" s="60" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="H37" s="57" t="s">
         <v>238</v>
@@ -3797,37 +3829,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="66" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="70" t="s">
+      <c r="B1" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="R1" s="70"/>
-      <c r="S1" s="70"/>
-      <c r="T1" s="70"/>
-      <c r="U1" s="70"/>
-      <c r="V1" s="70"/>
-      <c r="W1" s="70"/>
-      <c r="X1" s="70"/>
-      <c r="Y1" s="70"/>
-      <c r="Z1" s="70"/>
-      <c r="AA1" s="70"/>
-      <c r="AB1" s="70"/>
-      <c r="AC1" s="70"/>
-      <c r="AD1" s="70"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="71"/>
+      <c r="Q1" s="71"/>
+      <c r="R1" s="71"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="71"/>
+      <c r="U1" s="71"/>
+      <c r="V1" s="71"/>
+      <c r="W1" s="71"/>
+      <c r="X1" s="71"/>
+      <c r="Y1" s="71"/>
+      <c r="Z1" s="71"/>
+      <c r="AA1" s="71"/>
+      <c r="AB1" s="71"/>
+      <c r="AC1" s="71"/>
+      <c r="AD1" s="71"/>
     </row>
     <row r="2" spans="1:30" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="55" t="s">
@@ -3839,120 +3871,120 @@
       <c r="C2" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="86" t="s">
+      <c r="D2" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
-      <c r="G2" s="88"/>
-      <c r="H2" s="71" t="s">
+      <c r="E2" s="88"/>
+      <c r="F2" s="88"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="72" t="s">
         <v>21</v>
       </c>
-      <c r="I2" s="72"/>
-      <c r="J2" s="72"/>
-      <c r="K2" s="72"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="72"/>
-      <c r="N2" s="72"/>
-      <c r="O2" s="72"/>
-      <c r="P2" s="73"/>
-      <c r="Q2" s="80" t="s">
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="73"/>
+      <c r="O2" s="73"/>
+      <c r="P2" s="74"/>
+      <c r="Q2" s="81" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="81"/>
-      <c r="S2" s="81"/>
-      <c r="T2" s="81"/>
-      <c r="U2" s="81"/>
-      <c r="V2" s="81"/>
-      <c r="W2" s="81"/>
-      <c r="X2" s="81"/>
-      <c r="Y2" s="82"/>
-      <c r="Z2" s="63" t="s">
+      <c r="R2" s="82"/>
+      <c r="S2" s="82"/>
+      <c r="T2" s="82"/>
+      <c r="U2" s="82"/>
+      <c r="V2" s="82"/>
+      <c r="W2" s="82"/>
+      <c r="X2" s="82"/>
+      <c r="Y2" s="83"/>
+      <c r="Z2" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="AA2" s="64"/>
-      <c r="AB2" s="64"/>
-      <c r="AC2" s="64"/>
-      <c r="AD2" s="65"/>
+      <c r="AA2" s="65"/>
+      <c r="AB2" s="65"/>
+      <c r="AC2" s="65"/>
+      <c r="AD2" s="66"/>
     </row>
     <row r="3" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="56"/>
       <c r="B3" s="54"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="89" t="s">
+      <c r="C3" s="156"/>
+      <c r="D3" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="91"/>
-      <c r="H3" s="74" t="s">
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="92"/>
+      <c r="H3" s="75" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="75"/>
-      <c r="J3" s="75"/>
-      <c r="K3" s="75"/>
-      <c r="L3" s="75"/>
-      <c r="M3" s="75"/>
-      <c r="N3" s="75"/>
-      <c r="O3" s="75"/>
-      <c r="P3" s="76"/>
-      <c r="Q3" s="83" t="s">
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="76"/>
+      <c r="L3" s="76"/>
+      <c r="M3" s="76"/>
+      <c r="N3" s="76"/>
+      <c r="O3" s="76"/>
+      <c r="P3" s="77"/>
+      <c r="Q3" s="84" t="s">
         <v>1</v>
       </c>
-      <c r="R3" s="84"/>
-      <c r="S3" s="84"/>
-      <c r="T3" s="84"/>
-      <c r="U3" s="84"/>
-      <c r="V3" s="84"/>
-      <c r="W3" s="84"/>
-      <c r="X3" s="84"/>
-      <c r="Y3" s="85"/>
-      <c r="Z3" s="66" t="s">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="67"/>
-      <c r="AB3" s="67"/>
-      <c r="AC3" s="67"/>
-      <c r="AD3" s="68"/>
+      <c r="R3" s="85"/>
+      <c r="S3" s="85"/>
+      <c r="T3" s="85"/>
+      <c r="U3" s="85"/>
+      <c r="V3" s="85"/>
+      <c r="W3" s="85"/>
+      <c r="X3" s="85"/>
+      <c r="Y3" s="86"/>
+      <c r="Z3" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="68"/>
+      <c r="AB3" s="68"/>
+      <c r="AC3" s="68"/>
+      <c r="AD3" s="69"/>
     </row>
     <row r="4" spans="1:30" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="56"/>
-      <c r="B4" s="54"/>
+      <c r="B4" s="155"/>
       <c r="C4" s="56"/>
-      <c r="D4" s="92" t="s">
+      <c r="D4" s="93" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="78"/>
-      <c r="F4" s="78"/>
+      <c r="E4" s="79"/>
+      <c r="F4" s="79"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="77" t="s">
+      <c r="H4" s="78" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="78"/>
-      <c r="J4" s="78"/>
-      <c r="K4" s="78"/>
-      <c r="L4" s="78"/>
-      <c r="M4" s="78"/>
-      <c r="N4" s="78"/>
-      <c r="O4" s="79"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="79"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
+      <c r="N4" s="79"/>
+      <c r="O4" s="80"/>
       <c r="P4" s="3"/>
-      <c r="Q4" s="77" t="s">
+      <c r="Q4" s="78" t="s">
         <v>24</v>
       </c>
-      <c r="R4" s="78"/>
-      <c r="S4" s="78"/>
-      <c r="T4" s="78"/>
-      <c r="U4" s="78"/>
-      <c r="V4" s="78"/>
-      <c r="W4" s="78"/>
-      <c r="X4" s="79"/>
+      <c r="R4" s="79"/>
+      <c r="S4" s="79"/>
+      <c r="T4" s="79"/>
+      <c r="U4" s="79"/>
+      <c r="V4" s="79"/>
+      <c r="W4" s="79"/>
+      <c r="X4" s="80"/>
       <c r="Y4" s="13"/>
-      <c r="Z4" s="69" t="s">
+      <c r="Z4" s="70" t="s">
         <v>24</v>
       </c>
-      <c r="AA4" s="69"/>
-      <c r="AB4" s="69"/>
-      <c r="AC4" s="69"/>
+      <c r="AA4" s="70"/>
+      <c r="AB4" s="70"/>
+      <c r="AC4" s="70"/>
       <c r="AD4" s="3"/>
     </row>
     <row r="5" spans="1:30" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3982,7 +4014,7 @@
       <c r="L5" s="29"/>
       <c r="M5" s="29"/>
       <c r="N5" s="29" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="O5" s="29"/>
       <c r="P5" s="12" t="s">
@@ -5605,7 +5637,7 @@
       <c r="A34" s="21">
         <v>29</v>
       </c>
-      <c r="B34" s="62" t="str">
+      <c r="B34" s="154" t="str">
         <f>+Inscritos!B32</f>
         <v xml:space="preserve">KENDIS ESTER MONTIEL VILLALOBOS </v>
       </c>
@@ -5662,7 +5694,7 @@
       <c r="A35" s="21">
         <v>30</v>
       </c>
-      <c r="B35" s="62" t="str">
+      <c r="B35" s="154" t="str">
         <f>+Inscritos!B33</f>
         <v xml:space="preserve">KEVIN DAVID ACOSTA RAMOS </v>
       </c>
@@ -5719,7 +5751,7 @@
       <c r="A36" s="21">
         <v>31</v>
       </c>
-      <c r="B36" s="62" t="str">
+      <c r="B36" s="154" t="str">
         <f>+Inscritos!B34</f>
         <v xml:space="preserve">LENIS ENITH ORTEGA FUENTES </v>
       </c>
@@ -5776,7 +5808,7 @@
       <c r="A37" s="21">
         <v>32</v>
       </c>
-      <c r="B37" s="62" t="str">
+      <c r="B37" s="154" t="str">
         <f>+Inscritos!B35</f>
         <v xml:space="preserve">LILIANA ÁLVAREZ FLÓREZ </v>
       </c>
@@ -5833,7 +5865,7 @@
       <c r="A38" s="21">
         <v>33</v>
       </c>
-      <c r="B38" s="19" t="str">
+      <c r="B38" s="153" t="str">
         <f>+Inscritos!B36</f>
         <v xml:space="preserve">LUISA FERNANDA VILORIA VASQUEZ </v>
       </c>
@@ -5890,7 +5922,7 @@
       <c r="A39" s="21">
         <v>34</v>
       </c>
-      <c r="B39" s="19" t="str">
+      <c r="B39" s="153" t="str">
         <f>+Inscritos!B37</f>
         <v xml:space="preserve">MARÍA ISABEL QUIÑONES HERNÁNDEZ </v>
       </c>
@@ -5947,7 +5979,7 @@
       <c r="A40" s="21">
         <v>35</v>
       </c>
-      <c r="B40" s="19" t="str">
+      <c r="B40" s="153" t="str">
         <f>+Inscritos!B38</f>
         <v>MARÍA JOSEFINA MONTIEL BARRETO</v>
       </c>
@@ -6004,7 +6036,7 @@
       <c r="A41" s="21">
         <v>36</v>
       </c>
-      <c r="B41" s="19" t="str">
+      <c r="B41" s="153" t="str">
         <f>+Inscritos!B39</f>
         <v xml:space="preserve">MICHELL GONZALEZ SEVERICHE </v>
       </c>
@@ -6061,7 +6093,7 @@
       <c r="A42" s="21">
         <v>37</v>
       </c>
-      <c r="B42" s="19" t="str">
+      <c r="B42" s="153" t="str">
         <f>+Inscritos!B40</f>
         <v>MISHEEL UPARELA OLEA</v>
       </c>
@@ -6118,7 +6150,7 @@
       <c r="A43" s="21">
         <v>38</v>
       </c>
-      <c r="B43" s="19" t="str">
+      <c r="B43" s="153" t="str">
         <f>+Inscritos!B41</f>
         <v>NEIDER ENRIQUE ALMANZA RUIZ</v>
       </c>
@@ -6175,7 +6207,7 @@
       <c r="A44" s="21">
         <v>39</v>
       </c>
-      <c r="B44" s="19" t="str">
+      <c r="B44" s="153" t="str">
         <f>+Inscritos!B42</f>
         <v xml:space="preserve">NINA ISABEL GUERRERO AVILEZ </v>
       </c>
@@ -7330,38 +7362,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" s="152" t="s">
-        <v>253</v>
+      <c r="A1" s="63" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" s="63" t="s">
         <v>258</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" s="152" t="s">
-        <v>259</v>
       </c>
     </row>
   </sheetData>
@@ -7393,123 +7425,123 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="72.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B1" s="127" t="s">
+      <c r="B1" s="98" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="127"/>
-      <c r="J1" s="127"/>
-      <c r="K1" s="127"/>
-      <c r="L1" s="127"/>
-      <c r="M1" s="127"/>
-      <c r="N1" s="127"/>
-      <c r="O1" s="127"/>
-      <c r="P1" s="127"/>
-      <c r="Q1" s="127"/>
-      <c r="R1" s="127"/>
-      <c r="S1" s="127"/>
-      <c r="T1" s="127"/>
+      <c r="C1" s="98"/>
+      <c r="D1" s="98"/>
+      <c r="E1" s="98"/>
+      <c r="F1" s="98"/>
+      <c r="G1" s="98"/>
+      <c r="H1" s="98"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="98"/>
+      <c r="K1" s="98"/>
+      <c r="L1" s="98"/>
+      <c r="M1" s="98"/>
+      <c r="N1" s="98"/>
+      <c r="O1" s="98"/>
+      <c r="P1" s="98"/>
+      <c r="Q1" s="98"/>
+      <c r="R1" s="98"/>
+      <c r="S1" s="98"/>
+      <c r="T1" s="98"/>
     </row>
     <row r="2" spans="1:20" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="109" t="s">
+      <c r="A2" s="135" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="123" t="s">
+      <c r="B2" s="149" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="125" t="s">
+      <c r="C2" s="151" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="97" t="str">
+      <c r="D2" s="126" t="str">
         <f>Asistencia!D2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="E2" s="98"/>
-      <c r="F2" s="99"/>
-      <c r="G2" s="97" t="str">
+      <c r="E2" s="127"/>
+      <c r="F2" s="128"/>
+      <c r="G2" s="126" t="str">
         <f>Asistencia!H2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="H2" s="98"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="97" t="s">
+      <c r="H2" s="127"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="127"/>
+      <c r="K2" s="128"/>
+      <c r="L2" s="126" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="98"/>
-      <c r="N2" s="98"/>
-      <c r="O2" s="98"/>
-      <c r="P2" s="99"/>
-      <c r="Q2" s="97" t="str">
+      <c r="M2" s="127"/>
+      <c r="N2" s="127"/>
+      <c r="O2" s="127"/>
+      <c r="P2" s="128"/>
+      <c r="Q2" s="126" t="str">
         <f>Asistencia!Z2</f>
         <v>NOMBRE DOCENTE</v>
       </c>
-      <c r="R2" s="98"/>
-      <c r="S2" s="98"/>
-      <c r="T2" s="99"/>
+      <c r="R2" s="127"/>
+      <c r="S2" s="127"/>
+      <c r="T2" s="128"/>
     </row>
     <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="110"/>
-      <c r="B3" s="124"/>
-      <c r="C3" s="126"/>
-      <c r="D3" s="117" t="s">
+      <c r="A3" s="136"/>
+      <c r="B3" s="150"/>
+      <c r="C3" s="152"/>
+      <c r="D3" s="143" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="118"/>
-      <c r="F3" s="119"/>
-      <c r="G3" s="111" t="s">
+      <c r="E3" s="144"/>
+      <c r="F3" s="145"/>
+      <c r="G3" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="112"/>
-      <c r="I3" s="112"/>
-      <c r="J3" s="112"/>
-      <c r="K3" s="113"/>
-      <c r="L3" s="146" t="s">
+      <c r="H3" s="138"/>
+      <c r="I3" s="138"/>
+      <c r="J3" s="138"/>
+      <c r="K3" s="139"/>
+      <c r="L3" s="120" t="s">
         <v>1</v>
       </c>
-      <c r="M3" s="147"/>
-      <c r="N3" s="147"/>
-      <c r="O3" s="147"/>
-      <c r="P3" s="148"/>
-      <c r="Q3" s="100" t="s">
-        <v>0</v>
-      </c>
-      <c r="R3" s="101"/>
-      <c r="S3" s="101"/>
-      <c r="T3" s="102"/>
+      <c r="M3" s="121"/>
+      <c r="N3" s="121"/>
+      <c r="O3" s="121"/>
+      <c r="P3" s="122"/>
+      <c r="Q3" s="129" t="s">
+        <v>0</v>
+      </c>
+      <c r="R3" s="130"/>
+      <c r="S3" s="130"/>
+      <c r="T3" s="131"/>
     </row>
     <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="110"/>
-      <c r="B4" s="124"/>
-      <c r="C4" s="126"/>
-      <c r="D4" s="120"/>
-      <c r="E4" s="121"/>
-      <c r="F4" s="122"/>
-      <c r="G4" s="114"/>
-      <c r="H4" s="115"/>
-      <c r="I4" s="115"/>
-      <c r="J4" s="115"/>
-      <c r="K4" s="116"/>
-      <c r="L4" s="149"/>
-      <c r="M4" s="150"/>
-      <c r="N4" s="150"/>
-      <c r="O4" s="150"/>
-      <c r="P4" s="151"/>
-      <c r="Q4" s="103"/>
-      <c r="R4" s="104"/>
-      <c r="S4" s="104"/>
-      <c r="T4" s="105"/>
+      <c r="A4" s="136"/>
+      <c r="B4" s="150"/>
+      <c r="C4" s="152"/>
+      <c r="D4" s="146"/>
+      <c r="E4" s="147"/>
+      <c r="F4" s="148"/>
+      <c r="G4" s="140"/>
+      <c r="H4" s="141"/>
+      <c r="I4" s="141"/>
+      <c r="J4" s="141"/>
+      <c r="K4" s="142"/>
+      <c r="L4" s="123"/>
+      <c r="M4" s="124"/>
+      <c r="N4" s="124"/>
+      <c r="O4" s="124"/>
+      <c r="P4" s="125"/>
+      <c r="Q4" s="132"/>
+      <c r="R4" s="133"/>
+      <c r="S4" s="133"/>
+      <c r="T4" s="134"/>
     </row>
     <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="110"/>
-      <c r="B5" s="124"/>
-      <c r="C5" s="126"/>
+      <c r="A5" s="136"/>
+      <c r="B5" s="150"/>
+      <c r="C5" s="152"/>
       <c r="D5" s="23">
         <v>0.75</v>
       </c>
@@ -10041,183 +10073,192 @@
       </c>
     </row>
     <row r="65" spans="4:19" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D65" s="131" t="s">
+      <c r="D65" s="102" t="s">
         <v>26</v>
       </c>
-      <c r="E65" s="134" t="s">
+      <c r="E65" s="105" t="s">
         <v>12</v>
       </c>
-      <c r="G65" s="128" t="s">
+      <c r="G65" s="99" t="s">
         <v>8</v>
       </c>
-      <c r="H65" s="140" t="s">
+      <c r="H65" s="114" t="s">
         <v>9</v>
       </c>
-      <c r="I65" s="140" t="s">
+      <c r="I65" s="114" t="s">
         <v>10</v>
       </c>
-      <c r="J65" s="128" t="s">
+      <c r="J65" s="99" t="s">
         <v>11</v>
       </c>
-      <c r="L65" s="106" t="s">
+      <c r="L65" s="108" t="s">
         <v>8</v>
       </c>
-      <c r="M65" s="137" t="s">
+      <c r="M65" s="111" t="s">
         <v>9</v>
       </c>
-      <c r="N65" s="137" t="s">
+      <c r="N65" s="111" t="s">
         <v>10</v>
       </c>
-      <c r="O65" s="106" t="s">
+      <c r="O65" s="108" t="s">
         <v>11</v>
       </c>
-      <c r="Q65" s="143" t="s">
+      <c r="Q65" s="117" t="s">
         <v>26</v>
       </c>
-      <c r="R65" s="143" t="s">
+      <c r="R65" s="117" t="s">
         <v>4</v>
       </c>
-      <c r="S65" s="143" t="s">
+      <c r="S65" s="117" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="66" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D66" s="132"/>
-      <c r="E66" s="135"/>
-      <c r="G66" s="129"/>
-      <c r="H66" s="141"/>
-      <c r="I66" s="141"/>
-      <c r="J66" s="129"/>
-      <c r="L66" s="107"/>
-      <c r="M66" s="138"/>
-      <c r="N66" s="138"/>
-      <c r="O66" s="107"/>
-      <c r="Q66" s="144"/>
-      <c r="R66" s="144"/>
-      <c r="S66" s="144"/>
+      <c r="D66" s="103"/>
+      <c r="E66" s="106"/>
+      <c r="G66" s="100"/>
+      <c r="H66" s="115"/>
+      <c r="I66" s="115"/>
+      <c r="J66" s="100"/>
+      <c r="L66" s="109"/>
+      <c r="M66" s="112"/>
+      <c r="N66" s="112"/>
+      <c r="O66" s="109"/>
+      <c r="Q66" s="118"/>
+      <c r="R66" s="118"/>
+      <c r="S66" s="118"/>
     </row>
     <row r="67" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D67" s="132"/>
-      <c r="E67" s="135"/>
-      <c r="G67" s="129"/>
-      <c r="H67" s="141"/>
-      <c r="I67" s="141"/>
-      <c r="J67" s="129"/>
-      <c r="L67" s="107"/>
-      <c r="M67" s="138"/>
-      <c r="N67" s="138"/>
-      <c r="O67" s="107"/>
-      <c r="Q67" s="144"/>
-      <c r="R67" s="144"/>
-      <c r="S67" s="144"/>
+      <c r="D67" s="103"/>
+      <c r="E67" s="106"/>
+      <c r="G67" s="100"/>
+      <c r="H67" s="115"/>
+      <c r="I67" s="115"/>
+      <c r="J67" s="100"/>
+      <c r="L67" s="109"/>
+      <c r="M67" s="112"/>
+      <c r="N67" s="112"/>
+      <c r="O67" s="109"/>
+      <c r="Q67" s="118"/>
+      <c r="R67" s="118"/>
+      <c r="S67" s="118"/>
     </row>
     <row r="68" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D68" s="132"/>
-      <c r="E68" s="135"/>
-      <c r="G68" s="129"/>
-      <c r="H68" s="141"/>
-      <c r="I68" s="141"/>
-      <c r="J68" s="129"/>
-      <c r="L68" s="107"/>
-      <c r="M68" s="138"/>
-      <c r="N68" s="138"/>
-      <c r="O68" s="107"/>
-      <c r="Q68" s="144"/>
-      <c r="R68" s="144"/>
-      <c r="S68" s="144"/>
+      <c r="D68" s="103"/>
+      <c r="E68" s="106"/>
+      <c r="G68" s="100"/>
+      <c r="H68" s="115"/>
+      <c r="I68" s="115"/>
+      <c r="J68" s="100"/>
+      <c r="L68" s="109"/>
+      <c r="M68" s="112"/>
+      <c r="N68" s="112"/>
+      <c r="O68" s="109"/>
+      <c r="Q68" s="118"/>
+      <c r="R68" s="118"/>
+      <c r="S68" s="118"/>
     </row>
     <row r="69" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D69" s="132"/>
-      <c r="E69" s="135"/>
-      <c r="G69" s="129"/>
-      <c r="H69" s="141"/>
-      <c r="I69" s="141"/>
-      <c r="J69" s="129"/>
-      <c r="L69" s="107"/>
-      <c r="M69" s="138"/>
-      <c r="N69" s="138"/>
-      <c r="O69" s="107"/>
-      <c r="Q69" s="144"/>
-      <c r="R69" s="144"/>
-      <c r="S69" s="144"/>
+      <c r="D69" s="103"/>
+      <c r="E69" s="106"/>
+      <c r="G69" s="100"/>
+      <c r="H69" s="115"/>
+      <c r="I69" s="115"/>
+      <c r="J69" s="100"/>
+      <c r="L69" s="109"/>
+      <c r="M69" s="112"/>
+      <c r="N69" s="112"/>
+      <c r="O69" s="109"/>
+      <c r="Q69" s="118"/>
+      <c r="R69" s="118"/>
+      <c r="S69" s="118"/>
     </row>
     <row r="70" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D70" s="132"/>
-      <c r="E70" s="135"/>
-      <c r="G70" s="129"/>
-      <c r="H70" s="141"/>
-      <c r="I70" s="141"/>
-      <c r="J70" s="129"/>
-      <c r="L70" s="107"/>
-      <c r="M70" s="138"/>
-      <c r="N70" s="138"/>
-      <c r="O70" s="107"/>
-      <c r="Q70" s="144"/>
-      <c r="R70" s="144"/>
-      <c r="S70" s="144"/>
+      <c r="D70" s="103"/>
+      <c r="E70" s="106"/>
+      <c r="G70" s="100"/>
+      <c r="H70" s="115"/>
+      <c r="I70" s="115"/>
+      <c r="J70" s="100"/>
+      <c r="L70" s="109"/>
+      <c r="M70" s="112"/>
+      <c r="N70" s="112"/>
+      <c r="O70" s="109"/>
+      <c r="Q70" s="118"/>
+      <c r="R70" s="118"/>
+      <c r="S70" s="118"/>
     </row>
     <row r="71" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D71" s="132"/>
-      <c r="E71" s="135"/>
-      <c r="G71" s="129"/>
-      <c r="H71" s="141"/>
-      <c r="I71" s="141"/>
-      <c r="J71" s="129"/>
-      <c r="L71" s="107"/>
-      <c r="M71" s="138"/>
-      <c r="N71" s="138"/>
-      <c r="O71" s="107"/>
-      <c r="Q71" s="144"/>
-      <c r="R71" s="144"/>
-      <c r="S71" s="144"/>
+      <c r="D71" s="103"/>
+      <c r="E71" s="106"/>
+      <c r="G71" s="100"/>
+      <c r="H71" s="115"/>
+      <c r="I71" s="115"/>
+      <c r="J71" s="100"/>
+      <c r="L71" s="109"/>
+      <c r="M71" s="112"/>
+      <c r="N71" s="112"/>
+      <c r="O71" s="109"/>
+      <c r="Q71" s="118"/>
+      <c r="R71" s="118"/>
+      <c r="S71" s="118"/>
     </row>
     <row r="72" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D72" s="132"/>
-      <c r="E72" s="135"/>
-      <c r="G72" s="129"/>
-      <c r="H72" s="141"/>
-      <c r="I72" s="141"/>
-      <c r="J72" s="129"/>
-      <c r="L72" s="107"/>
-      <c r="M72" s="138"/>
-      <c r="N72" s="138"/>
-      <c r="O72" s="107"/>
-      <c r="Q72" s="144"/>
-      <c r="R72" s="144"/>
-      <c r="S72" s="144"/>
+      <c r="D72" s="103"/>
+      <c r="E72" s="106"/>
+      <c r="G72" s="100"/>
+      <c r="H72" s="115"/>
+      <c r="I72" s="115"/>
+      <c r="J72" s="100"/>
+      <c r="L72" s="109"/>
+      <c r="M72" s="112"/>
+      <c r="N72" s="112"/>
+      <c r="O72" s="109"/>
+      <c r="Q72" s="118"/>
+      <c r="R72" s="118"/>
+      <c r="S72" s="118"/>
     </row>
     <row r="73" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D73" s="132"/>
-      <c r="E73" s="135"/>
-      <c r="G73" s="129"/>
-      <c r="H73" s="141"/>
-      <c r="I73" s="141"/>
-      <c r="J73" s="129"/>
-      <c r="L73" s="107"/>
-      <c r="M73" s="138"/>
-      <c r="N73" s="138"/>
-      <c r="O73" s="107"/>
-      <c r="Q73" s="144"/>
-      <c r="R73" s="144"/>
-      <c r="S73" s="144"/>
+      <c r="D73" s="103"/>
+      <c r="E73" s="106"/>
+      <c r="G73" s="100"/>
+      <c r="H73" s="115"/>
+      <c r="I73" s="115"/>
+      <c r="J73" s="100"/>
+      <c r="L73" s="109"/>
+      <c r="M73" s="112"/>
+      <c r="N73" s="112"/>
+      <c r="O73" s="109"/>
+      <c r="Q73" s="118"/>
+      <c r="R73" s="118"/>
+      <c r="S73" s="118"/>
     </row>
     <row r="74" spans="4:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D74" s="133"/>
-      <c r="E74" s="136"/>
-      <c r="G74" s="130"/>
-      <c r="H74" s="142"/>
-      <c r="I74" s="142"/>
-      <c r="J74" s="130"/>
-      <c r="L74" s="108"/>
-      <c r="M74" s="139"/>
-      <c r="N74" s="139"/>
-      <c r="O74" s="108"/>
-      <c r="Q74" s="145"/>
-      <c r="R74" s="145"/>
-      <c r="S74" s="145"/>
+      <c r="D74" s="104"/>
+      <c r="E74" s="107"/>
+      <c r="G74" s="101"/>
+      <c r="H74" s="116"/>
+      <c r="I74" s="116"/>
+      <c r="J74" s="101"/>
+      <c r="L74" s="110"/>
+      <c r="M74" s="113"/>
+      <c r="N74" s="113"/>
+      <c r="O74" s="110"/>
+      <c r="Q74" s="119"/>
+      <c r="R74" s="119"/>
+      <c r="S74" s="119"/>
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="Q3:T4"/>
+    <mergeCell ref="O65:O74"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="G3:K4"/>
+    <mergeCell ref="D3:F4"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="J65:J74"/>
     <mergeCell ref="D65:D74"/>
@@ -10234,15 +10275,6 @@
     <mergeCell ref="I65:I74"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="L2:P2"/>
-    <mergeCell ref="G2:K2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="Q3:T4"/>
-    <mergeCell ref="O65:O74"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="G3:K4"/>
-    <mergeCell ref="D3:F4"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>